<commit_message>
Redesign Summary tab with investor-focused stats table
Replace asset class summary, multi-year performance grid, and key metrics
sections with a single Summary Statistics table organized into four
sub-sections:

- Return Metrics: Net IRR, Gross IRR, MOIC, DPI, TVPI
- Capital Metrics: committed capital, ending AUM, growth, cumulative income, peak AUM
- Fee & Expense Metrics: total fees by type, fee drag, net-to-gross ratio
- Yield & Risk Metrics: Year 1/20 yields, best/worst year, gross-to-net spread, leverage contribution

Fund Parameters section retained as-is with editable inputs.

https://claude.ai/code/session_01LxHqBVCxmLCLG5Hb92NmWS
</commit_message>
<xml_diff>
--- a/LP_Financial_Model.xlsx
+++ b/LP_Financial_Model.xlsx
@@ -17,10 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0&quot; bps&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="0.00x"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -204,7 +205,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -227,45 +228,41 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="10" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="10" fontId="5" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="10" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="10" fontId="5" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -674,7 +671,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H52"/>
+  <dimension ref="A1:H46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -795,7 +792,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Asset Class Summary (Year 1)</t>
+          <t>Summary Statistics</t>
         </is>
       </c>
       <c r="B13" s="3" t="n"/>
@@ -809,806 +806,371 @@
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Asset Class</t>
-        </is>
-      </c>
-      <c r="B14" s="9" t="inlineStr"/>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Allocation</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Expected Yield</t>
-        </is>
-      </c>
+          <t>Return Metrics</t>
+        </is>
+      </c>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="10" t="n"/>
+      <c r="H14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
-        <is>
-          <t>LIHTC Loans</t>
-        </is>
-      </c>
-      <c r="B15" s="5" t="n"/>
-      <c r="C15" s="10">
-        <f>'Annual Model'!C6</f>
-        <v/>
-      </c>
-      <c r="D15" s="10">
-        <f>'Annual Model'!C13</f>
+      <c r="A15" s="11" t="inlineStr">
+        <is>
+          <t>Net IRR (Avg Annual Net Yield)</t>
+        </is>
+      </c>
+      <c r="C15" s="12">
+        <f>AVERAGE('Annual Model'!C47,'Annual Model'!D47,'Annual Model'!E47,'Annual Model'!F47,'Annual Model'!G47,'Annual Model'!H47,'Annual Model'!I47,'Annual Model'!J47,'Annual Model'!K47,'Annual Model'!L47,'Annual Model'!M47,'Annual Model'!N47,'Annual Model'!O47,'Annual Model'!P47,'Annual Model'!Q47,'Annual Model'!R47,'Annual Model'!S47,'Annual Model'!T47,'Annual Model'!U47,'Annual Model'!V47)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Municipal Bonds</t>
-        </is>
-      </c>
-      <c r="B16" s="5" t="n"/>
-      <c r="C16" s="10">
-        <f>'Annual Model'!C7</f>
-        <v/>
-      </c>
-      <c r="D16" s="10">
-        <f>'Annual Model'!C14</f>
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Gross IRR (Avg Annual Gross Yield)</t>
+        </is>
+      </c>
+      <c r="C16" s="12">
+        <f>AVERAGE('Annual Model'!C20,'Annual Model'!D20,'Annual Model'!E20,'Annual Model'!F20,'Annual Model'!G20,'Annual Model'!H20,'Annual Model'!I20,'Annual Model'!J20,'Annual Model'!K20,'Annual Model'!L20,'Annual Model'!M20,'Annual Model'!N20,'Annual Model'!O20,'Annual Model'!P20,'Annual Model'!Q20,'Annual Model'!R20,'Annual Model'!S20,'Annual Model'!T20,'Annual Model'!U20,'Annual Model'!V20)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t>JVs</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n"/>
-      <c r="C17" s="10">
-        <f>'Annual Model'!C8</f>
-        <v/>
-      </c>
-      <c r="D17" s="10">
-        <f>'Annual Model'!C15</f>
+      <c r="A17" s="11" t="inlineStr">
+        <is>
+          <t>MOIC (Multiple on Invested Capital)</t>
+        </is>
+      </c>
+      <c r="C17" s="13">
+        <f>'Annual Model'!V48/Summary!$C$5</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr">
-        <is>
-          <t>Securitization Residuals (B-Pieces)</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="n"/>
-      <c r="C18" s="10">
-        <f>'Annual Model'!C9</f>
-        <v/>
-      </c>
-      <c r="D18" s="10">
-        <f>'Annual Model'!C16</f>
+      <c r="A18" s="11" t="inlineStr">
+        <is>
+          <t>DPI (Distributions to Paid-In)</t>
+        </is>
+      </c>
+      <c r="C18" s="13">
+        <f>('Annual Model'!C46+'Annual Model'!D46+'Annual Model'!E46+'Annual Model'!F46+'Annual Model'!G46+'Annual Model'!H46+'Annual Model'!I46+'Annual Model'!J46+'Annual Model'!K46+'Annual Model'!L46+'Annual Model'!M46+'Annual Model'!N46+'Annual Model'!O46+'Annual Model'!P46+'Annual Model'!Q46+'Annual Model'!R46+'Annual Model'!S46+'Annual Model'!T46+'Annual Model'!U46+'Annual Model'!V46)/Summary!$C$5</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t>Cash</t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="n"/>
-      <c r="C19" s="10">
-        <f>'Annual Model'!C10</f>
-        <v/>
-      </c>
-      <c r="D19" s="10">
-        <f>'Annual Model'!C17</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>Total Allocation</t>
-        </is>
-      </c>
-      <c r="C20" s="12">
-        <f>SUM(C15:C19)</f>
-        <v/>
-      </c>
+      <c r="A19" s="11" t="inlineStr">
+        <is>
+          <t>Total Value to Paid-In (TVPI)</t>
+        </is>
+      </c>
+      <c r="C19" s="13">
+        <f>('Annual Model'!V48+'Annual Model'!C46+'Annual Model'!D46+'Annual Model'!E46+'Annual Model'!F46+'Annual Model'!G46+'Annual Model'!H46+'Annual Model'!I46+'Annual Model'!J46+'Annual Model'!K46+'Annual Model'!L46+'Annual Model'!M46+'Annual Model'!N46+'Annual Model'!O46+'Annual Model'!P46+'Annual Model'!Q46+'Annual Model'!R46+'Annual Model'!S46+'Annual Model'!T46+'Annual Model'!U46+'Annual Model'!V46)/Summary!$C$5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Capital Metrics</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="n"/>
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="10" t="n"/>
+      <c r="H21" s="10" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Multi-Year Performance Summary</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="n"/>
-      <c r="C22" s="3" t="n"/>
-      <c r="D22" s="3" t="n"/>
-      <c r="E22" s="3" t="n"/>
-      <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
+      <c r="A22" s="11" t="inlineStr">
+        <is>
+          <t>Initial Committed Capital</t>
+        </is>
+      </c>
+      <c r="C22" s="14">
+        <f>Summary!$C$5</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="B23" s="9" t="inlineStr"/>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>Beginning AUM</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>Gross Yield</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>Net Yield</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>Net Income</t>
-        </is>
-      </c>
-      <c r="G23" s="9" t="inlineStr">
-        <is>
-          <t>Ending AUM</t>
-        </is>
-      </c>
-      <c r="H23" s="9" t="inlineStr"/>
+      <c r="A23" s="11" t="inlineStr">
+        <is>
+          <t>Ending AUM (Year 20)</t>
+        </is>
+      </c>
+      <c r="C23" s="14">
+        <f>'Annual Model'!V48</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="B24" s="14" t="n"/>
-      <c r="C24" s="15">
-        <f>'Annual Model'!C19</f>
-        <v/>
-      </c>
-      <c r="D24" s="10">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
+          <t>Total AUM Growth</t>
+        </is>
+      </c>
+      <c r="C24" s="12">
+        <f>'Annual Model'!V48/Summary!$C$5-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>Total Cumulative Net Income</t>
+        </is>
+      </c>
+      <c r="C25" s="14">
+        <f>'Annual Model'!C46+'Annual Model'!D46+'Annual Model'!E46+'Annual Model'!F46+'Annual Model'!G46+'Annual Model'!H46+'Annual Model'!I46+'Annual Model'!J46+'Annual Model'!K46+'Annual Model'!L46+'Annual Model'!M46+'Annual Model'!N46+'Annual Model'!O46+'Annual Model'!P46+'Annual Model'!Q46+'Annual Model'!R46+'Annual Model'!S46+'Annual Model'!T46+'Annual Model'!U46+'Annual Model'!V46</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>Total Cumulative Gross Income</t>
+        </is>
+      </c>
+      <c r="C26" s="14">
+        <f>'Annual Model'!C36+'Annual Model'!D36+'Annual Model'!E36+'Annual Model'!F36+'Annual Model'!G36+'Annual Model'!H36+'Annual Model'!I36+'Annual Model'!J36+'Annual Model'!K36+'Annual Model'!L36+'Annual Model'!M36+'Annual Model'!N36+'Annual Model'!O36+'Annual Model'!P36+'Annual Model'!Q36+'Annual Model'!R36+'Annual Model'!S36+'Annual Model'!T36+'Annual Model'!U36+'Annual Model'!V36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
+          <t>Peak AUM</t>
+        </is>
+      </c>
+      <c r="C27" s="14">
+        <f>MAX('Annual Model'!C48,'Annual Model'!D48,'Annual Model'!E48,'Annual Model'!F48,'Annual Model'!G48,'Annual Model'!H48,'Annual Model'!I48,'Annual Model'!J48,'Annual Model'!K48,'Annual Model'!L48,'Annual Model'!M48,'Annual Model'!N48,'Annual Model'!O48,'Annual Model'!P48,'Annual Model'!Q48,'Annual Model'!R48,'Annual Model'!S48,'Annual Model'!T48,'Annual Model'!U48,'Annual Model'!V48)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Fee &amp; Expense Metrics</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="n"/>
+      <c r="C29" s="10" t="n"/>
+      <c r="D29" s="10" t="n"/>
+      <c r="E29" s="10" t="n"/>
+      <c r="F29" s="10" t="n"/>
+      <c r="G29" s="10" t="n"/>
+      <c r="H29" s="10" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Total Management Fees</t>
+        </is>
+      </c>
+      <c r="C30" s="14">
+        <f>'Annual Model'!C39+'Annual Model'!D39+'Annual Model'!E39+'Annual Model'!F39+'Annual Model'!G39+'Annual Model'!H39+'Annual Model'!I39+'Annual Model'!J39+'Annual Model'!K39+'Annual Model'!L39+'Annual Model'!M39+'Annual Model'!N39+'Annual Model'!O39+'Annual Model'!P39+'Annual Model'!Q39+'Annual Model'!R39+'Annual Model'!S39+'Annual Model'!T39+'Annual Model'!U39+'Annual Model'!V39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Total Performance Fees</t>
+        </is>
+      </c>
+      <c r="C31" s="14">
+        <f>'Annual Model'!C41+'Annual Model'!D41+'Annual Model'!E41+'Annual Model'!F41+'Annual Model'!G41+'Annual Model'!H41+'Annual Model'!I41+'Annual Model'!J41+'Annual Model'!K41+'Annual Model'!L41+'Annual Model'!M41+'Annual Model'!N41+'Annual Model'!O41+'Annual Model'!P41+'Annual Model'!Q41+'Annual Model'!R41+'Annual Model'!S41+'Annual Model'!T41+'Annual Model'!U41+'Annual Model'!V41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Total Other Expenses</t>
+        </is>
+      </c>
+      <c r="C32" s="14">
+        <f>'Annual Model'!C42+'Annual Model'!D42+'Annual Model'!E42+'Annual Model'!F42+'Annual Model'!G42+'Annual Model'!H42+'Annual Model'!I42+'Annual Model'!J42+'Annual Model'!K42+'Annual Model'!L42+'Annual Model'!M42+'Annual Model'!N42+'Annual Model'!O42+'Annual Model'!P42+'Annual Model'!Q42+'Annual Model'!R42+'Annual Model'!S42+'Annual Model'!T42+'Annual Model'!U42+'Annual Model'!V42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Total All-In Fees &amp; Expenses</t>
+        </is>
+      </c>
+      <c r="C33" s="14">
+        <f>'Annual Model'!C43+'Annual Model'!D43+'Annual Model'!E43+'Annual Model'!F43+'Annual Model'!G43+'Annual Model'!H43+'Annual Model'!I43+'Annual Model'!J43+'Annual Model'!K43+'Annual Model'!L43+'Annual Model'!M43+'Annual Model'!N43+'Annual Model'!O43+'Annual Model'!P43+'Annual Model'!Q43+'Annual Model'!R43+'Annual Model'!S43+'Annual Model'!T43+'Annual Model'!U43+'Annual Model'!V43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>Fee Drag (Fees / Gross Income)</t>
+        </is>
+      </c>
+      <c r="C34" s="12">
+        <f>IF(C26=0,0,C33/C26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="11" t="inlineStr">
+        <is>
+          <t>Net-to-Gross Ratio</t>
+        </is>
+      </c>
+      <c r="C35" s="12">
+        <f>IF(C26=0,0,C25/C26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>Yield &amp; Risk Metrics</t>
+        </is>
+      </c>
+      <c r="B37" s="10" t="n"/>
+      <c r="C37" s="10" t="n"/>
+      <c r="D37" s="10" t="n"/>
+      <c r="E37" s="10" t="n"/>
+      <c r="F37" s="10" t="n"/>
+      <c r="G37" s="10" t="n"/>
+      <c r="H37" s="10" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="11" t="inlineStr">
+        <is>
+          <t>Year 1 Net Yield</t>
+        </is>
+      </c>
+      <c r="C38" s="12">
+        <f>'Annual Model'!C47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="11" t="inlineStr">
+        <is>
+          <t>Year 20 Net Yield</t>
+        </is>
+      </c>
+      <c r="C39" s="12">
+        <f>'Annual Model'!V47</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>Best Year Net Yield</t>
+        </is>
+      </c>
+      <c r="C40" s="12">
+        <f>MAX('Annual Model'!C47,'Annual Model'!D47,'Annual Model'!E47,'Annual Model'!F47,'Annual Model'!G47,'Annual Model'!H47,'Annual Model'!I47,'Annual Model'!J47,'Annual Model'!K47,'Annual Model'!L47,'Annual Model'!M47,'Annual Model'!N47,'Annual Model'!O47,'Annual Model'!P47,'Annual Model'!Q47,'Annual Model'!R47,'Annual Model'!S47,'Annual Model'!T47,'Annual Model'!U47,'Annual Model'!V47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>Worst Year Net Yield</t>
+        </is>
+      </c>
+      <c r="C41" s="12">
+        <f>MIN('Annual Model'!C47,'Annual Model'!D47,'Annual Model'!E47,'Annual Model'!F47,'Annual Model'!G47,'Annual Model'!H47,'Annual Model'!I47,'Annual Model'!J47,'Annual Model'!K47,'Annual Model'!L47,'Annual Model'!M47,'Annual Model'!N47,'Annual Model'!O47,'Annual Model'!P47,'Annual Model'!Q47,'Annual Model'!R47,'Annual Model'!S47,'Annual Model'!T47,'Annual Model'!U47,'Annual Model'!V47)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
+        <is>
+          <t>Year 1 Gross Yield</t>
+        </is>
+      </c>
+      <c r="C42" s="12">
         <f>'Annual Model'!C20</f>
         <v/>
       </c>
-      <c r="E24" s="10">
-        <f>'Annual Model'!C47</f>
-        <v/>
-      </c>
-      <c r="F24" s="15">
-        <f>'Annual Model'!C46</f>
-        <v/>
-      </c>
-      <c r="G24" s="15">
-        <f>'Annual Model'!C48</f>
-        <v/>
-      </c>
-      <c r="H24" s="14" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="13" t="n">
-        <v>2</v>
-      </c>
-      <c r="B25" s="14" t="n"/>
-      <c r="C25" s="15">
-        <f>'Annual Model'!D19</f>
-        <v/>
-      </c>
-      <c r="D25" s="10">
-        <f>'Annual Model'!D20</f>
-        <v/>
-      </c>
-      <c r="E25" s="10">
-        <f>'Annual Model'!D47</f>
-        <v/>
-      </c>
-      <c r="F25" s="15">
-        <f>'Annual Model'!D46</f>
-        <v/>
-      </c>
-      <c r="G25" s="15">
-        <f>'Annual Model'!D48</f>
-        <v/>
-      </c>
-      <c r="H25" s="14" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="13" t="n">
-        <v>3</v>
-      </c>
-      <c r="B26" s="14" t="n"/>
-      <c r="C26" s="15">
-        <f>'Annual Model'!E19</f>
-        <v/>
-      </c>
-      <c r="D26" s="10">
-        <f>'Annual Model'!E20</f>
-        <v/>
-      </c>
-      <c r="E26" s="10">
-        <f>'Annual Model'!E47</f>
-        <v/>
-      </c>
-      <c r="F26" s="15">
-        <f>'Annual Model'!E46</f>
-        <v/>
-      </c>
-      <c r="G26" s="15">
-        <f>'Annual Model'!E48</f>
-        <v/>
-      </c>
-      <c r="H26" s="14" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="13" t="n">
-        <v>4</v>
-      </c>
-      <c r="B27" s="14" t="n"/>
-      <c r="C27" s="15">
-        <f>'Annual Model'!F19</f>
-        <v/>
-      </c>
-      <c r="D27" s="10">
-        <f>'Annual Model'!F20</f>
-        <v/>
-      </c>
-      <c r="E27" s="10">
-        <f>'Annual Model'!F47</f>
-        <v/>
-      </c>
-      <c r="F27" s="15">
-        <f>'Annual Model'!F46</f>
-        <v/>
-      </c>
-      <c r="G27" s="15">
-        <f>'Annual Model'!F48</f>
-        <v/>
-      </c>
-      <c r="H27" s="14" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="B28" s="14" t="n"/>
-      <c r="C28" s="15">
-        <f>'Annual Model'!G19</f>
-        <v/>
-      </c>
-      <c r="D28" s="10">
-        <f>'Annual Model'!G20</f>
-        <v/>
-      </c>
-      <c r="E28" s="10">
-        <f>'Annual Model'!G47</f>
-        <v/>
-      </c>
-      <c r="F28" s="15">
-        <f>'Annual Model'!G46</f>
-        <v/>
-      </c>
-      <c r="G28" s="15">
-        <f>'Annual Model'!G48</f>
-        <v/>
-      </c>
-      <c r="H28" s="14" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="13" t="n">
-        <v>6</v>
-      </c>
-      <c r="B29" s="14" t="n"/>
-      <c r="C29" s="15">
-        <f>'Annual Model'!H19</f>
-        <v/>
-      </c>
-      <c r="D29" s="10">
-        <f>'Annual Model'!H20</f>
-        <v/>
-      </c>
-      <c r="E29" s="10">
-        <f>'Annual Model'!H47</f>
-        <v/>
-      </c>
-      <c r="F29" s="15">
-        <f>'Annual Model'!H46</f>
-        <v/>
-      </c>
-      <c r="G29" s="15">
-        <f>'Annual Model'!H48</f>
-        <v/>
-      </c>
-      <c r="H29" s="14" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="13" t="n">
-        <v>7</v>
-      </c>
-      <c r="B30" s="14" t="n"/>
-      <c r="C30" s="15">
-        <f>'Annual Model'!I19</f>
-        <v/>
-      </c>
-      <c r="D30" s="10">
-        <f>'Annual Model'!I20</f>
-        <v/>
-      </c>
-      <c r="E30" s="10">
-        <f>'Annual Model'!I47</f>
-        <v/>
-      </c>
-      <c r="F30" s="15">
-        <f>'Annual Model'!I46</f>
-        <v/>
-      </c>
-      <c r="G30" s="15">
-        <f>'Annual Model'!I48</f>
-        <v/>
-      </c>
-      <c r="H30" s="14" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="13" t="n">
-        <v>8</v>
-      </c>
-      <c r="B31" s="14" t="n"/>
-      <c r="C31" s="15">
-        <f>'Annual Model'!J19</f>
-        <v/>
-      </c>
-      <c r="D31" s="10">
-        <f>'Annual Model'!J20</f>
-        <v/>
-      </c>
-      <c r="E31" s="10">
-        <f>'Annual Model'!J47</f>
-        <v/>
-      </c>
-      <c r="F31" s="15">
-        <f>'Annual Model'!J46</f>
-        <v/>
-      </c>
-      <c r="G31" s="15">
-        <f>'Annual Model'!J48</f>
-        <v/>
-      </c>
-      <c r="H31" s="14" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="13" t="n">
-        <v>9</v>
-      </c>
-      <c r="B32" s="14" t="n"/>
-      <c r="C32" s="15">
-        <f>'Annual Model'!K19</f>
-        <v/>
-      </c>
-      <c r="D32" s="10">
-        <f>'Annual Model'!K20</f>
-        <v/>
-      </c>
-      <c r="E32" s="10">
-        <f>'Annual Model'!K47</f>
-        <v/>
-      </c>
-      <c r="F32" s="15">
-        <f>'Annual Model'!K46</f>
-        <v/>
-      </c>
-      <c r="G32" s="15">
-        <f>'Annual Model'!K48</f>
-        <v/>
-      </c>
-      <c r="H32" s="14" t="n"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="13" t="n">
-        <v>10</v>
-      </c>
-      <c r="B33" s="14" t="n"/>
-      <c r="C33" s="15">
-        <f>'Annual Model'!L19</f>
-        <v/>
-      </c>
-      <c r="D33" s="10">
-        <f>'Annual Model'!L20</f>
-        <v/>
-      </c>
-      <c r="E33" s="10">
-        <f>'Annual Model'!L47</f>
-        <v/>
-      </c>
-      <c r="F33" s="15">
-        <f>'Annual Model'!L46</f>
-        <v/>
-      </c>
-      <c r="G33" s="15">
-        <f>'Annual Model'!L48</f>
-        <v/>
-      </c>
-      <c r="H33" s="14" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="13" t="n">
-        <v>11</v>
-      </c>
-      <c r="B34" s="14" t="n"/>
-      <c r="C34" s="15">
-        <f>'Annual Model'!M19</f>
-        <v/>
-      </c>
-      <c r="D34" s="10">
-        <f>'Annual Model'!M20</f>
-        <v/>
-      </c>
-      <c r="E34" s="10">
-        <f>'Annual Model'!M47</f>
-        <v/>
-      </c>
-      <c r="F34" s="15">
-        <f>'Annual Model'!M46</f>
-        <v/>
-      </c>
-      <c r="G34" s="15">
-        <f>'Annual Model'!M48</f>
-        <v/>
-      </c>
-      <c r="H34" s="14" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="B35" s="14" t="n"/>
-      <c r="C35" s="15">
-        <f>'Annual Model'!N19</f>
-        <v/>
-      </c>
-      <c r="D35" s="10">
-        <f>'Annual Model'!N20</f>
-        <v/>
-      </c>
-      <c r="E35" s="10">
-        <f>'Annual Model'!N47</f>
-        <v/>
-      </c>
-      <c r="F35" s="15">
-        <f>'Annual Model'!N46</f>
-        <v/>
-      </c>
-      <c r="G35" s="15">
-        <f>'Annual Model'!N48</f>
-        <v/>
-      </c>
-      <c r="H35" s="14" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="13" t="n">
-        <v>13</v>
-      </c>
-      <c r="B36" s="14" t="n"/>
-      <c r="C36" s="15">
-        <f>'Annual Model'!O19</f>
-        <v/>
-      </c>
-      <c r="D36" s="10">
-        <f>'Annual Model'!O20</f>
-        <v/>
-      </c>
-      <c r="E36" s="10">
-        <f>'Annual Model'!O47</f>
-        <v/>
-      </c>
-      <c r="F36" s="15">
-        <f>'Annual Model'!O46</f>
-        <v/>
-      </c>
-      <c r="G36" s="15">
-        <f>'Annual Model'!O48</f>
-        <v/>
-      </c>
-      <c r="H36" s="14" t="n"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="13" t="n">
-        <v>14</v>
-      </c>
-      <c r="B37" s="14" t="n"/>
-      <c r="C37" s="15">
-        <f>'Annual Model'!P19</f>
-        <v/>
-      </c>
-      <c r="D37" s="10">
-        <f>'Annual Model'!P20</f>
-        <v/>
-      </c>
-      <c r="E37" s="10">
-        <f>'Annual Model'!P47</f>
-        <v/>
-      </c>
-      <c r="F37" s="15">
-        <f>'Annual Model'!P46</f>
-        <v/>
-      </c>
-      <c r="G37" s="15">
-        <f>'Annual Model'!P48</f>
-        <v/>
-      </c>
-      <c r="H37" s="14" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="13" t="n">
-        <v>15</v>
-      </c>
-      <c r="B38" s="14" t="n"/>
-      <c r="C38" s="15">
-        <f>'Annual Model'!Q19</f>
-        <v/>
-      </c>
-      <c r="D38" s="10">
-        <f>'Annual Model'!Q20</f>
-        <v/>
-      </c>
-      <c r="E38" s="10">
-        <f>'Annual Model'!Q47</f>
-        <v/>
-      </c>
-      <c r="F38" s="15">
-        <f>'Annual Model'!Q46</f>
-        <v/>
-      </c>
-      <c r="G38" s="15">
-        <f>'Annual Model'!Q48</f>
-        <v/>
-      </c>
-      <c r="H38" s="14" t="n"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="13" t="n">
-        <v>16</v>
-      </c>
-      <c r="B39" s="14" t="n"/>
-      <c r="C39" s="15">
-        <f>'Annual Model'!R19</f>
-        <v/>
-      </c>
-      <c r="D39" s="10">
-        <f>'Annual Model'!R20</f>
-        <v/>
-      </c>
-      <c r="E39" s="10">
-        <f>'Annual Model'!R47</f>
-        <v/>
-      </c>
-      <c r="F39" s="15">
-        <f>'Annual Model'!R46</f>
-        <v/>
-      </c>
-      <c r="G39" s="15">
-        <f>'Annual Model'!R48</f>
-        <v/>
-      </c>
-      <c r="H39" s="14" t="n"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="13" t="n">
-        <v>17</v>
-      </c>
-      <c r="B40" s="14" t="n"/>
-      <c r="C40" s="15">
-        <f>'Annual Model'!S19</f>
-        <v/>
-      </c>
-      <c r="D40" s="10">
-        <f>'Annual Model'!S20</f>
-        <v/>
-      </c>
-      <c r="E40" s="10">
-        <f>'Annual Model'!S47</f>
-        <v/>
-      </c>
-      <c r="F40" s="15">
-        <f>'Annual Model'!S46</f>
-        <v/>
-      </c>
-      <c r="G40" s="15">
-        <f>'Annual Model'!S48</f>
-        <v/>
-      </c>
-      <c r="H40" s="14" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="13" t="n">
-        <v>18</v>
-      </c>
-      <c r="B41" s="14" t="n"/>
-      <c r="C41" s="15">
-        <f>'Annual Model'!T19</f>
-        <v/>
-      </c>
-      <c r="D41" s="10">
-        <f>'Annual Model'!T20</f>
-        <v/>
-      </c>
-      <c r="E41" s="10">
-        <f>'Annual Model'!T47</f>
-        <v/>
-      </c>
-      <c r="F41" s="15">
-        <f>'Annual Model'!T46</f>
-        <v/>
-      </c>
-      <c r="G41" s="15">
-        <f>'Annual Model'!T48</f>
-        <v/>
-      </c>
-      <c r="H41" s="14" t="n"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="13" t="n">
-        <v>19</v>
-      </c>
-      <c r="B42" s="14" t="n"/>
-      <c r="C42" s="15">
-        <f>'Annual Model'!U19</f>
-        <v/>
-      </c>
-      <c r="D42" s="10">
-        <f>'Annual Model'!U20</f>
-        <v/>
-      </c>
-      <c r="E42" s="10">
-        <f>'Annual Model'!U47</f>
-        <v/>
-      </c>
-      <c r="F42" s="15">
-        <f>'Annual Model'!U46</f>
-        <v/>
-      </c>
-      <c r="G42" s="15">
-        <f>'Annual Model'!U48</f>
-        <v/>
-      </c>
-      <c r="H42" s="14" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="13" t="n">
-        <v>20</v>
-      </c>
-      <c r="B43" s="14" t="n"/>
-      <c r="C43" s="15">
-        <f>'Annual Model'!V19</f>
-        <v/>
-      </c>
-      <c r="D43" s="10">
-        <f>'Annual Model'!V20</f>
-        <v/>
-      </c>
-      <c r="E43" s="10">
-        <f>'Annual Model'!V47</f>
-        <v/>
-      </c>
-      <c r="F43" s="15">
-        <f>'Annual Model'!V46</f>
-        <v/>
-      </c>
-      <c r="G43" s="15">
-        <f>'Annual Model'!V48</f>
-        <v/>
-      </c>
-      <c r="H43" s="14" t="n"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="3" t="inlineStr">
-        <is>
-          <t>Key Metrics</t>
-        </is>
-      </c>
-      <c r="B45" s="3" t="n"/>
-      <c r="C45" s="3" t="n"/>
-      <c r="D45" s="3" t="n"/>
-      <c r="E45" s="3" t="n"/>
-      <c r="F45" s="3" t="n"/>
-      <c r="G45" s="3" t="n"/>
-      <c r="H45" s="3" t="n"/>
+      <c r="A43" s="11" t="inlineStr">
+        <is>
+          <t>Gross-to-Net Spread (Avg)</t>
+        </is>
+      </c>
+      <c r="C43" s="12">
+        <f>C16-C15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
+        <is>
+          <t>Leverage Contribution (Year 1)</t>
+        </is>
+      </c>
+      <c r="C44" s="12">
+        <f>IF('Annual Model'!C28=0,0,'Annual Model'!C34/'Annual Model'!C28)</f>
+        <v/>
+      </c>
     </row>
     <row r="46">
-      <c r="A46" s="16" t="inlineStr">
-        <is>
-          <t>Cumulative Net Income</t>
-        </is>
-      </c>
-      <c r="C46" s="17">
-        <f>SUM(F24:F43)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" s="16" t="inlineStr">
-        <is>
-          <t>Average Net Yield (Annualized)</t>
-        </is>
-      </c>
-      <c r="C47" s="18">
-        <f>AVERAGE(E24:E43)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" s="16" t="inlineStr">
-        <is>
-          <t>Total AUM Growth</t>
-        </is>
-      </c>
-      <c r="C48" s="18">
-        <f>G43/C24-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="16" t="inlineStr">
-        <is>
-          <t>Total Management Fees Paid</t>
-        </is>
-      </c>
-      <c r="C49" s="17">
-        <f>'Annual Model'!C39+'Annual Model'!D39+'Annual Model'!E39+'Annual Model'!F39+'Annual Model'!G39+'Annual Model'!H39+'Annual Model'!I39+'Annual Model'!J39+'Annual Model'!K39+'Annual Model'!L39+'Annual Model'!M39+'Annual Model'!N39+'Annual Model'!O39+'Annual Model'!P39+'Annual Model'!Q39+'Annual Model'!R39+'Annual Model'!S39+'Annual Model'!T39+'Annual Model'!U39+'Annual Model'!V39</f>
-        <v/>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="16" t="inlineStr">
-        <is>
-          <t>Total Performance Fees Paid</t>
-        </is>
-      </c>
-      <c r="C50" s="17">
-        <f>'Annual Model'!C41+'Annual Model'!D41+'Annual Model'!E41+'Annual Model'!F41+'Annual Model'!G41+'Annual Model'!H41+'Annual Model'!I41+'Annual Model'!J41+'Annual Model'!K41+'Annual Model'!L41+'Annual Model'!M41+'Annual Model'!N41+'Annual Model'!O41+'Annual Model'!P41+'Annual Model'!Q41+'Annual Model'!R41+'Annual Model'!S41+'Annual Model'!T41+'Annual Model'!U41+'Annual Model'!V41</f>
-        <v/>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" s="19" t="inlineStr">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>Input cells are highlighted in orange. Modify inputs to update the model.</t>
         </is>
       </c>
-      <c r="E52" s="20">
+      <c r="E46" s="16">
         <f> Input</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="24">
-    <mergeCell ref="A48:B48"/>
+  <mergeCells count="35">
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A30:B30"/>
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="A11:B11"/>
-    <mergeCell ref="A49:B49"/>
-    <mergeCell ref="A52:D52"/>
-    <mergeCell ref="A45:H45"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A16:B16"/>
     <mergeCell ref="A7:B7"/>
-    <mergeCell ref="A46:B46"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="A41:B41"/>
     <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A50:B50"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="A26:B26"/>
     <mergeCell ref="A3:H3"/>
-    <mergeCell ref="A47:B47"/>
+    <mergeCell ref="A33:B33"/>
     <mergeCell ref="A5:B5"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="A32:B32"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="A17:B17"/>
     <mergeCell ref="A8:B8"/>
-    <mergeCell ref="A22:H22"/>
-    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A46:D46"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A35:B35"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="A43:B43"/>
     <mergeCell ref="A19:B19"/>
     <mergeCell ref="A10:B10"/>
     <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A44:B44"/>
+    <mergeCell ref="A40:B40"/>
     <mergeCell ref="A9:B9"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="A34:B34"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1705,938 +1267,938 @@
       <c r="V3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="inlineStr"/>
-      <c r="B4" s="22" t="n"/>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr"/>
+      <c r="B4" s="17" t="n"/>
+      <c r="C4" s="18" t="inlineStr">
         <is>
           <t>Year 1</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="18" t="inlineStr">
         <is>
           <t>Year 2</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="18" t="inlineStr">
         <is>
           <t>Year 3</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
+      <c r="F4" s="18" t="inlineStr">
         <is>
           <t>Year 4</t>
         </is>
       </c>
-      <c r="G4" s="9" t="inlineStr">
+      <c r="G4" s="18" t="inlineStr">
         <is>
           <t>Year 5</t>
         </is>
       </c>
-      <c r="H4" s="9" t="inlineStr">
+      <c r="H4" s="18" t="inlineStr">
         <is>
           <t>Year 6</t>
         </is>
       </c>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="I4" s="18" t="inlineStr">
         <is>
           <t>Year 7</t>
         </is>
       </c>
-      <c r="J4" s="9" t="inlineStr">
+      <c r="J4" s="18" t="inlineStr">
         <is>
           <t>Year 8</t>
         </is>
       </c>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="K4" s="18" t="inlineStr">
         <is>
           <t>Year 9</t>
         </is>
       </c>
-      <c r="L4" s="9" t="inlineStr">
+      <c r="L4" s="18" t="inlineStr">
         <is>
           <t>Year 10</t>
         </is>
       </c>
-      <c r="M4" s="9" t="inlineStr">
+      <c r="M4" s="18" t="inlineStr">
         <is>
           <t>Year 11</t>
         </is>
       </c>
-      <c r="N4" s="9" t="inlineStr">
+      <c r="N4" s="18" t="inlineStr">
         <is>
           <t>Year 12</t>
         </is>
       </c>
-      <c r="O4" s="9" t="inlineStr">
+      <c r="O4" s="18" t="inlineStr">
         <is>
           <t>Year 13</t>
         </is>
       </c>
-      <c r="P4" s="9" t="inlineStr">
+      <c r="P4" s="18" t="inlineStr">
         <is>
           <t>Year 14</t>
         </is>
       </c>
-      <c r="Q4" s="9" t="inlineStr">
+      <c r="Q4" s="18" t="inlineStr">
         <is>
           <t>Year 15</t>
         </is>
       </c>
-      <c r="R4" s="9" t="inlineStr">
+      <c r="R4" s="18" t="inlineStr">
         <is>
           <t>Year 16</t>
         </is>
       </c>
-      <c r="S4" s="9" t="inlineStr">
+      <c r="S4" s="18" t="inlineStr">
         <is>
           <t>Year 17</t>
         </is>
       </c>
-      <c r="T4" s="9" t="inlineStr">
+      <c r="T4" s="18" t="inlineStr">
         <is>
           <t>Year 18</t>
         </is>
       </c>
-      <c r="U4" s="9" t="inlineStr">
+      <c r="U4" s="18" t="inlineStr">
         <is>
           <t>Year 19</t>
         </is>
       </c>
-      <c r="V4" s="9" t="inlineStr">
+      <c r="V4" s="18" t="inlineStr">
         <is>
           <t>Year 20</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Asset Allocation</t>
         </is>
       </c>
-      <c r="B5" s="21" t="inlineStr">
+      <c r="B5" s="10" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C5" s="21" t="n"/>
-      <c r="D5" s="21" t="n"/>
-      <c r="E5" s="21" t="n"/>
-      <c r="F5" s="21" t="n"/>
-      <c r="G5" s="21" t="n"/>
-      <c r="H5" s="21" t="n"/>
-      <c r="I5" s="21" t="n"/>
-      <c r="J5" s="21" t="n"/>
-      <c r="K5" s="21" t="n"/>
-      <c r="L5" s="21" t="n"/>
-      <c r="M5" s="21" t="n"/>
-      <c r="N5" s="21" t="n"/>
-      <c r="O5" s="21" t="n"/>
-      <c r="P5" s="21" t="n"/>
-      <c r="Q5" s="21" t="n"/>
-      <c r="R5" s="21" t="n"/>
-      <c r="S5" s="21" t="n"/>
-      <c r="T5" s="21" t="n"/>
-      <c r="U5" s="21" t="n"/>
-      <c r="V5" s="21" t="n"/>
+      <c r="C5" s="10" t="n"/>
+      <c r="D5" s="10" t="n"/>
+      <c r="E5" s="10" t="n"/>
+      <c r="F5" s="10" t="n"/>
+      <c r="G5" s="10" t="n"/>
+      <c r="H5" s="10" t="n"/>
+      <c r="I5" s="10" t="n"/>
+      <c r="J5" s="10" t="n"/>
+      <c r="K5" s="10" t="n"/>
+      <c r="L5" s="10" t="n"/>
+      <c r="M5" s="10" t="n"/>
+      <c r="N5" s="10" t="n"/>
+      <c r="O5" s="10" t="n"/>
+      <c r="P5" s="10" t="n"/>
+      <c r="Q5" s="10" t="n"/>
+      <c r="R5" s="10" t="n"/>
+      <c r="S5" s="10" t="n"/>
+      <c r="T5" s="10" t="n"/>
+      <c r="U5" s="10" t="n"/>
+      <c r="V5" s="10" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>LIHTC Loans</t>
         </is>
       </c>
-      <c r="B6" s="14" t="n"/>
-      <c r="C6" s="25" t="n">
+      <c r="B6" s="19" t="n"/>
+      <c r="C6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="D6" s="25" t="n">
+      <c r="D6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="E6" s="25" t="n">
+      <c r="E6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="F6" s="25" t="n">
+      <c r="F6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="G6" s="25" t="n">
+      <c r="G6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="H6" s="25" t="n">
+      <c r="H6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="I6" s="25" t="n">
+      <c r="I6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="J6" s="25" t="n">
+      <c r="J6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="K6" s="25" t="n">
+      <c r="K6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="L6" s="25" t="n">
+      <c r="L6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="M6" s="25" t="n">
+      <c r="M6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="N6" s="25" t="n">
+      <c r="N6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="O6" s="25" t="n">
+      <c r="O6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="P6" s="25" t="n">
+      <c r="P6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="Q6" s="25" t="n">
+      <c r="Q6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="R6" s="25" t="n">
+      <c r="R6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="S6" s="25" t="n">
+      <c r="S6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="T6" s="25" t="n">
+      <c r="T6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="U6" s="25" t="n">
+      <c r="U6" s="20" t="n">
         <v>0.35</v>
       </c>
-      <c r="V6" s="25" t="n">
+      <c r="V6" s="20" t="n">
         <v>0.35</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>Municipal Bonds</t>
         </is>
       </c>
-      <c r="B7" s="14" t="n"/>
-      <c r="C7" s="25" t="n">
+      <c r="B7" s="19" t="n"/>
+      <c r="C7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="D7" s="25" t="n">
+      <c r="D7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="E7" s="25" t="n">
+      <c r="E7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="F7" s="25" t="n">
+      <c r="F7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="G7" s="25" t="n">
+      <c r="G7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="H7" s="25" t="n">
+      <c r="H7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="I7" s="25" t="n">
+      <c r="I7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="J7" s="25" t="n">
+      <c r="J7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="K7" s="25" t="n">
+      <c r="K7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="L7" s="25" t="n">
+      <c r="L7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="M7" s="25" t="n">
+      <c r="M7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="N7" s="25" t="n">
+      <c r="N7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="O7" s="25" t="n">
+      <c r="O7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="P7" s="25" t="n">
+      <c r="P7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q7" s="25" t="n">
+      <c r="Q7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="R7" s="25" t="n">
+      <c r="R7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="S7" s="25" t="n">
+      <c r="S7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="T7" s="25" t="n">
+      <c r="T7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="U7" s="25" t="n">
+      <c r="U7" s="20" t="n">
         <v>0.25</v>
       </c>
-      <c r="V7" s="25" t="n">
+      <c r="V7" s="20" t="n">
         <v>0.25</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>JVs</t>
         </is>
       </c>
-      <c r="B8" s="14" t="n"/>
-      <c r="C8" s="25" t="n">
+      <c r="B8" s="19" t="n"/>
+      <c r="C8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="D8" s="25" t="n">
+      <c r="D8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="E8" s="25" t="n">
+      <c r="E8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="F8" s="25" t="n">
+      <c r="F8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="G8" s="25" t="n">
+      <c r="G8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="H8" s="25" t="n">
+      <c r="H8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="I8" s="25" t="n">
+      <c r="I8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="J8" s="25" t="n">
+      <c r="J8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="K8" s="25" t="n">
+      <c r="K8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="L8" s="25" t="n">
+      <c r="L8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="M8" s="25" t="n">
+      <c r="M8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="N8" s="25" t="n">
+      <c r="N8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="O8" s="25" t="n">
+      <c r="O8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="P8" s="25" t="n">
+      <c r="P8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="Q8" s="25" t="n">
+      <c r="Q8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="R8" s="25" t="n">
+      <c r="R8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="S8" s="25" t="n">
+      <c r="S8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="T8" s="25" t="n">
+      <c r="T8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="U8" s="25" t="n">
+      <c r="U8" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="V8" s="25" t="n">
+      <c r="V8" s="20" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>Securitization Residuals (B-Pieces)</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n"/>
-      <c r="C9" s="25" t="n">
+      <c r="B9" s="19" t="n"/>
+      <c r="C9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="D9" s="25" t="n">
+      <c r="D9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="E9" s="25" t="n">
+      <c r="E9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="F9" s="25" t="n">
+      <c r="F9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="G9" s="25" t="n">
+      <c r="G9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="H9" s="25" t="n">
+      <c r="H9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="I9" s="25" t="n">
+      <c r="I9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="J9" s="25" t="n">
+      <c r="J9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="K9" s="25" t="n">
+      <c r="K9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="L9" s="25" t="n">
+      <c r="L9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="M9" s="25" t="n">
+      <c r="M9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="N9" s="25" t="n">
+      <c r="N9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="O9" s="25" t="n">
+      <c r="O9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="P9" s="25" t="n">
+      <c r="P9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="Q9" s="25" t="n">
+      <c r="Q9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="R9" s="25" t="n">
+      <c r="R9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="S9" s="25" t="n">
+      <c r="S9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="T9" s="25" t="n">
+      <c r="T9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="U9" s="25" t="n">
+      <c r="U9" s="20" t="n">
         <v>0.15</v>
       </c>
-      <c r="V9" s="25" t="n">
+      <c r="V9" s="20" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="B10" s="14" t="n"/>
-      <c r="C10" s="25" t="n">
+      <c r="B10" s="19" t="n"/>
+      <c r="C10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="D10" s="25" t="n">
+      <c r="D10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="E10" s="25" t="n">
+      <c r="E10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="F10" s="25" t="n">
+      <c r="F10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="G10" s="25" t="n">
+      <c r="G10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="H10" s="25" t="n">
+      <c r="H10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="I10" s="25" t="n">
+      <c r="I10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="J10" s="25" t="n">
+      <c r="J10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="K10" s="25" t="n">
+      <c r="K10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="L10" s="25" t="n">
+      <c r="L10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="M10" s="25" t="n">
+      <c r="M10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="N10" s="25" t="n">
+      <c r="N10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="O10" s="25" t="n">
+      <c r="O10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="P10" s="25" t="n">
+      <c r="P10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q10" s="25" t="n">
+      <c r="Q10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="R10" s="25" t="n">
+      <c r="R10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="S10" s="25" t="n">
+      <c r="S10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="T10" s="25" t="n">
+      <c r="T10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="U10" s="25" t="n">
+      <c r="U10" s="20" t="n">
         <v>0.1</v>
       </c>
-      <c r="V10" s="25" t="n">
+      <c r="V10" s="20" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>Total Allocation</t>
         </is>
       </c>
-      <c r="B11" s="14" t="n"/>
-      <c r="C11" s="12">
+      <c r="B11" s="19" t="n"/>
+      <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="12">
+      <c r="D11" s="22">
         <f>SUM(D6:D10)</f>
         <v/>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="22">
         <f>SUM(E6:E10)</f>
         <v/>
       </c>
-      <c r="F11" s="12">
+      <c r="F11" s="22">
         <f>SUM(F6:F10)</f>
         <v/>
       </c>
-      <c r="G11" s="12">
+      <c r="G11" s="22">
         <f>SUM(G6:G10)</f>
         <v/>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="22">
         <f>SUM(H6:H10)</f>
         <v/>
       </c>
-      <c r="I11" s="12">
+      <c r="I11" s="22">
         <f>SUM(I6:I10)</f>
         <v/>
       </c>
-      <c r="J11" s="12">
+      <c r="J11" s="22">
         <f>SUM(J6:J10)</f>
         <v/>
       </c>
-      <c r="K11" s="12">
+      <c r="K11" s="22">
         <f>SUM(K6:K10)</f>
         <v/>
       </c>
-      <c r="L11" s="12">
+      <c r="L11" s="22">
         <f>SUM(L6:L10)</f>
         <v/>
       </c>
-      <c r="M11" s="12">
+      <c r="M11" s="22">
         <f>SUM(M6:M10)</f>
         <v/>
       </c>
-      <c r="N11" s="12">
+      <c r="N11" s="22">
         <f>SUM(N6:N10)</f>
         <v/>
       </c>
-      <c r="O11" s="12">
+      <c r="O11" s="22">
         <f>SUM(O6:O10)</f>
         <v/>
       </c>
-      <c r="P11" s="12">
+      <c r="P11" s="22">
         <f>SUM(P6:P10)</f>
         <v/>
       </c>
-      <c r="Q11" s="12">
+      <c r="Q11" s="22">
         <f>SUM(Q6:Q10)</f>
         <v/>
       </c>
-      <c r="R11" s="12">
+      <c r="R11" s="22">
         <f>SUM(R6:R10)</f>
         <v/>
       </c>
-      <c r="S11" s="12">
+      <c r="S11" s="22">
         <f>SUM(S6:S10)</f>
         <v/>
       </c>
-      <c r="T11" s="12">
+      <c r="T11" s="22">
         <f>SUM(T6:T10)</f>
         <v/>
       </c>
-      <c r="U11" s="12">
+      <c r="U11" s="22">
         <f>SUM(U6:U10)</f>
         <v/>
       </c>
-      <c r="V11" s="12">
+      <c r="V11" s="22">
         <f>SUM(V6:V10)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="23" t="inlineStr">
+      <c r="A12" s="9" t="inlineStr">
         <is>
           <t>Expected Yields</t>
         </is>
       </c>
-      <c r="B12" s="21" t="inlineStr">
+      <c r="B12" s="10" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C12" s="21" t="n"/>
-      <c r="D12" s="21" t="n"/>
-      <c r="E12" s="21" t="n"/>
-      <c r="F12" s="21" t="n"/>
-      <c r="G12" s="21" t="n"/>
-      <c r="H12" s="21" t="n"/>
-      <c r="I12" s="21" t="n"/>
-      <c r="J12" s="21" t="n"/>
-      <c r="K12" s="21" t="n"/>
-      <c r="L12" s="21" t="n"/>
-      <c r="M12" s="21" t="n"/>
-      <c r="N12" s="21" t="n"/>
-      <c r="O12" s="21" t="n"/>
-      <c r="P12" s="21" t="n"/>
-      <c r="Q12" s="21" t="n"/>
-      <c r="R12" s="21" t="n"/>
-      <c r="S12" s="21" t="n"/>
-      <c r="T12" s="21" t="n"/>
-      <c r="U12" s="21" t="n"/>
-      <c r="V12" s="21" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
+      <c r="H12" s="10" t="n"/>
+      <c r="I12" s="10" t="n"/>
+      <c r="J12" s="10" t="n"/>
+      <c r="K12" s="10" t="n"/>
+      <c r="L12" s="10" t="n"/>
+      <c r="M12" s="10" t="n"/>
+      <c r="N12" s="10" t="n"/>
+      <c r="O12" s="10" t="n"/>
+      <c r="P12" s="10" t="n"/>
+      <c r="Q12" s="10" t="n"/>
+      <c r="R12" s="10" t="n"/>
+      <c r="S12" s="10" t="n"/>
+      <c r="T12" s="10" t="n"/>
+      <c r="U12" s="10" t="n"/>
+      <c r="V12" s="10" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="24" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>LIHTC Loans</t>
         </is>
       </c>
-      <c r="B13" s="14" t="n"/>
-      <c r="C13" s="25" t="n">
+      <c r="B13" s="19" t="n"/>
+      <c r="C13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="D13" s="25" t="n">
+      <c r="D13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="E13" s="25" t="n">
+      <c r="E13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="F13" s="25" t="n">
+      <c r="F13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="G13" s="25" t="n">
+      <c r="G13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="H13" s="25" t="n">
+      <c r="H13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="I13" s="25" t="n">
+      <c r="I13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="J13" s="25" t="n">
+      <c r="J13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="K13" s="25" t="n">
+      <c r="K13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="L13" s="25" t="n">
+      <c r="L13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="M13" s="25" t="n">
+      <c r="M13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="N13" s="25" t="n">
+      <c r="N13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="O13" s="25" t="n">
+      <c r="O13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="P13" s="25" t="n">
+      <c r="P13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q13" s="25" t="n">
+      <c r="Q13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="R13" s="25" t="n">
+      <c r="R13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="S13" s="25" t="n">
+      <c r="S13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="T13" s="25" t="n">
+      <c r="T13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="U13" s="25" t="n">
+      <c r="U13" s="20" t="n">
         <v>0.065</v>
       </c>
-      <c r="V13" s="25" t="n">
+      <c r="V13" s="20" t="n">
         <v>0.065</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="24" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>Municipal Bonds</t>
         </is>
       </c>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="25" t="n">
+      <c r="B14" s="19" t="n"/>
+      <c r="C14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="D14" s="25" t="n">
+      <c r="D14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="E14" s="25" t="n">
+      <c r="E14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="F14" s="25" t="n">
+      <c r="F14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="G14" s="25" t="n">
+      <c r="G14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="H14" s="25" t="n">
+      <c r="H14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="I14" s="25" t="n">
+      <c r="I14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="J14" s="25" t="n">
+      <c r="J14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="K14" s="25" t="n">
+      <c r="K14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="L14" s="25" t="n">
+      <c r="L14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="M14" s="25" t="n">
+      <c r="M14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="N14" s="25" t="n">
+      <c r="N14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="O14" s="25" t="n">
+      <c r="O14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="P14" s="25" t="n">
+      <c r="P14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="Q14" s="25" t="n">
+      <c r="Q14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="R14" s="25" t="n">
+      <c r="R14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="S14" s="25" t="n">
+      <c r="S14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="T14" s="25" t="n">
+      <c r="T14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="U14" s="25" t="n">
+      <c r="U14" s="20" t="n">
         <v>0.045</v>
       </c>
-      <c r="V14" s="25" t="n">
+      <c r="V14" s="20" t="n">
         <v>0.045</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="24" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>JVs</t>
         </is>
       </c>
-      <c r="B15" s="14" t="n"/>
-      <c r="C15" s="25" t="n">
+      <c r="B15" s="19" t="n"/>
+      <c r="C15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="D15" s="25" t="n">
+      <c r="D15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="E15" s="25" t="n">
+      <c r="E15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="F15" s="25" t="n">
+      <c r="F15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="G15" s="25" t="n">
+      <c r="G15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="H15" s="25" t="n">
+      <c r="H15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="I15" s="25" t="n">
+      <c r="I15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="J15" s="25" t="n">
+      <c r="J15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="K15" s="25" t="n">
+      <c r="K15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="L15" s="25" t="n">
+      <c r="L15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="M15" s="25" t="n">
+      <c r="M15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="N15" s="25" t="n">
+      <c r="N15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="O15" s="25" t="n">
+      <c r="O15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="P15" s="25" t="n">
+      <c r="P15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="Q15" s="25" t="n">
+      <c r="Q15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="R15" s="25" t="n">
+      <c r="R15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="S15" s="25" t="n">
+      <c r="S15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="T15" s="25" t="n">
+      <c r="T15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="U15" s="25" t="n">
+      <c r="U15" s="20" t="n">
         <v>0.08</v>
       </c>
-      <c r="V15" s="25" t="n">
+      <c r="V15" s="20" t="n">
         <v>0.08</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="24" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Securitization Residuals (B-Pieces)</t>
         </is>
       </c>
-      <c r="B16" s="14" t="n"/>
-      <c r="C16" s="25" t="n">
+      <c r="B16" s="19" t="n"/>
+      <c r="C16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="D16" s="25" t="n">
+      <c r="D16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="E16" s="25" t="n">
+      <c r="E16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="F16" s="25" t="n">
+      <c r="F16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="G16" s="25" t="n">
+      <c r="G16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="H16" s="25" t="n">
+      <c r="H16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="I16" s="25" t="n">
+      <c r="I16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="J16" s="25" t="n">
+      <c r="J16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="K16" s="25" t="n">
+      <c r="K16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="L16" s="25" t="n">
+      <c r="L16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="M16" s="25" t="n">
+      <c r="M16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="N16" s="25" t="n">
+      <c r="N16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="O16" s="25" t="n">
+      <c r="O16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="P16" s="25" t="n">
+      <c r="P16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="Q16" s="25" t="n">
+      <c r="Q16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="R16" s="25" t="n">
+      <c r="R16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="S16" s="25" t="n">
+      <c r="S16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="T16" s="25" t="n">
+      <c r="T16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="U16" s="25" t="n">
+      <c r="U16" s="20" t="n">
         <v>0.075</v>
       </c>
-      <c r="V16" s="25" t="n">
+      <c r="V16" s="20" t="n">
         <v>0.075</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="24" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="B17" s="14" t="n"/>
-      <c r="C17" s="25" t="n">
+      <c r="B17" s="19" t="n"/>
+      <c r="C17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="D17" s="25" t="n">
+      <c r="D17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="E17" s="25" t="n">
+      <c r="E17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="F17" s="25" t="n">
+      <c r="F17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="G17" s="25" t="n">
+      <c r="G17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="H17" s="25" t="n">
+      <c r="H17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="I17" s="25" t="n">
+      <c r="I17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="J17" s="25" t="n">
+      <c r="J17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="K17" s="25" t="n">
+      <c r="K17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="L17" s="25" t="n">
+      <c r="L17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="M17" s="25" t="n">
+      <c r="M17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="N17" s="25" t="n">
+      <c r="N17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="O17" s="25" t="n">
+      <c r="O17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="P17" s="25" t="n">
+      <c r="P17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="Q17" s="25" t="n">
+      <c r="Q17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="R17" s="25" t="n">
+      <c r="R17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="S17" s="25" t="n">
+      <c r="S17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="T17" s="25" t="n">
+      <c r="T17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="U17" s="25" t="n">
+      <c r="U17" s="20" t="n">
         <v>0.02</v>
       </c>
-      <c r="V17" s="25" t="n">
+      <c r="V17" s="20" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -2669,1217 +2231,1217 @@
       <c r="V18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>Beginning AUM</t>
         </is>
       </c>
-      <c r="B19" s="26" t="inlineStr">
+      <c r="B19" s="23" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="C19" s="17">
+      <c r="C19" s="14">
         <f>Summary!$C$5</f>
         <v/>
       </c>
-      <c r="D19" s="17">
+      <c r="D19" s="14">
         <f>C48</f>
         <v/>
       </c>
-      <c r="E19" s="17">
+      <c r="E19" s="14">
         <f>D48</f>
         <v/>
       </c>
-      <c r="F19" s="17">
+      <c r="F19" s="14">
         <f>E48</f>
         <v/>
       </c>
-      <c r="G19" s="17">
+      <c r="G19" s="14">
         <f>F48</f>
         <v/>
       </c>
-      <c r="H19" s="17">
+      <c r="H19" s="14">
         <f>G48</f>
         <v/>
       </c>
-      <c r="I19" s="17">
+      <c r="I19" s="14">
         <f>H48</f>
         <v/>
       </c>
-      <c r="J19" s="17">
+      <c r="J19" s="14">
         <f>I48</f>
         <v/>
       </c>
-      <c r="K19" s="17">
+      <c r="K19" s="14">
         <f>J48</f>
         <v/>
       </c>
-      <c r="L19" s="17">
+      <c r="L19" s="14">
         <f>K48</f>
         <v/>
       </c>
-      <c r="M19" s="17">
+      <c r="M19" s="14">
         <f>L48</f>
         <v/>
       </c>
-      <c r="N19" s="17">
+      <c r="N19" s="14">
         <f>M48</f>
         <v/>
       </c>
-      <c r="O19" s="17">
+      <c r="O19" s="14">
         <f>N48</f>
         <v/>
       </c>
-      <c r="P19" s="17">
+      <c r="P19" s="14">
         <f>O48</f>
         <v/>
       </c>
-      <c r="Q19" s="17">
+      <c r="Q19" s="14">
         <f>P48</f>
         <v/>
       </c>
-      <c r="R19" s="17">
+      <c r="R19" s="14">
         <f>Q48</f>
         <v/>
       </c>
-      <c r="S19" s="17">
+      <c r="S19" s="14">
         <f>R48</f>
         <v/>
       </c>
-      <c r="T19" s="17">
+      <c r="T19" s="14">
         <f>S48</f>
         <v/>
       </c>
-      <c r="U19" s="17">
+      <c r="U19" s="14">
         <f>T48</f>
         <v/>
       </c>
-      <c r="V19" s="17">
+      <c r="V19" s="14">
         <f>U48</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="21" t="inlineStr">
         <is>
           <t>Gross Portfolio Yield</t>
         </is>
       </c>
-      <c r="B20" s="26" t="inlineStr">
+      <c r="B20" s="23" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C20" s="18">
+      <c r="C20" s="12">
         <f>SUMPRODUCT(C6:C10,C13:C17)</f>
         <v/>
       </c>
-      <c r="D20" s="18">
+      <c r="D20" s="12">
         <f>SUMPRODUCT(D6:D10,D13:D17)</f>
         <v/>
       </c>
-      <c r="E20" s="18">
+      <c r="E20" s="12">
         <f>SUMPRODUCT(E6:E10,E13:E17)</f>
         <v/>
       </c>
-      <c r="F20" s="18">
+      <c r="F20" s="12">
         <f>SUMPRODUCT(F6:F10,F13:F17)</f>
         <v/>
       </c>
-      <c r="G20" s="18">
+      <c r="G20" s="12">
         <f>SUMPRODUCT(G6:G10,G13:G17)</f>
         <v/>
       </c>
-      <c r="H20" s="18">
+      <c r="H20" s="12">
         <f>SUMPRODUCT(H6:H10,H13:H17)</f>
         <v/>
       </c>
-      <c r="I20" s="18">
+      <c r="I20" s="12">
         <f>SUMPRODUCT(I6:I10,I13:I17)</f>
         <v/>
       </c>
-      <c r="J20" s="18">
+      <c r="J20" s="12">
         <f>SUMPRODUCT(J6:J10,J13:J17)</f>
         <v/>
       </c>
-      <c r="K20" s="18">
+      <c r="K20" s="12">
         <f>SUMPRODUCT(K6:K10,K13:K17)</f>
         <v/>
       </c>
-      <c r="L20" s="18">
+      <c r="L20" s="12">
         <f>SUMPRODUCT(L6:L10,L13:L17)</f>
         <v/>
       </c>
-      <c r="M20" s="18">
+      <c r="M20" s="12">
         <f>SUMPRODUCT(M6:M10,M13:M17)</f>
         <v/>
       </c>
-      <c r="N20" s="18">
+      <c r="N20" s="12">
         <f>SUMPRODUCT(N6:N10,N13:N17)</f>
         <v/>
       </c>
-      <c r="O20" s="18">
+      <c r="O20" s="12">
         <f>SUMPRODUCT(O6:O10,O13:O17)</f>
         <v/>
       </c>
-      <c r="P20" s="18">
+      <c r="P20" s="12">
         <f>SUMPRODUCT(P6:P10,P13:P17)</f>
         <v/>
       </c>
-      <c r="Q20" s="18">
+      <c r="Q20" s="12">
         <f>SUMPRODUCT(Q6:Q10,Q13:Q17)</f>
         <v/>
       </c>
-      <c r="R20" s="18">
+      <c r="R20" s="12">
         <f>SUMPRODUCT(R6:R10,R13:R17)</f>
         <v/>
       </c>
-      <c r="S20" s="18">
+      <c r="S20" s="12">
         <f>SUMPRODUCT(S6:S10,S13:S17)</f>
         <v/>
       </c>
-      <c r="T20" s="18">
+      <c r="T20" s="12">
         <f>SUMPRODUCT(T6:T10,T13:T17)</f>
         <v/>
       </c>
-      <c r="U20" s="18">
+      <c r="U20" s="12">
         <f>SUMPRODUCT(U6:U10,U13:U17)</f>
         <v/>
       </c>
-      <c r="V20" s="18">
+      <c r="V20" s="12">
         <f>SUMPRODUCT(V6:V10,V13:V17)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="23" t="inlineStr">
+      <c r="A22" s="9" t="inlineStr">
         <is>
           <t>Income by Asset Class</t>
         </is>
       </c>
-      <c r="B22" s="21" t="inlineStr">
+      <c r="B22" s="10" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="C22" s="21" t="n"/>
-      <c r="D22" s="21" t="n"/>
-      <c r="E22" s="21" t="n"/>
-      <c r="F22" s="21" t="n"/>
-      <c r="G22" s="21" t="n"/>
-      <c r="H22" s="21" t="n"/>
-      <c r="I22" s="21" t="n"/>
-      <c r="J22" s="21" t="n"/>
-      <c r="K22" s="21" t="n"/>
-      <c r="L22" s="21" t="n"/>
-      <c r="M22" s="21" t="n"/>
-      <c r="N22" s="21" t="n"/>
-      <c r="O22" s="21" t="n"/>
-      <c r="P22" s="21" t="n"/>
-      <c r="Q22" s="21" t="n"/>
-      <c r="R22" s="21" t="n"/>
-      <c r="S22" s="21" t="n"/>
-      <c r="T22" s="21" t="n"/>
-      <c r="U22" s="21" t="n"/>
-      <c r="V22" s="21" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="10" t="n"/>
+      <c r="H22" s="10" t="n"/>
+      <c r="I22" s="10" t="n"/>
+      <c r="J22" s="10" t="n"/>
+      <c r="K22" s="10" t="n"/>
+      <c r="L22" s="10" t="n"/>
+      <c r="M22" s="10" t="n"/>
+      <c r="N22" s="10" t="n"/>
+      <c r="O22" s="10" t="n"/>
+      <c r="P22" s="10" t="n"/>
+      <c r="Q22" s="10" t="n"/>
+      <c r="R22" s="10" t="n"/>
+      <c r="S22" s="10" t="n"/>
+      <c r="T22" s="10" t="n"/>
+      <c r="U22" s="10" t="n"/>
+      <c r="V22" s="10" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="24" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>LIHTC Loans</t>
         </is>
       </c>
-      <c r="B23" s="14" t="n"/>
-      <c r="C23" s="15">
+      <c r="B23" s="19" t="n"/>
+      <c r="C23" s="24">
         <f>C19*C6*C13</f>
         <v/>
       </c>
-      <c r="D23" s="15">
+      <c r="D23" s="24">
         <f>D19*D6*D13</f>
         <v/>
       </c>
-      <c r="E23" s="15">
+      <c r="E23" s="24">
         <f>E19*E6*E13</f>
         <v/>
       </c>
-      <c r="F23" s="15">
+      <c r="F23" s="24">
         <f>F19*F6*F13</f>
         <v/>
       </c>
-      <c r="G23" s="15">
+      <c r="G23" s="24">
         <f>G19*G6*G13</f>
         <v/>
       </c>
-      <c r="H23" s="15">
+      <c r="H23" s="24">
         <f>H19*H6*H13</f>
         <v/>
       </c>
-      <c r="I23" s="15">
+      <c r="I23" s="24">
         <f>I19*I6*I13</f>
         <v/>
       </c>
-      <c r="J23" s="15">
+      <c r="J23" s="24">
         <f>J19*J6*J13</f>
         <v/>
       </c>
-      <c r="K23" s="15">
+      <c r="K23" s="24">
         <f>K19*K6*K13</f>
         <v/>
       </c>
-      <c r="L23" s="15">
+      <c r="L23" s="24">
         <f>L19*L6*L13</f>
         <v/>
       </c>
-      <c r="M23" s="15">
+      <c r="M23" s="24">
         <f>M19*M6*M13</f>
         <v/>
       </c>
-      <c r="N23" s="15">
+      <c r="N23" s="24">
         <f>N19*N6*N13</f>
         <v/>
       </c>
-      <c r="O23" s="15">
+      <c r="O23" s="24">
         <f>O19*O6*O13</f>
         <v/>
       </c>
-      <c r="P23" s="15">
+      <c r="P23" s="24">
         <f>P19*P6*P13</f>
         <v/>
       </c>
-      <c r="Q23" s="15">
+      <c r="Q23" s="24">
         <f>Q19*Q6*Q13</f>
         <v/>
       </c>
-      <c r="R23" s="15">
+      <c r="R23" s="24">
         <f>R19*R6*R13</f>
         <v/>
       </c>
-      <c r="S23" s="15">
+      <c r="S23" s="24">
         <f>S19*S6*S13</f>
         <v/>
       </c>
-      <c r="T23" s="15">
+      <c r="T23" s="24">
         <f>T19*T6*T13</f>
         <v/>
       </c>
-      <c r="U23" s="15">
+      <c r="U23" s="24">
         <f>U19*U6*U13</f>
         <v/>
       </c>
-      <c r="V23" s="15">
+      <c r="V23" s="24">
         <f>V19*V6*V13</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="24" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>Municipal Bonds</t>
         </is>
       </c>
-      <c r="B24" s="14" t="n"/>
-      <c r="C24" s="15">
+      <c r="B24" s="19" t="n"/>
+      <c r="C24" s="24">
         <f>C19*C7*C14</f>
         <v/>
       </c>
-      <c r="D24" s="15">
+      <c r="D24" s="24">
         <f>D19*D7*D14</f>
         <v/>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="24">
         <f>E19*E7*E14</f>
         <v/>
       </c>
-      <c r="F24" s="15">
+      <c r="F24" s="24">
         <f>F19*F7*F14</f>
         <v/>
       </c>
-      <c r="G24" s="15">
+      <c r="G24" s="24">
         <f>G19*G7*G14</f>
         <v/>
       </c>
-      <c r="H24" s="15">
+      <c r="H24" s="24">
         <f>H19*H7*H14</f>
         <v/>
       </c>
-      <c r="I24" s="15">
+      <c r="I24" s="24">
         <f>I19*I7*I14</f>
         <v/>
       </c>
-      <c r="J24" s="15">
+      <c r="J24" s="24">
         <f>J19*J7*J14</f>
         <v/>
       </c>
-      <c r="K24" s="15">
+      <c r="K24" s="24">
         <f>K19*K7*K14</f>
         <v/>
       </c>
-      <c r="L24" s="15">
+      <c r="L24" s="24">
         <f>L19*L7*L14</f>
         <v/>
       </c>
-      <c r="M24" s="15">
+      <c r="M24" s="24">
         <f>M19*M7*M14</f>
         <v/>
       </c>
-      <c r="N24" s="15">
+      <c r="N24" s="24">
         <f>N19*N7*N14</f>
         <v/>
       </c>
-      <c r="O24" s="15">
+      <c r="O24" s="24">
         <f>O19*O7*O14</f>
         <v/>
       </c>
-      <c r="P24" s="15">
+      <c r="P24" s="24">
         <f>P19*P7*P14</f>
         <v/>
       </c>
-      <c r="Q24" s="15">
+      <c r="Q24" s="24">
         <f>Q19*Q7*Q14</f>
         <v/>
       </c>
-      <c r="R24" s="15">
+      <c r="R24" s="24">
         <f>R19*R7*R14</f>
         <v/>
       </c>
-      <c r="S24" s="15">
+      <c r="S24" s="24">
         <f>S19*S7*S14</f>
         <v/>
       </c>
-      <c r="T24" s="15">
+      <c r="T24" s="24">
         <f>T19*T7*T14</f>
         <v/>
       </c>
-      <c r="U24" s="15">
+      <c r="U24" s="24">
         <f>U19*U7*U14</f>
         <v/>
       </c>
-      <c r="V24" s="15">
+      <c r="V24" s="24">
         <f>V19*V7*V14</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="24" t="inlineStr">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>JVs</t>
         </is>
       </c>
-      <c r="B25" s="14" t="n"/>
-      <c r="C25" s="15">
+      <c r="B25" s="19" t="n"/>
+      <c r="C25" s="24">
         <f>C19*C8*C15</f>
         <v/>
       </c>
-      <c r="D25" s="15">
+      <c r="D25" s="24">
         <f>D19*D8*D15</f>
         <v/>
       </c>
-      <c r="E25" s="15">
+      <c r="E25" s="24">
         <f>E19*E8*E15</f>
         <v/>
       </c>
-      <c r="F25" s="15">
+      <c r="F25" s="24">
         <f>F19*F8*F15</f>
         <v/>
       </c>
-      <c r="G25" s="15">
+      <c r="G25" s="24">
         <f>G19*G8*G15</f>
         <v/>
       </c>
-      <c r="H25" s="15">
+      <c r="H25" s="24">
         <f>H19*H8*H15</f>
         <v/>
       </c>
-      <c r="I25" s="15">
+      <c r="I25" s="24">
         <f>I19*I8*I15</f>
         <v/>
       </c>
-      <c r="J25" s="15">
+      <c r="J25" s="24">
         <f>J19*J8*J15</f>
         <v/>
       </c>
-      <c r="K25" s="15">
+      <c r="K25" s="24">
         <f>K19*K8*K15</f>
         <v/>
       </c>
-      <c r="L25" s="15">
+      <c r="L25" s="24">
         <f>L19*L8*L15</f>
         <v/>
       </c>
-      <c r="M25" s="15">
+      <c r="M25" s="24">
         <f>M19*M8*M15</f>
         <v/>
       </c>
-      <c r="N25" s="15">
+      <c r="N25" s="24">
         <f>N19*N8*N15</f>
         <v/>
       </c>
-      <c r="O25" s="15">
+      <c r="O25" s="24">
         <f>O19*O8*O15</f>
         <v/>
       </c>
-      <c r="P25" s="15">
+      <c r="P25" s="24">
         <f>P19*P8*P15</f>
         <v/>
       </c>
-      <c r="Q25" s="15">
+      <c r="Q25" s="24">
         <f>Q19*Q8*Q15</f>
         <v/>
       </c>
-      <c r="R25" s="15">
+      <c r="R25" s="24">
         <f>R19*R8*R15</f>
         <v/>
       </c>
-      <c r="S25" s="15">
+      <c r="S25" s="24">
         <f>S19*S8*S15</f>
         <v/>
       </c>
-      <c r="T25" s="15">
+      <c r="T25" s="24">
         <f>T19*T8*T15</f>
         <v/>
       </c>
-      <c r="U25" s="15">
+      <c r="U25" s="24">
         <f>U19*U8*U15</f>
         <v/>
       </c>
-      <c r="V25" s="15">
+      <c r="V25" s="24">
         <f>V19*V8*V15</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="24" t="inlineStr">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>Securitization Residuals (B-Pieces)</t>
         </is>
       </c>
-      <c r="B26" s="14" t="n"/>
-      <c r="C26" s="15">
+      <c r="B26" s="19" t="n"/>
+      <c r="C26" s="24">
         <f>C19*C9*C16</f>
         <v/>
       </c>
-      <c r="D26" s="15">
+      <c r="D26" s="24">
         <f>D19*D9*D16</f>
         <v/>
       </c>
-      <c r="E26" s="15">
+      <c r="E26" s="24">
         <f>E19*E9*E16</f>
         <v/>
       </c>
-      <c r="F26" s="15">
+      <c r="F26" s="24">
         <f>F19*F9*F16</f>
         <v/>
       </c>
-      <c r="G26" s="15">
+      <c r="G26" s="24">
         <f>G19*G9*G16</f>
         <v/>
       </c>
-      <c r="H26" s="15">
+      <c r="H26" s="24">
         <f>H19*H9*H16</f>
         <v/>
       </c>
-      <c r="I26" s="15">
+      <c r="I26" s="24">
         <f>I19*I9*I16</f>
         <v/>
       </c>
-      <c r="J26" s="15">
+      <c r="J26" s="24">
         <f>J19*J9*J16</f>
         <v/>
       </c>
-      <c r="K26" s="15">
+      <c r="K26" s="24">
         <f>K19*K9*K16</f>
         <v/>
       </c>
-      <c r="L26" s="15">
+      <c r="L26" s="24">
         <f>L19*L9*L16</f>
         <v/>
       </c>
-      <c r="M26" s="15">
+      <c r="M26" s="24">
         <f>M19*M9*M16</f>
         <v/>
       </c>
-      <c r="N26" s="15">
+      <c r="N26" s="24">
         <f>N19*N9*N16</f>
         <v/>
       </c>
-      <c r="O26" s="15">
+      <c r="O26" s="24">
         <f>O19*O9*O16</f>
         <v/>
       </c>
-      <c r="P26" s="15">
+      <c r="P26" s="24">
         <f>P19*P9*P16</f>
         <v/>
       </c>
-      <c r="Q26" s="15">
+      <c r="Q26" s="24">
         <f>Q19*Q9*Q16</f>
         <v/>
       </c>
-      <c r="R26" s="15">
+      <c r="R26" s="24">
         <f>R19*R9*R16</f>
         <v/>
       </c>
-      <c r="S26" s="15">
+      <c r="S26" s="24">
         <f>S19*S9*S16</f>
         <v/>
       </c>
-      <c r="T26" s="15">
+      <c r="T26" s="24">
         <f>T19*T9*T16</f>
         <v/>
       </c>
-      <c r="U26" s="15">
+      <c r="U26" s="24">
         <f>U19*U9*U16</f>
         <v/>
       </c>
-      <c r="V26" s="15">
+      <c r="V26" s="24">
         <f>V19*V9*V16</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="24" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="B27" s="14" t="n"/>
-      <c r="C27" s="15">
+      <c r="B27" s="19" t="n"/>
+      <c r="C27" s="24">
         <f>C19*C10*C17</f>
         <v/>
       </c>
-      <c r="D27" s="15">
+      <c r="D27" s="24">
         <f>D19*D10*D17</f>
         <v/>
       </c>
-      <c r="E27" s="15">
+      <c r="E27" s="24">
         <f>E19*E10*E17</f>
         <v/>
       </c>
-      <c r="F27" s="15">
+      <c r="F27" s="24">
         <f>F19*F10*F17</f>
         <v/>
       </c>
-      <c r="G27" s="15">
+      <c r="G27" s="24">
         <f>G19*G10*G17</f>
         <v/>
       </c>
-      <c r="H27" s="15">
+      <c r="H27" s="24">
         <f>H19*H10*H17</f>
         <v/>
       </c>
-      <c r="I27" s="15">
+      <c r="I27" s="24">
         <f>I19*I10*I17</f>
         <v/>
       </c>
-      <c r="J27" s="15">
+      <c r="J27" s="24">
         <f>J19*J10*J17</f>
         <v/>
       </c>
-      <c r="K27" s="15">
+      <c r="K27" s="24">
         <f>K19*K10*K17</f>
         <v/>
       </c>
-      <c r="L27" s="15">
+      <c r="L27" s="24">
         <f>L19*L10*L17</f>
         <v/>
       </c>
-      <c r="M27" s="15">
+      <c r="M27" s="24">
         <f>M19*M10*M17</f>
         <v/>
       </c>
-      <c r="N27" s="15">
+      <c r="N27" s="24">
         <f>N19*N10*N17</f>
         <v/>
       </c>
-      <c r="O27" s="15">
+      <c r="O27" s="24">
         <f>O19*O10*O17</f>
         <v/>
       </c>
-      <c r="P27" s="15">
+      <c r="P27" s="24">
         <f>P19*P10*P17</f>
         <v/>
       </c>
-      <c r="Q27" s="15">
+      <c r="Q27" s="24">
         <f>Q19*Q10*Q17</f>
         <v/>
       </c>
-      <c r="R27" s="15">
+      <c r="R27" s="24">
         <f>R19*R10*R17</f>
         <v/>
       </c>
-      <c r="S27" s="15">
+      <c r="S27" s="24">
         <f>S19*S10*S17</f>
         <v/>
       </c>
-      <c r="T27" s="15">
+      <c r="T27" s="24">
         <f>T19*T10*T17</f>
         <v/>
       </c>
-      <c r="U27" s="15">
+      <c r="U27" s="24">
         <f>U19*U10*U17</f>
         <v/>
       </c>
-      <c r="V27" s="15">
+      <c r="V27" s="24">
         <f>V19*V10*V17</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="21" t="inlineStr">
         <is>
           <t>Total Asset Income</t>
         </is>
       </c>
-      <c r="B28" s="14" t="n"/>
-      <c r="C28" s="27">
+      <c r="B28" s="19" t="n"/>
+      <c r="C28" s="25">
         <f>SUM(C23:C27)</f>
         <v/>
       </c>
-      <c r="D28" s="27">
+      <c r="D28" s="25">
         <f>SUM(D23:D27)</f>
         <v/>
       </c>
-      <c r="E28" s="27">
+      <c r="E28" s="25">
         <f>SUM(E23:E27)</f>
         <v/>
       </c>
-      <c r="F28" s="27">
+      <c r="F28" s="25">
         <f>SUM(F23:F27)</f>
         <v/>
       </c>
-      <c r="G28" s="27">
+      <c r="G28" s="25">
         <f>SUM(G23:G27)</f>
         <v/>
       </c>
-      <c r="H28" s="27">
+      <c r="H28" s="25">
         <f>SUM(H23:H27)</f>
         <v/>
       </c>
-      <c r="I28" s="27">
+      <c r="I28" s="25">
         <f>SUM(I23:I27)</f>
         <v/>
       </c>
-      <c r="J28" s="27">
+      <c r="J28" s="25">
         <f>SUM(J23:J27)</f>
         <v/>
       </c>
-      <c r="K28" s="27">
+      <c r="K28" s="25">
         <f>SUM(K23:K27)</f>
         <v/>
       </c>
-      <c r="L28" s="27">
+      <c r="L28" s="25">
         <f>SUM(L23:L27)</f>
         <v/>
       </c>
-      <c r="M28" s="27">
+      <c r="M28" s="25">
         <f>SUM(M23:M27)</f>
         <v/>
       </c>
-      <c r="N28" s="27">
+      <c r="N28" s="25">
         <f>SUM(N23:N27)</f>
         <v/>
       </c>
-      <c r="O28" s="27">
+      <c r="O28" s="25">
         <f>SUM(O23:O27)</f>
         <v/>
       </c>
-      <c r="P28" s="27">
+      <c r="P28" s="25">
         <f>SUM(P23:P27)</f>
         <v/>
       </c>
-      <c r="Q28" s="27">
+      <c r="Q28" s="25">
         <f>SUM(Q23:Q27)</f>
         <v/>
       </c>
-      <c r="R28" s="27">
+      <c r="R28" s="25">
         <f>SUM(R23:R27)</f>
         <v/>
       </c>
-      <c r="S28" s="27">
+      <c r="S28" s="25">
         <f>SUM(S23:S27)</f>
         <v/>
       </c>
-      <c r="T28" s="27">
+      <c r="T28" s="25">
         <f>SUM(T23:T27)</f>
         <v/>
       </c>
-      <c r="U28" s="27">
+      <c r="U28" s="25">
         <f>SUM(U23:U27)</f>
         <v/>
       </c>
-      <c r="V28" s="27">
+      <c r="V28" s="25">
         <f>SUM(V23:V27)</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="23" t="inlineStr">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>Leverage</t>
         </is>
       </c>
-      <c r="B30" s="21" t="inlineStr">
+      <c r="B30" s="10" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="C30" s="21" t="n"/>
-      <c r="D30" s="21" t="n"/>
-      <c r="E30" s="21" t="n"/>
-      <c r="F30" s="21" t="n"/>
-      <c r="G30" s="21" t="n"/>
-      <c r="H30" s="21" t="n"/>
-      <c r="I30" s="21" t="n"/>
-      <c r="J30" s="21" t="n"/>
-      <c r="K30" s="21" t="n"/>
-      <c r="L30" s="21" t="n"/>
-      <c r="M30" s="21" t="n"/>
-      <c r="N30" s="21" t="n"/>
-      <c r="O30" s="21" t="n"/>
-      <c r="P30" s="21" t="n"/>
-      <c r="Q30" s="21" t="n"/>
-      <c r="R30" s="21" t="n"/>
-      <c r="S30" s="21" t="n"/>
-      <c r="T30" s="21" t="n"/>
-      <c r="U30" s="21" t="n"/>
-      <c r="V30" s="21" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="10" t="n"/>
+      <c r="G30" s="10" t="n"/>
+      <c r="H30" s="10" t="n"/>
+      <c r="I30" s="10" t="n"/>
+      <c r="J30" s="10" t="n"/>
+      <c r="K30" s="10" t="n"/>
+      <c r="L30" s="10" t="n"/>
+      <c r="M30" s="10" t="n"/>
+      <c r="N30" s="10" t="n"/>
+      <c r="O30" s="10" t="n"/>
+      <c r="P30" s="10" t="n"/>
+      <c r="Q30" s="10" t="n"/>
+      <c r="R30" s="10" t="n"/>
+      <c r="S30" s="10" t="n"/>
+      <c r="T30" s="10" t="n"/>
+      <c r="U30" s="10" t="n"/>
+      <c r="V30" s="10" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="24" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>Leveraged AUM</t>
         </is>
       </c>
-      <c r="B31" s="14" t="n"/>
-      <c r="C31" s="15">
+      <c r="B31" s="19" t="n"/>
+      <c r="C31" s="24">
         <f>C19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="D31" s="15">
+      <c r="D31" s="24">
         <f>D19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="E31" s="15">
+      <c r="E31" s="24">
         <f>E19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="F31" s="15">
+      <c r="F31" s="24">
         <f>F19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="G31" s="15">
+      <c r="G31" s="24">
         <f>G19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="H31" s="15">
+      <c r="H31" s="24">
         <f>H19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="I31" s="15">
+      <c r="I31" s="24">
         <f>I19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="J31" s="15">
+      <c r="J31" s="24">
         <f>J19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="K31" s="15">
+      <c r="K31" s="24">
         <f>K19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="L31" s="15">
+      <c r="L31" s="24">
         <f>L19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="M31" s="15">
+      <c r="M31" s="24">
         <f>M19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="N31" s="15">
+      <c r="N31" s="24">
         <f>N19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="O31" s="15">
+      <c r="O31" s="24">
         <f>O19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="P31" s="15">
+      <c r="P31" s="24">
         <f>P19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="Q31" s="15">
+      <c r="Q31" s="24">
         <f>Q19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="R31" s="15">
+      <c r="R31" s="24">
         <f>R19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="S31" s="15">
+      <c r="S31" s="24">
         <f>S19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="T31" s="15">
+      <c r="T31" s="24">
         <f>T19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="U31" s="15">
+      <c r="U31" s="24">
         <f>U19*Summary!$C$10</f>
         <v/>
       </c>
-      <c r="V31" s="15">
+      <c r="V31" s="24">
         <f>V19*Summary!$C$10</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="24" t="inlineStr">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>Leveraged Income</t>
         </is>
       </c>
-      <c r="B32" s="14" t="n"/>
-      <c r="C32" s="15">
+      <c r="B32" s="19" t="n"/>
+      <c r="C32" s="24">
         <f>C31*C20</f>
         <v/>
       </c>
-      <c r="D32" s="15">
+      <c r="D32" s="24">
         <f>D31*D20</f>
         <v/>
       </c>
-      <c r="E32" s="15">
+      <c r="E32" s="24">
         <f>E31*E20</f>
         <v/>
       </c>
-      <c r="F32" s="15">
+      <c r="F32" s="24">
         <f>F31*F20</f>
         <v/>
       </c>
-      <c r="G32" s="15">
+      <c r="G32" s="24">
         <f>G31*G20</f>
         <v/>
       </c>
-      <c r="H32" s="15">
+      <c r="H32" s="24">
         <f>H31*H20</f>
         <v/>
       </c>
-      <c r="I32" s="15">
+      <c r="I32" s="24">
         <f>I31*I20</f>
         <v/>
       </c>
-      <c r="J32" s="15">
+      <c r="J32" s="24">
         <f>J31*J20</f>
         <v/>
       </c>
-      <c r="K32" s="15">
+      <c r="K32" s="24">
         <f>K31*K20</f>
         <v/>
       </c>
-      <c r="L32" s="15">
+      <c r="L32" s="24">
         <f>L31*L20</f>
         <v/>
       </c>
-      <c r="M32" s="15">
+      <c r="M32" s="24">
         <f>M31*M20</f>
         <v/>
       </c>
-      <c r="N32" s="15">
+      <c r="N32" s="24">
         <f>N31*N20</f>
         <v/>
       </c>
-      <c r="O32" s="15">
+      <c r="O32" s="24">
         <f>O31*O20</f>
         <v/>
       </c>
-      <c r="P32" s="15">
+      <c r="P32" s="24">
         <f>P31*P20</f>
         <v/>
       </c>
-      <c r="Q32" s="15">
+      <c r="Q32" s="24">
         <f>Q31*Q20</f>
         <v/>
       </c>
-      <c r="R32" s="15">
+      <c r="R32" s="24">
         <f>R31*R20</f>
         <v/>
       </c>
-      <c r="S32" s="15">
+      <c r="S32" s="24">
         <f>S31*S20</f>
         <v/>
       </c>
-      <c r="T32" s="15">
+      <c r="T32" s="24">
         <f>T31*T20</f>
         <v/>
       </c>
-      <c r="U32" s="15">
+      <c r="U32" s="24">
         <f>U31*U20</f>
         <v/>
       </c>
-      <c r="V32" s="15">
+      <c r="V32" s="24">
         <f>V31*V20</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="24" t="inlineStr">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>Leverage Cost</t>
         </is>
       </c>
-      <c r="B33" s="14" t="n"/>
-      <c r="C33" s="15">
+      <c r="B33" s="19" t="n"/>
+      <c r="C33" s="24">
         <f>C31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="D33" s="15">
+      <c r="D33" s="24">
         <f>D31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="E33" s="15">
+      <c r="E33" s="24">
         <f>E31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="F33" s="15">
+      <c r="F33" s="24">
         <f>F31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="G33" s="15">
+      <c r="G33" s="24">
         <f>G31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="H33" s="15">
+      <c r="H33" s="24">
         <f>H31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="I33" s="15">
+      <c r="I33" s="24">
         <f>I31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="J33" s="15">
+      <c r="J33" s="24">
         <f>J31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="K33" s="15">
+      <c r="K33" s="24">
         <f>K31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="L33" s="15">
+      <c r="L33" s="24">
         <f>L31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="M33" s="15">
+      <c r="M33" s="24">
         <f>M31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="N33" s="15">
+      <c r="N33" s="24">
         <f>N31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="O33" s="15">
+      <c r="O33" s="24">
         <f>O31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="P33" s="15">
+      <c r="P33" s="24">
         <f>P31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="Q33" s="15">
+      <c r="Q33" s="24">
         <f>Q31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="R33" s="15">
+      <c r="R33" s="24">
         <f>R31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="S33" s="15">
+      <c r="S33" s="24">
         <f>S31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="T33" s="15">
+      <c r="T33" s="24">
         <f>T31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="U33" s="15">
+      <c r="U33" s="24">
         <f>U31*Summary!$C$11/10000</f>
         <v/>
       </c>
-      <c r="V33" s="15">
+      <c r="V33" s="24">
         <f>V31*Summary!$C$11/10000</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
+      <c r="A34" s="21" t="inlineStr">
         <is>
           <t>Net Leverage Income</t>
         </is>
       </c>
-      <c r="B34" s="14" t="n"/>
-      <c r="C34" s="27">
+      <c r="B34" s="19" t="n"/>
+      <c r="C34" s="25">
         <f>C32-C33</f>
         <v/>
       </c>
-      <c r="D34" s="27">
+      <c r="D34" s="25">
         <f>D32-D33</f>
         <v/>
       </c>
-      <c r="E34" s="27">
+      <c r="E34" s="25">
         <f>E32-E33</f>
         <v/>
       </c>
-      <c r="F34" s="27">
+      <c r="F34" s="25">
         <f>F32-F33</f>
         <v/>
       </c>
-      <c r="G34" s="27">
+      <c r="G34" s="25">
         <f>G32-G33</f>
         <v/>
       </c>
-      <c r="H34" s="27">
+      <c r="H34" s="25">
         <f>H32-H33</f>
         <v/>
       </c>
-      <c r="I34" s="27">
+      <c r="I34" s="25">
         <f>I32-I33</f>
         <v/>
       </c>
-      <c r="J34" s="27">
+      <c r="J34" s="25">
         <f>J32-J33</f>
         <v/>
       </c>
-      <c r="K34" s="27">
+      <c r="K34" s="25">
         <f>K32-K33</f>
         <v/>
       </c>
-      <c r="L34" s="27">
+      <c r="L34" s="25">
         <f>L32-L33</f>
         <v/>
       </c>
-      <c r="M34" s="27">
+      <c r="M34" s="25">
         <f>M32-M33</f>
         <v/>
       </c>
-      <c r="N34" s="27">
+      <c r="N34" s="25">
         <f>N32-N33</f>
         <v/>
       </c>
-      <c r="O34" s="27">
+      <c r="O34" s="25">
         <f>O32-O33</f>
         <v/>
       </c>
-      <c r="P34" s="27">
+      <c r="P34" s="25">
         <f>P32-P33</f>
         <v/>
       </c>
-      <c r="Q34" s="27">
+      <c r="Q34" s="25">
         <f>Q32-Q33</f>
         <v/>
       </c>
-      <c r="R34" s="27">
+      <c r="R34" s="25">
         <f>R32-R33</f>
         <v/>
       </c>
-      <c r="S34" s="27">
+      <c r="S34" s="25">
         <f>S32-S33</f>
         <v/>
       </c>
-      <c r="T34" s="27">
+      <c r="T34" s="25">
         <f>T32-T33</f>
         <v/>
       </c>
-      <c r="U34" s="27">
+      <c r="U34" s="25">
         <f>U32-U33</f>
         <v/>
       </c>
-      <c r="V34" s="27">
+      <c r="V34" s="25">
         <f>V32-V33</f>
         <v/>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="28" t="inlineStr">
+      <c r="A36" s="26" t="inlineStr">
         <is>
           <t>TOTAL GROSS INCOME</t>
         </is>
       </c>
-      <c r="B36" s="29" t="n"/>
-      <c r="C36" s="30">
+      <c r="B36" s="27" t="n"/>
+      <c r="C36" s="28">
         <f>C28+C34</f>
         <v/>
       </c>
-      <c r="D36" s="30">
+      <c r="D36" s="28">
         <f>D28+D34</f>
         <v/>
       </c>
-      <c r="E36" s="30">
+      <c r="E36" s="28">
         <f>E28+E34</f>
         <v/>
       </c>
-      <c r="F36" s="30">
+      <c r="F36" s="28">
         <f>F28+F34</f>
         <v/>
       </c>
-      <c r="G36" s="30">
+      <c r="G36" s="28">
         <f>G28+G34</f>
         <v/>
       </c>
-      <c r="H36" s="30">
+      <c r="H36" s="28">
         <f>H28+H34</f>
         <v/>
       </c>
-      <c r="I36" s="30">
+      <c r="I36" s="28">
         <f>I28+I34</f>
         <v/>
       </c>
-      <c r="J36" s="30">
+      <c r="J36" s="28">
         <f>J28+J34</f>
         <v/>
       </c>
-      <c r="K36" s="30">
+      <c r="K36" s="28">
         <f>K28+K34</f>
         <v/>
       </c>
-      <c r="L36" s="30">
+      <c r="L36" s="28">
         <f>L28+L34</f>
         <v/>
       </c>
-      <c r="M36" s="30">
+      <c r="M36" s="28">
         <f>M28+M34</f>
         <v/>
       </c>
-      <c r="N36" s="30">
+      <c r="N36" s="28">
         <f>N28+N34</f>
         <v/>
       </c>
-      <c r="O36" s="30">
+      <c r="O36" s="28">
         <f>O28+O34</f>
         <v/>
       </c>
-      <c r="P36" s="30">
+      <c r="P36" s="28">
         <f>P28+P34</f>
         <v/>
       </c>
-      <c r="Q36" s="30">
+      <c r="Q36" s="28">
         <f>Q28+Q34</f>
         <v/>
       </c>
-      <c r="R36" s="30">
+      <c r="R36" s="28">
         <f>R28+R34</f>
         <v/>
       </c>
-      <c r="S36" s="30">
+      <c r="S36" s="28">
         <f>S28+S34</f>
         <v/>
       </c>
-      <c r="T36" s="30">
+      <c r="T36" s="28">
         <f>T28+T34</f>
         <v/>
       </c>
-      <c r="U36" s="30">
+      <c r="U36" s="28">
         <f>U28+U34</f>
         <v/>
       </c>
-      <c r="V36" s="30">
+      <c r="V36" s="28">
         <f>V28+V34</f>
         <v/>
       </c>
@@ -3913,441 +3475,441 @@
       <c r="V38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="24" t="inlineStr">
+      <c r="A39" s="11" t="inlineStr">
         <is>
           <t>Management Fee</t>
         </is>
       </c>
-      <c r="B39" s="14" t="n"/>
-      <c r="C39" s="15">
+      <c r="B39" s="19" t="n"/>
+      <c r="C39" s="24">
         <f>C19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="D39" s="15">
+      <c r="D39" s="24">
         <f>D19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="E39" s="15">
+      <c r="E39" s="24">
         <f>E19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="F39" s="15">
+      <c r="F39" s="24">
         <f>F19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="G39" s="15">
+      <c r="G39" s="24">
         <f>G19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="H39" s="15">
+      <c r="H39" s="24">
         <f>H19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="I39" s="15">
+      <c r="I39" s="24">
         <f>I19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="J39" s="15">
+      <c r="J39" s="24">
         <f>J19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="K39" s="15">
+      <c r="K39" s="24">
         <f>K19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="L39" s="15">
+      <c r="L39" s="24">
         <f>L19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="M39" s="15">
+      <c r="M39" s="24">
         <f>M19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="N39" s="15">
+      <c r="N39" s="24">
         <f>N19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="O39" s="15">
+      <c r="O39" s="24">
         <f>O19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="P39" s="15">
+      <c r="P39" s="24">
         <f>P19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="Q39" s="15">
+      <c r="Q39" s="24">
         <f>Q19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="R39" s="15">
+      <c r="R39" s="24">
         <f>R19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="S39" s="15">
+      <c r="S39" s="24">
         <f>S19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="T39" s="15">
+      <c r="T39" s="24">
         <f>T19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="U39" s="15">
+      <c r="U39" s="24">
         <f>U19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="V39" s="15">
+      <c r="V39" s="24">
         <f>V19*Summary!$C$6/10000</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="24" t="inlineStr">
+      <c r="A40" s="11" t="inlineStr">
         <is>
           <t>Return Above Hurdle</t>
         </is>
       </c>
-      <c r="B40" s="14" t="n"/>
-      <c r="C40" s="15">
+      <c r="B40" s="19" t="n"/>
+      <c r="C40" s="24">
         <f>MAX(0,C36-C19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="D40" s="15">
+      <c r="D40" s="24">
         <f>MAX(0,D36-D19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="E40" s="15">
+      <c r="E40" s="24">
         <f>MAX(0,E36-E19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="F40" s="15">
+      <c r="F40" s="24">
         <f>MAX(0,F36-F19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="G40" s="15">
+      <c r="G40" s="24">
         <f>MAX(0,G36-G19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="H40" s="15">
+      <c r="H40" s="24">
         <f>MAX(0,H36-H19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="I40" s="15">
+      <c r="I40" s="24">
         <f>MAX(0,I36-I19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="J40" s="15">
+      <c r="J40" s="24">
         <f>MAX(0,J36-J19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="K40" s="15">
+      <c r="K40" s="24">
         <f>MAX(0,K36-K19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="L40" s="15">
+      <c r="L40" s="24">
         <f>MAX(0,L36-L19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="M40" s="15">
+      <c r="M40" s="24">
         <f>MAX(0,M36-M19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="N40" s="15">
+      <c r="N40" s="24">
         <f>MAX(0,N36-N19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="O40" s="15">
+      <c r="O40" s="24">
         <f>MAX(0,O36-O19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="P40" s="15">
+      <c r="P40" s="24">
         <f>MAX(0,P36-P19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="Q40" s="15">
+      <c r="Q40" s="24">
         <f>MAX(0,Q36-Q19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="R40" s="15">
+      <c r="R40" s="24">
         <f>MAX(0,R36-R19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="S40" s="15">
+      <c r="S40" s="24">
         <f>MAX(0,S36-S19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="T40" s="15">
+      <c r="T40" s="24">
         <f>MAX(0,T36-T19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="U40" s="15">
+      <c r="U40" s="24">
         <f>MAX(0,U36-U19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="V40" s="15">
+      <c r="V40" s="24">
         <f>MAX(0,V36-V19*Summary!$C$8/10000)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="24" t="inlineStr">
+      <c r="A41" s="11" t="inlineStr">
         <is>
           <t>Performance Fee</t>
         </is>
       </c>
-      <c r="B41" s="14" t="n"/>
-      <c r="C41" s="15">
+      <c r="B41" s="19" t="n"/>
+      <c r="C41" s="24">
         <f>C40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="D41" s="15">
+      <c r="D41" s="24">
         <f>D40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="E41" s="15">
+      <c r="E41" s="24">
         <f>E40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="F41" s="15">
+      <c r="F41" s="24">
         <f>F40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="G41" s="15">
+      <c r="G41" s="24">
         <f>G40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="H41" s="15">
+      <c r="H41" s="24">
         <f>H40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="I41" s="15">
+      <c r="I41" s="24">
         <f>I40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="J41" s="15">
+      <c r="J41" s="24">
         <f>J40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="K41" s="15">
+      <c r="K41" s="24">
         <f>K40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="L41" s="15">
+      <c r="L41" s="24">
         <f>L40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="M41" s="15">
+      <c r="M41" s="24">
         <f>M40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="N41" s="15">
+      <c r="N41" s="24">
         <f>N40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="O41" s="15">
+      <c r="O41" s="24">
         <f>O40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="P41" s="15">
+      <c r="P41" s="24">
         <f>P40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="Q41" s="15">
+      <c r="Q41" s="24">
         <f>Q40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="R41" s="15">
+      <c r="R41" s="24">
         <f>R40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="S41" s="15">
+      <c r="S41" s="24">
         <f>S40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="T41" s="15">
+      <c r="T41" s="24">
         <f>T40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="U41" s="15">
+      <c r="U41" s="24">
         <f>U40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="V41" s="15">
+      <c r="V41" s="24">
         <f>V40*Summary!$C$7/10000</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="24" t="inlineStr">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t>Other Expenses</t>
         </is>
       </c>
-      <c r="B42" s="14" t="n"/>
-      <c r="C42" s="15">
+      <c r="B42" s="19" t="n"/>
+      <c r="C42" s="24">
         <f>C19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="D42" s="15">
+      <c r="D42" s="24">
         <f>D19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="E42" s="15">
+      <c r="E42" s="24">
         <f>E19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="F42" s="15">
+      <c r="F42" s="24">
         <f>F19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="G42" s="15">
+      <c r="G42" s="24">
         <f>G19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="H42" s="15">
+      <c r="H42" s="24">
         <f>H19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="I42" s="15">
+      <c r="I42" s="24">
         <f>I19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="J42" s="15">
+      <c r="J42" s="24">
         <f>J19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="K42" s="15">
+      <c r="K42" s="24">
         <f>K19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="L42" s="15">
+      <c r="L42" s="24">
         <f>L19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="M42" s="15">
+      <c r="M42" s="24">
         <f>M19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="N42" s="15">
+      <c r="N42" s="24">
         <f>N19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="O42" s="15">
+      <c r="O42" s="24">
         <f>O19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="P42" s="15">
+      <c r="P42" s="24">
         <f>P19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="Q42" s="15">
+      <c r="Q42" s="24">
         <f>Q19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="R42" s="15">
+      <c r="R42" s="24">
         <f>R19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="S42" s="15">
+      <c r="S42" s="24">
         <f>S19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="T42" s="15">
+      <c r="T42" s="24">
         <f>T19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="U42" s="15">
+      <c r="U42" s="24">
         <f>U19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="V42" s="15">
+      <c r="V42" s="24">
         <f>V19*Summary!$C$9/10000</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="inlineStr">
+      <c r="A43" s="21" t="inlineStr">
         <is>
           <t>Total Fees &amp; Expenses</t>
         </is>
       </c>
-      <c r="B43" s="14" t="n"/>
-      <c r="C43" s="27">
+      <c r="B43" s="19" t="n"/>
+      <c r="C43" s="25">
         <f>C39+C41+C42</f>
         <v/>
       </c>
-      <c r="D43" s="27">
+      <c r="D43" s="25">
         <f>D39+D41+D42</f>
         <v/>
       </c>
-      <c r="E43" s="27">
+      <c r="E43" s="25">
         <f>E39+E41+E42</f>
         <v/>
       </c>
-      <c r="F43" s="27">
+      <c r="F43" s="25">
         <f>F39+F41+F42</f>
         <v/>
       </c>
-      <c r="G43" s="27">
+      <c r="G43" s="25">
         <f>G39+G41+G42</f>
         <v/>
       </c>
-      <c r="H43" s="27">
+      <c r="H43" s="25">
         <f>H39+H41+H42</f>
         <v/>
       </c>
-      <c r="I43" s="27">
+      <c r="I43" s="25">
         <f>I39+I41+I42</f>
         <v/>
       </c>
-      <c r="J43" s="27">
+      <c r="J43" s="25">
         <f>J39+J41+J42</f>
         <v/>
       </c>
-      <c r="K43" s="27">
+      <c r="K43" s="25">
         <f>K39+K41+K42</f>
         <v/>
       </c>
-      <c r="L43" s="27">
+      <c r="L43" s="25">
         <f>L39+L41+L42</f>
         <v/>
       </c>
-      <c r="M43" s="27">
+      <c r="M43" s="25">
         <f>M39+M41+M42</f>
         <v/>
       </c>
-      <c r="N43" s="27">
+      <c r="N43" s="25">
         <f>N39+N41+N42</f>
         <v/>
       </c>
-      <c r="O43" s="27">
+      <c r="O43" s="25">
         <f>O39+O41+O42</f>
         <v/>
       </c>
-      <c r="P43" s="27">
+      <c r="P43" s="25">
         <f>P39+P41+P42</f>
         <v/>
       </c>
-      <c r="Q43" s="27">
+      <c r="Q43" s="25">
         <f>Q39+Q41+Q42</f>
         <v/>
       </c>
-      <c r="R43" s="27">
+      <c r="R43" s="25">
         <f>R39+R41+R42</f>
         <v/>
       </c>
-      <c r="S43" s="27">
+      <c r="S43" s="25">
         <f>S39+S41+S42</f>
         <v/>
       </c>
-      <c r="T43" s="27">
+      <c r="T43" s="25">
         <f>T39+T41+T42</f>
         <v/>
       </c>
-      <c r="U43" s="27">
+      <c r="U43" s="25">
         <f>U39+U41+U42</f>
         <v/>
       </c>
-      <c r="V43" s="27">
+      <c r="V43" s="25">
         <f>V39+V41+V42</f>
         <v/>
       </c>
@@ -4381,265 +3943,265 @@
       <c r="V45" s="3" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="31" t="inlineStr">
+      <c r="A46" s="29" t="inlineStr">
         <is>
           <t>NET INCOME</t>
         </is>
       </c>
-      <c r="B46" s="32" t="n"/>
-      <c r="C46" s="33">
+      <c r="B46" s="30" t="n"/>
+      <c r="C46" s="31">
         <f>C36-C43</f>
         <v/>
       </c>
-      <c r="D46" s="33">
+      <c r="D46" s="31">
         <f>D36-D43</f>
         <v/>
       </c>
-      <c r="E46" s="33">
+      <c r="E46" s="31">
         <f>E36-E43</f>
         <v/>
       </c>
-      <c r="F46" s="33">
+      <c r="F46" s="31">
         <f>F36-F43</f>
         <v/>
       </c>
-      <c r="G46" s="33">
+      <c r="G46" s="31">
         <f>G36-G43</f>
         <v/>
       </c>
-      <c r="H46" s="33">
+      <c r="H46" s="31">
         <f>H36-H43</f>
         <v/>
       </c>
-      <c r="I46" s="33">
+      <c r="I46" s="31">
         <f>I36-I43</f>
         <v/>
       </c>
-      <c r="J46" s="33">
+      <c r="J46" s="31">
         <f>J36-J43</f>
         <v/>
       </c>
-      <c r="K46" s="33">
+      <c r="K46" s="31">
         <f>K36-K43</f>
         <v/>
       </c>
-      <c r="L46" s="33">
+      <c r="L46" s="31">
         <f>L36-L43</f>
         <v/>
       </c>
-      <c r="M46" s="33">
+      <c r="M46" s="31">
         <f>M36-M43</f>
         <v/>
       </c>
-      <c r="N46" s="33">
+      <c r="N46" s="31">
         <f>N36-N43</f>
         <v/>
       </c>
-      <c r="O46" s="33">
+      <c r="O46" s="31">
         <f>O36-O43</f>
         <v/>
       </c>
-      <c r="P46" s="33">
+      <c r="P46" s="31">
         <f>P36-P43</f>
         <v/>
       </c>
-      <c r="Q46" s="33">
+      <c r="Q46" s="31">
         <f>Q36-Q43</f>
         <v/>
       </c>
-      <c r="R46" s="33">
+      <c r="R46" s="31">
         <f>R36-R43</f>
         <v/>
       </c>
-      <c r="S46" s="33">
+      <c r="S46" s="31">
         <f>S36-S43</f>
         <v/>
       </c>
-      <c r="T46" s="33">
+      <c r="T46" s="31">
         <f>T36-T43</f>
         <v/>
       </c>
-      <c r="U46" s="33">
+      <c r="U46" s="31">
         <f>U36-U43</f>
         <v/>
       </c>
-      <c r="V46" s="33">
+      <c r="V46" s="31">
         <f>V36-V43</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="31" t="inlineStr">
+      <c r="A47" s="29" t="inlineStr">
         <is>
           <t>NET YIELD (Return to LPs)</t>
         </is>
       </c>
-      <c r="B47" s="32" t="n"/>
-      <c r="C47" s="34">
+      <c r="B47" s="30" t="n"/>
+      <c r="C47" s="32">
         <f>IF(C19=0,0,C46/C19)</f>
         <v/>
       </c>
-      <c r="D47" s="34">
+      <c r="D47" s="32">
         <f>IF(D19=0,0,D46/D19)</f>
         <v/>
       </c>
-      <c r="E47" s="34">
+      <c r="E47" s="32">
         <f>IF(E19=0,0,E46/E19)</f>
         <v/>
       </c>
-      <c r="F47" s="34">
+      <c r="F47" s="32">
         <f>IF(F19=0,0,F46/F19)</f>
         <v/>
       </c>
-      <c r="G47" s="34">
+      <c r="G47" s="32">
         <f>IF(G19=0,0,G46/G19)</f>
         <v/>
       </c>
-      <c r="H47" s="34">
+      <c r="H47" s="32">
         <f>IF(H19=0,0,H46/H19)</f>
         <v/>
       </c>
-      <c r="I47" s="34">
+      <c r="I47" s="32">
         <f>IF(I19=0,0,I46/I19)</f>
         <v/>
       </c>
-      <c r="J47" s="34">
+      <c r="J47" s="32">
         <f>IF(J19=0,0,J46/J19)</f>
         <v/>
       </c>
-      <c r="K47" s="34">
+      <c r="K47" s="32">
         <f>IF(K19=0,0,K46/K19)</f>
         <v/>
       </c>
-      <c r="L47" s="34">
+      <c r="L47" s="32">
         <f>IF(L19=0,0,L46/L19)</f>
         <v/>
       </c>
-      <c r="M47" s="34">
+      <c r="M47" s="32">
         <f>IF(M19=0,0,M46/M19)</f>
         <v/>
       </c>
-      <c r="N47" s="34">
+      <c r="N47" s="32">
         <f>IF(N19=0,0,N46/N19)</f>
         <v/>
       </c>
-      <c r="O47" s="34">
+      <c r="O47" s="32">
         <f>IF(O19=0,0,O46/O19)</f>
         <v/>
       </c>
-      <c r="P47" s="34">
+      <c r="P47" s="32">
         <f>IF(P19=0,0,P46/P19)</f>
         <v/>
       </c>
-      <c r="Q47" s="34">
+      <c r="Q47" s="32">
         <f>IF(Q19=0,0,Q46/Q19)</f>
         <v/>
       </c>
-      <c r="R47" s="34">
+      <c r="R47" s="32">
         <f>IF(R19=0,0,R46/R19)</f>
         <v/>
       </c>
-      <c r="S47" s="34">
+      <c r="S47" s="32">
         <f>IF(S19=0,0,S46/S19)</f>
         <v/>
       </c>
-      <c r="T47" s="34">
+      <c r="T47" s="32">
         <f>IF(T19=0,0,T46/T19)</f>
         <v/>
       </c>
-      <c r="U47" s="34">
+      <c r="U47" s="32">
         <f>IF(U19=0,0,U46/U19)</f>
         <v/>
       </c>
-      <c r="V47" s="34">
+      <c r="V47" s="32">
         <f>IF(V19=0,0,V46/V19)</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="35" t="inlineStr">
+      <c r="A48" s="33" t="inlineStr">
         <is>
           <t>ENDING AUM</t>
         </is>
       </c>
-      <c r="B48" s="36" t="n"/>
-      <c r="C48" s="37">
+      <c r="B48" s="34" t="n"/>
+      <c r="C48" s="35">
         <f>C19+C46</f>
         <v/>
       </c>
-      <c r="D48" s="37">
+      <c r="D48" s="35">
         <f>D19+D46</f>
         <v/>
       </c>
-      <c r="E48" s="37">
+      <c r="E48" s="35">
         <f>E19+E46</f>
         <v/>
       </c>
-      <c r="F48" s="37">
+      <c r="F48" s="35">
         <f>F19+F46</f>
         <v/>
       </c>
-      <c r="G48" s="37">
+      <c r="G48" s="35">
         <f>G19+G46</f>
         <v/>
       </c>
-      <c r="H48" s="37">
+      <c r="H48" s="35">
         <f>H19+H46</f>
         <v/>
       </c>
-      <c r="I48" s="37">
+      <c r="I48" s="35">
         <f>I19+I46</f>
         <v/>
       </c>
-      <c r="J48" s="37">
+      <c r="J48" s="35">
         <f>J19+J46</f>
         <v/>
       </c>
-      <c r="K48" s="37">
+      <c r="K48" s="35">
         <f>K19+K46</f>
         <v/>
       </c>
-      <c r="L48" s="37">
+      <c r="L48" s="35">
         <f>L19+L46</f>
         <v/>
       </c>
-      <c r="M48" s="37">
+      <c r="M48" s="35">
         <f>M19+M46</f>
         <v/>
       </c>
-      <c r="N48" s="37">
+      <c r="N48" s="35">
         <f>N19+N46</f>
         <v/>
       </c>
-      <c r="O48" s="37">
+      <c r="O48" s="35">
         <f>O19+O46</f>
         <v/>
       </c>
-      <c r="P48" s="37">
+      <c r="P48" s="35">
         <f>P19+P46</f>
         <v/>
       </c>
-      <c r="Q48" s="37">
+      <c r="Q48" s="35">
         <f>Q19+Q46</f>
         <v/>
       </c>
-      <c r="R48" s="37">
+      <c r="R48" s="35">
         <f>R19+R46</f>
         <v/>
       </c>
-      <c r="S48" s="37">
+      <c r="S48" s="35">
         <f>S19+S46</f>
         <v/>
       </c>
-      <c r="T48" s="37">
+      <c r="T48" s="35">
         <f>T19+T46</f>
         <v/>
       </c>
-      <c r="U48" s="37">
+      <c r="U48" s="35">
         <f>U19+U46</f>
         <v/>
       </c>
-      <c r="V48" s="37">
+      <c r="V48" s="35">
         <f>V19+V46</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Regenerate Excel model without leverage calcs
https://claude.ai/code/session_015HvWwNhMMyRaKrg6b48d5x
</commit_message>
<xml_diff>
--- a/LP_Financial_Model.xlsx
+++ b/LP_Financial_Model.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Annual Model" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Annual Model" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,11 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
     <numFmt numFmtId="165" formatCode="0&quot; bps&quot;"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
-    <numFmt numFmtId="167" formatCode="0.00x"/>
+    <numFmt numFmtId="166" formatCode="0.00x"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -205,7 +204,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -224,9 +223,6 @@
     <xf numFmtId="165" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -237,7 +233,7 @@
     <xf numFmtId="10" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -767,28 +763,6 @@
         <v>15</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>Leverage Percentage</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="8" t="n">
-        <v>0.25</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>Leverage Cost</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n"/>
-      <c r="C11" s="7" t="n">
-        <v>350</v>
-      </c>
-    </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
@@ -804,342 +778,330 @@
       <c r="H13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A14" s="8" t="inlineStr">
         <is>
           <t>Return Metrics</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
-      <c r="H14" s="10" t="n"/>
+      <c r="B14" s="9" t="n"/>
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="9" t="n"/>
+      <c r="F14" s="9" t="n"/>
+      <c r="G14" s="9" t="n"/>
+      <c r="H14" s="9" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>Net IRR (Avg Annual Net Yield)</t>
         </is>
       </c>
-      <c r="C15" s="12">
+      <c r="C15" s="11">
         <f>AVERAGE('Annual Model'!C47,'Annual Model'!D47,'Annual Model'!E47,'Annual Model'!F47,'Annual Model'!G47,'Annual Model'!H47,'Annual Model'!I47,'Annual Model'!J47,'Annual Model'!K47,'Annual Model'!L47,'Annual Model'!M47,'Annual Model'!N47,'Annual Model'!O47,'Annual Model'!P47,'Annual Model'!Q47,'Annual Model'!R47,'Annual Model'!S47,'Annual Model'!T47,'Annual Model'!U47,'Annual Model'!V47)</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Gross IRR (Avg Annual Gross Yield)</t>
         </is>
       </c>
-      <c r="C16" s="12">
+      <c r="C16" s="11">
         <f>AVERAGE('Annual Model'!C20,'Annual Model'!D20,'Annual Model'!E20,'Annual Model'!F20,'Annual Model'!G20,'Annual Model'!H20,'Annual Model'!I20,'Annual Model'!J20,'Annual Model'!K20,'Annual Model'!L20,'Annual Model'!M20,'Annual Model'!N20,'Annual Model'!O20,'Annual Model'!P20,'Annual Model'!Q20,'Annual Model'!R20,'Annual Model'!S20,'Annual Model'!T20,'Annual Model'!U20,'Annual Model'!V20)</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>MOIC (Multiple on Invested Capital)</t>
         </is>
       </c>
-      <c r="C17" s="13">
+      <c r="C17" s="12">
         <f>'Annual Model'!V48/Summary!$C$5</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>DPI (Distributions to Paid-In)</t>
         </is>
       </c>
-      <c r="C18" s="13">
+      <c r="C18" s="12">
         <f>('Annual Model'!C46+'Annual Model'!D46+'Annual Model'!E46+'Annual Model'!F46+'Annual Model'!G46+'Annual Model'!H46+'Annual Model'!I46+'Annual Model'!J46+'Annual Model'!K46+'Annual Model'!L46+'Annual Model'!M46+'Annual Model'!N46+'Annual Model'!O46+'Annual Model'!P46+'Annual Model'!Q46+'Annual Model'!R46+'Annual Model'!S46+'Annual Model'!T46+'Annual Model'!U46+'Annual Model'!V46)/Summary!$C$5</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>Total Value to Paid-In (TVPI)</t>
         </is>
       </c>
-      <c r="C19" s="13">
+      <c r="C19" s="12">
         <f>('Annual Model'!V48+'Annual Model'!C46+'Annual Model'!D46+'Annual Model'!E46+'Annual Model'!F46+'Annual Model'!G46+'Annual Model'!H46+'Annual Model'!I46+'Annual Model'!J46+'Annual Model'!K46+'Annual Model'!L46+'Annual Model'!M46+'Annual Model'!N46+'Annual Model'!O46+'Annual Model'!P46+'Annual Model'!Q46+'Annual Model'!R46+'Annual Model'!S46+'Annual Model'!T46+'Annual Model'!U46+'Annual Model'!V46)/Summary!$C$5</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="9" t="inlineStr">
+      <c r="A21" s="8" t="inlineStr">
         <is>
           <t>Capital Metrics</t>
         </is>
       </c>
-      <c r="B21" s="10" t="n"/>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n"/>
-      <c r="E21" s="10" t="n"/>
-      <c r="F21" s="10" t="n"/>
-      <c r="G21" s="10" t="n"/>
-      <c r="H21" s="10" t="n"/>
+      <c r="B21" s="9" t="n"/>
+      <c r="C21" s="9" t="n"/>
+      <c r="D21" s="9" t="n"/>
+      <c r="E21" s="9" t="n"/>
+      <c r="F21" s="9" t="n"/>
+      <c r="G21" s="9" t="n"/>
+      <c r="H21" s="9" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="10" t="inlineStr">
         <is>
           <t>Initial Committed Capital</t>
         </is>
       </c>
-      <c r="C22" s="14">
+      <c r="C22" s="13">
         <f>Summary!$C$5</f>
         <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Ending AUM (Year 20)</t>
         </is>
       </c>
-      <c r="C23" s="14">
+      <c r="C23" s="13">
         <f>'Annual Model'!V48</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Total AUM Growth</t>
         </is>
       </c>
-      <c r="C24" s="12">
+      <c r="C24" s="11">
         <f>'Annual Model'!V48/Summary!$C$5-1</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Total Cumulative Net Income</t>
         </is>
       </c>
-      <c r="C25" s="14">
+      <c r="C25" s="13">
         <f>'Annual Model'!C46+'Annual Model'!D46+'Annual Model'!E46+'Annual Model'!F46+'Annual Model'!G46+'Annual Model'!H46+'Annual Model'!I46+'Annual Model'!J46+'Annual Model'!K46+'Annual Model'!L46+'Annual Model'!M46+'Annual Model'!N46+'Annual Model'!O46+'Annual Model'!P46+'Annual Model'!Q46+'Annual Model'!R46+'Annual Model'!S46+'Annual Model'!T46+'Annual Model'!U46+'Annual Model'!V46</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Total Cumulative Gross Income</t>
         </is>
       </c>
-      <c r="C26" s="14">
+      <c r="C26" s="13">
         <f>'Annual Model'!C36+'Annual Model'!D36+'Annual Model'!E36+'Annual Model'!F36+'Annual Model'!G36+'Annual Model'!H36+'Annual Model'!I36+'Annual Model'!J36+'Annual Model'!K36+'Annual Model'!L36+'Annual Model'!M36+'Annual Model'!N36+'Annual Model'!O36+'Annual Model'!P36+'Annual Model'!Q36+'Annual Model'!R36+'Annual Model'!S36+'Annual Model'!T36+'Annual Model'!U36+'Annual Model'!V36</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Peak AUM</t>
         </is>
       </c>
-      <c r="C27" s="14">
+      <c r="C27" s="13">
         <f>MAX('Annual Model'!C48,'Annual Model'!D48,'Annual Model'!E48,'Annual Model'!F48,'Annual Model'!G48,'Annual Model'!H48,'Annual Model'!I48,'Annual Model'!J48,'Annual Model'!K48,'Annual Model'!L48,'Annual Model'!M48,'Annual Model'!N48,'Annual Model'!O48,'Annual Model'!P48,'Annual Model'!Q48,'Annual Model'!R48,'Annual Model'!S48,'Annual Model'!T48,'Annual Model'!U48,'Annual Model'!V48)</f>
         <v/>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>Fee &amp; Expense Metrics</t>
         </is>
       </c>
-      <c r="B29" s="10" t="n"/>
-      <c r="C29" s="10" t="n"/>
-      <c r="D29" s="10" t="n"/>
-      <c r="E29" s="10" t="n"/>
-      <c r="F29" s="10" t="n"/>
-      <c r="G29" s="10" t="n"/>
-      <c r="H29" s="10" t="n"/>
+      <c r="B29" s="9" t="n"/>
+      <c r="C29" s="9" t="n"/>
+      <c r="D29" s="9" t="n"/>
+      <c r="E29" s="9" t="n"/>
+      <c r="F29" s="9" t="n"/>
+      <c r="G29" s="9" t="n"/>
+      <c r="H29" s="9" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="11" t="inlineStr">
+      <c r="A30" s="10" t="inlineStr">
         <is>
           <t>Total Management Fees</t>
         </is>
       </c>
-      <c r="C30" s="14">
+      <c r="C30" s="13">
         <f>'Annual Model'!C39+'Annual Model'!D39+'Annual Model'!E39+'Annual Model'!F39+'Annual Model'!G39+'Annual Model'!H39+'Annual Model'!I39+'Annual Model'!J39+'Annual Model'!K39+'Annual Model'!L39+'Annual Model'!M39+'Annual Model'!N39+'Annual Model'!O39+'Annual Model'!P39+'Annual Model'!Q39+'Annual Model'!R39+'Annual Model'!S39+'Annual Model'!T39+'Annual Model'!U39+'Annual Model'!V39</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="11" t="inlineStr">
+      <c r="A31" s="10" t="inlineStr">
         <is>
           <t>Total Performance Fees</t>
         </is>
       </c>
-      <c r="C31" s="14">
+      <c r="C31" s="13">
         <f>'Annual Model'!C41+'Annual Model'!D41+'Annual Model'!E41+'Annual Model'!F41+'Annual Model'!G41+'Annual Model'!H41+'Annual Model'!I41+'Annual Model'!J41+'Annual Model'!K41+'Annual Model'!L41+'Annual Model'!M41+'Annual Model'!N41+'Annual Model'!O41+'Annual Model'!P41+'Annual Model'!Q41+'Annual Model'!R41+'Annual Model'!S41+'Annual Model'!T41+'Annual Model'!U41+'Annual Model'!V41</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="11" t="inlineStr">
+      <c r="A32" s="10" t="inlineStr">
         <is>
           <t>Total Other Expenses</t>
         </is>
       </c>
-      <c r="C32" s="14">
+      <c r="C32" s="13">
         <f>'Annual Model'!C42+'Annual Model'!D42+'Annual Model'!E42+'Annual Model'!F42+'Annual Model'!G42+'Annual Model'!H42+'Annual Model'!I42+'Annual Model'!J42+'Annual Model'!K42+'Annual Model'!L42+'Annual Model'!M42+'Annual Model'!N42+'Annual Model'!O42+'Annual Model'!P42+'Annual Model'!Q42+'Annual Model'!R42+'Annual Model'!S42+'Annual Model'!T42+'Annual Model'!U42+'Annual Model'!V42</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="11" t="inlineStr">
+      <c r="A33" s="10" t="inlineStr">
         <is>
           <t>Total All-In Fees &amp; Expenses</t>
         </is>
       </c>
-      <c r="C33" s="14">
+      <c r="C33" s="13">
         <f>'Annual Model'!C43+'Annual Model'!D43+'Annual Model'!E43+'Annual Model'!F43+'Annual Model'!G43+'Annual Model'!H43+'Annual Model'!I43+'Annual Model'!J43+'Annual Model'!K43+'Annual Model'!L43+'Annual Model'!M43+'Annual Model'!N43+'Annual Model'!O43+'Annual Model'!P43+'Annual Model'!Q43+'Annual Model'!R43+'Annual Model'!S43+'Annual Model'!T43+'Annual Model'!U43+'Annual Model'!V43</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="11" t="inlineStr">
+      <c r="A34" s="10" t="inlineStr">
         <is>
           <t>Fee Drag (Fees / Gross Income)</t>
         </is>
       </c>
-      <c r="C34" s="12">
+      <c r="C34" s="11">
         <f>IF(C26=0,0,C33/C26)</f>
         <v/>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="11" t="inlineStr">
+      <c r="A35" s="10" t="inlineStr">
         <is>
           <t>Net-to-Gross Ratio</t>
         </is>
       </c>
-      <c r="C35" s="12">
+      <c r="C35" s="11">
         <f>IF(C26=0,0,C25/C26)</f>
         <v/>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="9" t="inlineStr">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>Yield &amp; Risk Metrics</t>
         </is>
       </c>
-      <c r="B37" s="10" t="n"/>
-      <c r="C37" s="10" t="n"/>
-      <c r="D37" s="10" t="n"/>
-      <c r="E37" s="10" t="n"/>
-      <c r="F37" s="10" t="n"/>
-      <c r="G37" s="10" t="n"/>
-      <c r="H37" s="10" t="n"/>
+      <c r="B37" s="9" t="n"/>
+      <c r="C37" s="9" t="n"/>
+      <c r="D37" s="9" t="n"/>
+      <c r="E37" s="9" t="n"/>
+      <c r="F37" s="9" t="n"/>
+      <c r="G37" s="9" t="n"/>
+      <c r="H37" s="9" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="11" t="inlineStr">
+      <c r="A38" s="10" t="inlineStr">
         <is>
           <t>Year 1 Net Yield</t>
         </is>
       </c>
-      <c r="C38" s="12">
+      <c r="C38" s="11">
         <f>'Annual Model'!C47</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="inlineStr">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>Year 20 Net Yield</t>
         </is>
       </c>
-      <c r="C39" s="12">
+      <c r="C39" s="11">
         <f>'Annual Model'!V47</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="inlineStr">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>Best Year Net Yield</t>
         </is>
       </c>
-      <c r="C40" s="12">
+      <c r="C40" s="11">
         <f>MAX('Annual Model'!C47,'Annual Model'!D47,'Annual Model'!E47,'Annual Model'!F47,'Annual Model'!G47,'Annual Model'!H47,'Annual Model'!I47,'Annual Model'!J47,'Annual Model'!K47,'Annual Model'!L47,'Annual Model'!M47,'Annual Model'!N47,'Annual Model'!O47,'Annual Model'!P47,'Annual Model'!Q47,'Annual Model'!R47,'Annual Model'!S47,'Annual Model'!T47,'Annual Model'!U47,'Annual Model'!V47)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="inlineStr">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>Worst Year Net Yield</t>
         </is>
       </c>
-      <c r="C41" s="12">
+      <c r="C41" s="11">
         <f>MIN('Annual Model'!C47,'Annual Model'!D47,'Annual Model'!E47,'Annual Model'!F47,'Annual Model'!G47,'Annual Model'!H47,'Annual Model'!I47,'Annual Model'!J47,'Annual Model'!K47,'Annual Model'!L47,'Annual Model'!M47,'Annual Model'!N47,'Annual Model'!O47,'Annual Model'!P47,'Annual Model'!Q47,'Annual Model'!R47,'Annual Model'!S47,'Annual Model'!T47,'Annual Model'!U47,'Annual Model'!V47)</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="inlineStr">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>Year 1 Gross Yield</t>
         </is>
       </c>
-      <c r="C42" s="12">
+      <c r="C42" s="11">
         <f>'Annual Model'!C20</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="11" t="inlineStr">
+      <c r="A43" s="10" t="inlineStr">
         <is>
           <t>Gross-to-Net Spread (Avg)</t>
         </is>
       </c>
-      <c r="C43" s="12">
+      <c r="C43" s="11">
         <f>C16-C15</f>
         <v/>
       </c>
     </row>
-    <row r="44">
-      <c r="A44" s="11" t="inlineStr">
-        <is>
-          <t>Leverage Contribution (Year 1)</t>
-        </is>
-      </c>
-      <c r="C44" s="12">
-        <f>IF('Annual Model'!C28=0,0,'Annual Model'!C34/'Annual Model'!C28)</f>
-        <v/>
-      </c>
-    </row>
     <row r="46">
-      <c r="A46" s="15" t="inlineStr">
+      <c r="A46" s="14" t="inlineStr">
         <is>
           <t>Input cells are highlighted in orange. Modify inputs to update the model.</t>
         </is>
       </c>
-      <c r="E46" s="16">
+      <c r="E46" s="15">
         <f> Input</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="35">
+  <mergeCells count="32">
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A11:B11"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A16:B16"/>
@@ -1163,9 +1125,7 @@
     <mergeCell ref="A38:B38"/>
     <mergeCell ref="A43:B43"/>
     <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A10:B10"/>
     <mergeCell ref="A13:H13"/>
-    <mergeCell ref="A44:B44"/>
     <mergeCell ref="A40:B40"/>
     <mergeCell ref="A9:B9"/>
     <mergeCell ref="A31:B31"/>
@@ -1267,938 +1227,938 @@
       <c r="V3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr"/>
-      <c r="B4" s="17" t="n"/>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="A4" s="9" t="inlineStr"/>
+      <c r="B4" s="16" t="n"/>
+      <c r="C4" s="17" t="inlineStr">
         <is>
           <t>Year 1</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>Year 2</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>Year 3</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>Year 4</t>
         </is>
       </c>
-      <c r="G4" s="18" t="inlineStr">
+      <c r="G4" s="17" t="inlineStr">
         <is>
           <t>Year 5</t>
         </is>
       </c>
-      <c r="H4" s="18" t="inlineStr">
+      <c r="H4" s="17" t="inlineStr">
         <is>
           <t>Year 6</t>
         </is>
       </c>
-      <c r="I4" s="18" t="inlineStr">
+      <c r="I4" s="17" t="inlineStr">
         <is>
           <t>Year 7</t>
         </is>
       </c>
-      <c r="J4" s="18" t="inlineStr">
+      <c r="J4" s="17" t="inlineStr">
         <is>
           <t>Year 8</t>
         </is>
       </c>
-      <c r="K4" s="18" t="inlineStr">
+      <c r="K4" s="17" t="inlineStr">
         <is>
           <t>Year 9</t>
         </is>
       </c>
-      <c r="L4" s="18" t="inlineStr">
+      <c r="L4" s="17" t="inlineStr">
         <is>
           <t>Year 10</t>
         </is>
       </c>
-      <c r="M4" s="18" t="inlineStr">
+      <c r="M4" s="17" t="inlineStr">
         <is>
           <t>Year 11</t>
         </is>
       </c>
-      <c r="N4" s="18" t="inlineStr">
+      <c r="N4" s="17" t="inlineStr">
         <is>
           <t>Year 12</t>
         </is>
       </c>
-      <c r="O4" s="18" t="inlineStr">
+      <c r="O4" s="17" t="inlineStr">
         <is>
           <t>Year 13</t>
         </is>
       </c>
-      <c r="P4" s="18" t="inlineStr">
+      <c r="P4" s="17" t="inlineStr">
         <is>
           <t>Year 14</t>
         </is>
       </c>
-      <c r="Q4" s="18" t="inlineStr">
+      <c r="Q4" s="17" t="inlineStr">
         <is>
           <t>Year 15</t>
         </is>
       </c>
-      <c r="R4" s="18" t="inlineStr">
+      <c r="R4" s="17" t="inlineStr">
         <is>
           <t>Year 16</t>
         </is>
       </c>
-      <c r="S4" s="18" t="inlineStr">
+      <c r="S4" s="17" t="inlineStr">
         <is>
           <t>Year 17</t>
         </is>
       </c>
-      <c r="T4" s="18" t="inlineStr">
+      <c r="T4" s="17" t="inlineStr">
         <is>
           <t>Year 18</t>
         </is>
       </c>
-      <c r="U4" s="18" t="inlineStr">
+      <c r="U4" s="17" t="inlineStr">
         <is>
           <t>Year 19</t>
         </is>
       </c>
-      <c r="V4" s="18" t="inlineStr">
+      <c r="V4" s="17" t="inlineStr">
         <is>
           <t>Year 20</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>Asset Allocation</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
+      <c r="B5" s="9" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C5" s="10" t="n"/>
-      <c r="D5" s="10" t="n"/>
-      <c r="E5" s="10" t="n"/>
-      <c r="F5" s="10" t="n"/>
-      <c r="G5" s="10" t="n"/>
-      <c r="H5" s="10" t="n"/>
-      <c r="I5" s="10" t="n"/>
-      <c r="J5" s="10" t="n"/>
-      <c r="K5" s="10" t="n"/>
-      <c r="L5" s="10" t="n"/>
-      <c r="M5" s="10" t="n"/>
-      <c r="N5" s="10" t="n"/>
-      <c r="O5" s="10" t="n"/>
-      <c r="P5" s="10" t="n"/>
-      <c r="Q5" s="10" t="n"/>
-      <c r="R5" s="10" t="n"/>
-      <c r="S5" s="10" t="n"/>
-      <c r="T5" s="10" t="n"/>
-      <c r="U5" s="10" t="n"/>
-      <c r="V5" s="10" t="n"/>
+      <c r="C5" s="9" t="n"/>
+      <c r="D5" s="9" t="n"/>
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="9" t="n"/>
+      <c r="G5" s="9" t="n"/>
+      <c r="H5" s="9" t="n"/>
+      <c r="I5" s="9" t="n"/>
+      <c r="J5" s="9" t="n"/>
+      <c r="K5" s="9" t="n"/>
+      <c r="L5" s="9" t="n"/>
+      <c r="M5" s="9" t="n"/>
+      <c r="N5" s="9" t="n"/>
+      <c r="O5" s="9" t="n"/>
+      <c r="P5" s="9" t="n"/>
+      <c r="Q5" s="9" t="n"/>
+      <c r="R5" s="9" t="n"/>
+      <c r="S5" s="9" t="n"/>
+      <c r="T5" s="9" t="n"/>
+      <c r="U5" s="9" t="n"/>
+      <c r="V5" s="9" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>LIHTC Loans</t>
         </is>
       </c>
-      <c r="B6" s="19" t="n"/>
-      <c r="C6" s="20" t="n">
+      <c r="B6" s="18" t="n"/>
+      <c r="C6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="D6" s="20" t="n">
+      <c r="D6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="F6" s="20" t="n">
+      <c r="F6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="G6" s="20" t="n">
+      <c r="G6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="H6" s="20" t="n">
+      <c r="H6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="I6" s="20" t="n">
+      <c r="I6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="J6" s="20" t="n">
+      <c r="J6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="K6" s="20" t="n">
+      <c r="K6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="L6" s="20" t="n">
+      <c r="L6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="M6" s="20" t="n">
+      <c r="M6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="N6" s="20" t="n">
+      <c r="N6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="O6" s="20" t="n">
+      <c r="O6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="P6" s="20" t="n">
+      <c r="P6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="Q6" s="20" t="n">
+      <c r="Q6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="R6" s="20" t="n">
+      <c r="R6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="S6" s="20" t="n">
+      <c r="S6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="T6" s="20" t="n">
+      <c r="T6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="U6" s="20" t="n">
+      <c r="U6" s="19" t="n">
         <v>0.35</v>
       </c>
-      <c r="V6" s="20" t="n">
+      <c r="V6" s="19" t="n">
         <v>0.35</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Municipal Bonds</t>
         </is>
       </c>
-      <c r="B7" s="19" t="n"/>
-      <c r="C7" s="20" t="n">
+      <c r="B7" s="18" t="n"/>
+      <c r="C7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="D7" s="20" t="n">
+      <c r="D7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="E7" s="20" t="n">
+      <c r="E7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="F7" s="20" t="n">
+      <c r="F7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="G7" s="20" t="n">
+      <c r="G7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="H7" s="20" t="n">
+      <c r="H7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="I7" s="20" t="n">
+      <c r="I7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="J7" s="20" t="n">
+      <c r="J7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="K7" s="20" t="n">
+      <c r="K7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="L7" s="20" t="n">
+      <c r="L7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="M7" s="20" t="n">
+      <c r="M7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="N7" s="20" t="n">
+      <c r="N7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="O7" s="20" t="n">
+      <c r="O7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="P7" s="20" t="n">
+      <c r="P7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="Q7" s="20" t="n">
+      <c r="Q7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="R7" s="20" t="n">
+      <c r="R7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="S7" s="20" t="n">
+      <c r="S7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="T7" s="20" t="n">
+      <c r="T7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="U7" s="20" t="n">
+      <c r="U7" s="19" t="n">
         <v>0.25</v>
       </c>
-      <c r="V7" s="20" t="n">
+      <c r="V7" s="19" t="n">
         <v>0.25</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>JVs</t>
         </is>
       </c>
-      <c r="B8" s="19" t="n"/>
-      <c r="C8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="G8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="J8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="L8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="M8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="N8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="O8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="P8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="Q8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="S8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="T8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="U8" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="V8" s="20" t="n">
+      <c r="B8" s="18" t="n"/>
+      <c r="C8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="L8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="R8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="T8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="U8" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V8" s="19" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Securitization Residuals (B-Pieces)</t>
         </is>
       </c>
-      <c r="B9" s="19" t="n"/>
-      <c r="C9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="D9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="E9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="G9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="H9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="I9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="J9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="K9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="L9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="M9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="N9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="O9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="P9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="Q9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="R9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="S9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="T9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="U9" s="20" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="V9" s="20" t="n">
+      <c r="B9" s="18" t="n"/>
+      <c r="C9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="I9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="K9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="L9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="M9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="P9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="Q9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="R9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="T9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="U9" s="19" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="V9" s="19" t="n">
         <v>0.15</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="B10" s="19" t="n"/>
-      <c r="C10" s="20" t="n">
+      <c r="B10" s="18" t="n"/>
+      <c r="C10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="D10" s="20" t="n">
+      <c r="D10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="G10" s="20" t="n">
+      <c r="G10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="H10" s="20" t="n">
+      <c r="H10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="I10" s="20" t="n">
+      <c r="I10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="J10" s="20" t="n">
+      <c r="J10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="K10" s="20" t="n">
+      <c r="K10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="L10" s="20" t="n">
+      <c r="L10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="M10" s="20" t="n">
+      <c r="M10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="N10" s="20" t="n">
+      <c r="N10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="O10" s="20" t="n">
+      <c r="O10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="P10" s="20" t="n">
+      <c r="P10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="Q10" s="20" t="n">
+      <c r="Q10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="R10" s="20" t="n">
+      <c r="R10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="S10" s="20" t="n">
+      <c r="S10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="T10" s="20" t="n">
+      <c r="T10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="U10" s="20" t="n">
+      <c r="U10" s="19" t="n">
         <v>0.1</v>
       </c>
-      <c r="V10" s="20" t="n">
+      <c r="V10" s="19" t="n">
         <v>0.1</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Total Allocation</t>
         </is>
       </c>
-      <c r="B11" s="19" t="n"/>
-      <c r="C11" s="22">
+      <c r="B11" s="18" t="n"/>
+      <c r="C11" s="21">
         <f>SUM(C6:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="22">
+      <c r="D11" s="21">
         <f>SUM(D6:D10)</f>
         <v/>
       </c>
-      <c r="E11" s="22">
+      <c r="E11" s="21">
         <f>SUM(E6:E10)</f>
         <v/>
       </c>
-      <c r="F11" s="22">
+      <c r="F11" s="21">
         <f>SUM(F6:F10)</f>
         <v/>
       </c>
-      <c r="G11" s="22">
+      <c r="G11" s="21">
         <f>SUM(G6:G10)</f>
         <v/>
       </c>
-      <c r="H11" s="22">
+      <c r="H11" s="21">
         <f>SUM(H6:H10)</f>
         <v/>
       </c>
-      <c r="I11" s="22">
+      <c r="I11" s="21">
         <f>SUM(I6:I10)</f>
         <v/>
       </c>
-      <c r="J11" s="22">
+      <c r="J11" s="21">
         <f>SUM(J6:J10)</f>
         <v/>
       </c>
-      <c r="K11" s="22">
+      <c r="K11" s="21">
         <f>SUM(K6:K10)</f>
         <v/>
       </c>
-      <c r="L11" s="22">
+      <c r="L11" s="21">
         <f>SUM(L6:L10)</f>
         <v/>
       </c>
-      <c r="M11" s="22">
+      <c r="M11" s="21">
         <f>SUM(M6:M10)</f>
         <v/>
       </c>
-      <c r="N11" s="22">
+      <c r="N11" s="21">
         <f>SUM(N6:N10)</f>
         <v/>
       </c>
-      <c r="O11" s="22">
+      <c r="O11" s="21">
         <f>SUM(O6:O10)</f>
         <v/>
       </c>
-      <c r="P11" s="22">
+      <c r="P11" s="21">
         <f>SUM(P6:P10)</f>
         <v/>
       </c>
-      <c r="Q11" s="22">
+      <c r="Q11" s="21">
         <f>SUM(Q6:Q10)</f>
         <v/>
       </c>
-      <c r="R11" s="22">
+      <c r="R11" s="21">
         <f>SUM(R6:R10)</f>
         <v/>
       </c>
-      <c r="S11" s="22">
+      <c r="S11" s="21">
         <f>SUM(S6:S10)</f>
         <v/>
       </c>
-      <c r="T11" s="22">
+      <c r="T11" s="21">
         <f>SUM(T6:T10)</f>
         <v/>
       </c>
-      <c r="U11" s="22">
+      <c r="U11" s="21">
         <f>SUM(U6:U10)</f>
         <v/>
       </c>
-      <c r="V11" s="22">
+      <c r="V11" s="21">
         <f>SUM(V6:V10)</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>Expected Yields</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="9" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
-      <c r="H12" s="10" t="n"/>
-      <c r="I12" s="10" t="n"/>
-      <c r="J12" s="10" t="n"/>
-      <c r="K12" s="10" t="n"/>
-      <c r="L12" s="10" t="n"/>
-      <c r="M12" s="10" t="n"/>
-      <c r="N12" s="10" t="n"/>
-      <c r="O12" s="10" t="n"/>
-      <c r="P12" s="10" t="n"/>
-      <c r="Q12" s="10" t="n"/>
-      <c r="R12" s="10" t="n"/>
-      <c r="S12" s="10" t="n"/>
-      <c r="T12" s="10" t="n"/>
-      <c r="U12" s="10" t="n"/>
-      <c r="V12" s="10" t="n"/>
+      <c r="C12" s="9" t="n"/>
+      <c r="D12" s="9" t="n"/>
+      <c r="E12" s="9" t="n"/>
+      <c r="F12" s="9" t="n"/>
+      <c r="G12" s="9" t="n"/>
+      <c r="H12" s="9" t="n"/>
+      <c r="I12" s="9" t="n"/>
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="9" t="n"/>
+      <c r="L12" s="9" t="n"/>
+      <c r="M12" s="9" t="n"/>
+      <c r="N12" s="9" t="n"/>
+      <c r="O12" s="9" t="n"/>
+      <c r="P12" s="9" t="n"/>
+      <c r="Q12" s="9" t="n"/>
+      <c r="R12" s="9" t="n"/>
+      <c r="S12" s="9" t="n"/>
+      <c r="T12" s="9" t="n"/>
+      <c r="U12" s="9" t="n"/>
+      <c r="V12" s="9" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>LIHTC Loans</t>
         </is>
       </c>
-      <c r="B13" s="19" t="n"/>
-      <c r="C13" s="20" t="n">
+      <c r="B13" s="18" t="n"/>
+      <c r="C13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="D13" s="20" t="n">
+      <c r="D13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="E13" s="20" t="n">
+      <c r="E13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="F13" s="20" t="n">
+      <c r="F13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="G13" s="20" t="n">
+      <c r="G13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="H13" s="20" t="n">
+      <c r="H13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="I13" s="20" t="n">
+      <c r="I13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="J13" s="20" t="n">
+      <c r="J13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="K13" s="20" t="n">
+      <c r="K13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="L13" s="20" t="n">
+      <c r="L13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="M13" s="20" t="n">
+      <c r="M13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="N13" s="20" t="n">
+      <c r="N13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="O13" s="20" t="n">
+      <c r="O13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="P13" s="20" t="n">
+      <c r="P13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="Q13" s="20" t="n">
+      <c r="Q13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="R13" s="20" t="n">
+      <c r="R13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="S13" s="20" t="n">
+      <c r="S13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="T13" s="20" t="n">
+      <c r="T13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="U13" s="20" t="n">
+      <c r="U13" s="19" t="n">
         <v>0.065</v>
       </c>
-      <c r="V13" s="20" t="n">
+      <c r="V13" s="19" t="n">
         <v>0.065</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>Municipal Bonds</t>
         </is>
       </c>
-      <c r="B14" s="19" t="n"/>
-      <c r="C14" s="20" t="n">
+      <c r="B14" s="18" t="n"/>
+      <c r="C14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="D14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="F14" s="20" t="n">
+      <c r="F14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="G14" s="20" t="n">
+      <c r="G14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="H14" s="20" t="n">
+      <c r="H14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="I14" s="20" t="n">
+      <c r="I14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="J14" s="20" t="n">
+      <c r="J14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="K14" s="20" t="n">
+      <c r="K14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="L14" s="20" t="n">
+      <c r="L14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="M14" s="20" t="n">
+      <c r="M14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="N14" s="20" t="n">
+      <c r="N14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="O14" s="20" t="n">
+      <c r="O14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="P14" s="20" t="n">
+      <c r="P14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="Q14" s="20" t="n">
+      <c r="Q14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="R14" s="20" t="n">
+      <c r="R14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="S14" s="20" t="n">
+      <c r="S14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="T14" s="20" t="n">
+      <c r="T14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="U14" s="20" t="n">
+      <c r="U14" s="19" t="n">
         <v>0.045</v>
       </c>
-      <c r="V14" s="20" t="n">
+      <c r="V14" s="19" t="n">
         <v>0.045</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="10" t="inlineStr">
         <is>
           <t>JVs</t>
         </is>
       </c>
-      <c r="B15" s="19" t="n"/>
-      <c r="C15" s="20" t="n">
+      <c r="B15" s="18" t="n"/>
+      <c r="C15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="D15" s="20" t="n">
+      <c r="D15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="E15" s="20" t="n">
+      <c r="E15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="F15" s="20" t="n">
+      <c r="F15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="G15" s="20" t="n">
+      <c r="G15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="H15" s="20" t="n">
+      <c r="H15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="I15" s="20" t="n">
+      <c r="I15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="J15" s="20" t="n">
+      <c r="J15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="K15" s="20" t="n">
+      <c r="K15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="L15" s="20" t="n">
+      <c r="L15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="M15" s="20" t="n">
+      <c r="M15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="N15" s="20" t="n">
+      <c r="N15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="O15" s="20" t="n">
+      <c r="O15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="P15" s="20" t="n">
+      <c r="P15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="Q15" s="20" t="n">
+      <c r="Q15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="R15" s="20" t="n">
+      <c r="R15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="S15" s="20" t="n">
+      <c r="S15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="T15" s="20" t="n">
+      <c r="T15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="U15" s="20" t="n">
+      <c r="U15" s="19" t="n">
         <v>0.08</v>
       </c>
-      <c r="V15" s="20" t="n">
+      <c r="V15" s="19" t="n">
         <v>0.08</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="10" t="inlineStr">
         <is>
           <t>Securitization Residuals (B-Pieces)</t>
         </is>
       </c>
-      <c r="B16" s="19" t="n"/>
-      <c r="C16" s="20" t="n">
+      <c r="B16" s="18" t="n"/>
+      <c r="C16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="D16" s="20" t="n">
+      <c r="D16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="E16" s="20" t="n">
+      <c r="E16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="F16" s="20" t="n">
+      <c r="F16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="G16" s="20" t="n">
+      <c r="G16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="H16" s="20" t="n">
+      <c r="H16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="I16" s="20" t="n">
+      <c r="I16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="J16" s="20" t="n">
+      <c r="J16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="K16" s="20" t="n">
+      <c r="K16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="L16" s="20" t="n">
+      <c r="L16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="M16" s="20" t="n">
+      <c r="M16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="N16" s="20" t="n">
+      <c r="N16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="O16" s="20" t="n">
+      <c r="O16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="P16" s="20" t="n">
+      <c r="P16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="Q16" s="20" t="n">
+      <c r="Q16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="R16" s="20" t="n">
+      <c r="R16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="S16" s="20" t="n">
+      <c r="S16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="T16" s="20" t="n">
+      <c r="T16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="U16" s="20" t="n">
+      <c r="U16" s="19" t="n">
         <v>0.075</v>
       </c>
-      <c r="V16" s="20" t="n">
+      <c r="V16" s="19" t="n">
         <v>0.075</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="B17" s="19" t="n"/>
-      <c r="C17" s="20" t="n">
+      <c r="B17" s="18" t="n"/>
+      <c r="C17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="D17" s="20" t="n">
+      <c r="D17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="E17" s="20" t="n">
+      <c r="E17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="F17" s="20" t="n">
+      <c r="F17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="G17" s="20" t="n">
+      <c r="G17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="H17" s="20" t="n">
+      <c r="H17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="I17" s="20" t="n">
+      <c r="I17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="J17" s="20" t="n">
+      <c r="J17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="K17" s="20" t="n">
+      <c r="K17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="L17" s="20" t="n">
+      <c r="L17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="M17" s="20" t="n">
+      <c r="M17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="N17" s="20" t="n">
+      <c r="N17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="O17" s="20" t="n">
+      <c r="O17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="P17" s="20" t="n">
+      <c r="P17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="Q17" s="20" t="n">
+      <c r="Q17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="R17" s="20" t="n">
+      <c r="R17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="S17" s="20" t="n">
+      <c r="S17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="T17" s="20" t="n">
+      <c r="T17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="U17" s="20" t="n">
+      <c r="U17" s="19" t="n">
         <v>0.02</v>
       </c>
-      <c r="V17" s="20" t="n">
+      <c r="V17" s="19" t="n">
         <v>0.02</v>
       </c>
     </row>
@@ -2231,1218 +2191,834 @@
       <c r="V18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="20" t="inlineStr">
         <is>
           <t>Beginning AUM</t>
         </is>
       </c>
-      <c r="B19" s="23" t="inlineStr">
+      <c r="B19" s="22" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="C19" s="14">
+      <c r="C19" s="13">
         <f>Summary!$C$5</f>
         <v/>
       </c>
-      <c r="D19" s="14">
+      <c r="D19" s="13">
         <f>C48</f>
         <v/>
       </c>
-      <c r="E19" s="14">
+      <c r="E19" s="13">
         <f>D48</f>
         <v/>
       </c>
-      <c r="F19" s="14">
+      <c r="F19" s="13">
         <f>E48</f>
         <v/>
       </c>
-      <c r="G19" s="14">
+      <c r="G19" s="13">
         <f>F48</f>
         <v/>
       </c>
-      <c r="H19" s="14">
+      <c r="H19" s="13">
         <f>G48</f>
         <v/>
       </c>
-      <c r="I19" s="14">
+      <c r="I19" s="13">
         <f>H48</f>
         <v/>
       </c>
-      <c r="J19" s="14">
+      <c r="J19" s="13">
         <f>I48</f>
         <v/>
       </c>
-      <c r="K19" s="14">
+      <c r="K19" s="13">
         <f>J48</f>
         <v/>
       </c>
-      <c r="L19" s="14">
+      <c r="L19" s="13">
         <f>K48</f>
         <v/>
       </c>
-      <c r="M19" s="14">
+      <c r="M19" s="13">
         <f>L48</f>
         <v/>
       </c>
-      <c r="N19" s="14">
+      <c r="N19" s="13">
         <f>M48</f>
         <v/>
       </c>
-      <c r="O19" s="14">
+      <c r="O19" s="13">
         <f>N48</f>
         <v/>
       </c>
-      <c r="P19" s="14">
+      <c r="P19" s="13">
         <f>O48</f>
         <v/>
       </c>
-      <c r="Q19" s="14">
+      <c r="Q19" s="13">
         <f>P48</f>
         <v/>
       </c>
-      <c r="R19" s="14">
+      <c r="R19" s="13">
         <f>Q48</f>
         <v/>
       </c>
-      <c r="S19" s="14">
+      <c r="S19" s="13">
         <f>R48</f>
         <v/>
       </c>
-      <c r="T19" s="14">
+      <c r="T19" s="13">
         <f>S48</f>
         <v/>
       </c>
-      <c r="U19" s="14">
+      <c r="U19" s="13">
         <f>T48</f>
         <v/>
       </c>
-      <c r="V19" s="14">
+      <c r="V19" s="13">
         <f>U48</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="21" t="inlineStr">
+      <c r="A20" s="20" t="inlineStr">
         <is>
           <t>Gross Portfolio Yield</t>
         </is>
       </c>
-      <c r="B20" s="23" t="inlineStr">
+      <c r="B20" s="22" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="11">
         <f>SUMPRODUCT(C6:C10,C13:C17)</f>
         <v/>
       </c>
-      <c r="D20" s="12">
+      <c r="D20" s="11">
         <f>SUMPRODUCT(D6:D10,D13:D17)</f>
         <v/>
       </c>
-      <c r="E20" s="12">
+      <c r="E20" s="11">
         <f>SUMPRODUCT(E6:E10,E13:E17)</f>
         <v/>
       </c>
-      <c r="F20" s="12">
+      <c r="F20" s="11">
         <f>SUMPRODUCT(F6:F10,F13:F17)</f>
         <v/>
       </c>
-      <c r="G20" s="12">
+      <c r="G20" s="11">
         <f>SUMPRODUCT(G6:G10,G13:G17)</f>
         <v/>
       </c>
-      <c r="H20" s="12">
+      <c r="H20" s="11">
         <f>SUMPRODUCT(H6:H10,H13:H17)</f>
         <v/>
       </c>
-      <c r="I20" s="12">
+      <c r="I20" s="11">
         <f>SUMPRODUCT(I6:I10,I13:I17)</f>
         <v/>
       </c>
-      <c r="J20" s="12">
+      <c r="J20" s="11">
         <f>SUMPRODUCT(J6:J10,J13:J17)</f>
         <v/>
       </c>
-      <c r="K20" s="12">
+      <c r="K20" s="11">
         <f>SUMPRODUCT(K6:K10,K13:K17)</f>
         <v/>
       </c>
-      <c r="L20" s="12">
+      <c r="L20" s="11">
         <f>SUMPRODUCT(L6:L10,L13:L17)</f>
         <v/>
       </c>
-      <c r="M20" s="12">
+      <c r="M20" s="11">
         <f>SUMPRODUCT(M6:M10,M13:M17)</f>
         <v/>
       </c>
-      <c r="N20" s="12">
+      <c r="N20" s="11">
         <f>SUMPRODUCT(N6:N10,N13:N17)</f>
         <v/>
       </c>
-      <c r="O20" s="12">
+      <c r="O20" s="11">
         <f>SUMPRODUCT(O6:O10,O13:O17)</f>
         <v/>
       </c>
-      <c r="P20" s="12">
+      <c r="P20" s="11">
         <f>SUMPRODUCT(P6:P10,P13:P17)</f>
         <v/>
       </c>
-      <c r="Q20" s="12">
+      <c r="Q20" s="11">
         <f>SUMPRODUCT(Q6:Q10,Q13:Q17)</f>
         <v/>
       </c>
-      <c r="R20" s="12">
+      <c r="R20" s="11">
         <f>SUMPRODUCT(R6:R10,R13:R17)</f>
         <v/>
       </c>
-      <c r="S20" s="12">
+      <c r="S20" s="11">
         <f>SUMPRODUCT(S6:S10,S13:S17)</f>
         <v/>
       </c>
-      <c r="T20" s="12">
+      <c r="T20" s="11">
         <f>SUMPRODUCT(T6:T10,T13:T17)</f>
         <v/>
       </c>
-      <c r="U20" s="12">
+      <c r="U20" s="11">
         <f>SUMPRODUCT(U6:U10,U13:U17)</f>
         <v/>
       </c>
-      <c r="V20" s="12">
+      <c r="V20" s="11">
         <f>SUMPRODUCT(V6:V10,V13:V17)</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="inlineStr">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>Income by Asset Class</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="9" t="inlineStr">
         <is>
           <t>$</t>
         </is>
       </c>
-      <c r="C22" s="10" t="n"/>
-      <c r="D22" s="10" t="n"/>
-      <c r="E22" s="10" t="n"/>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
-      <c r="H22" s="10" t="n"/>
-      <c r="I22" s="10" t="n"/>
-      <c r="J22" s="10" t="n"/>
-      <c r="K22" s="10" t="n"/>
-      <c r="L22" s="10" t="n"/>
-      <c r="M22" s="10" t="n"/>
-      <c r="N22" s="10" t="n"/>
-      <c r="O22" s="10" t="n"/>
-      <c r="P22" s="10" t="n"/>
-      <c r="Q22" s="10" t="n"/>
-      <c r="R22" s="10" t="n"/>
-      <c r="S22" s="10" t="n"/>
-      <c r="T22" s="10" t="n"/>
-      <c r="U22" s="10" t="n"/>
-      <c r="V22" s="10" t="n"/>
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="9" t="n"/>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="9" t="n"/>
+      <c r="I22" s="9" t="n"/>
+      <c r="J22" s="9" t="n"/>
+      <c r="K22" s="9" t="n"/>
+      <c r="L22" s="9" t="n"/>
+      <c r="M22" s="9" t="n"/>
+      <c r="N22" s="9" t="n"/>
+      <c r="O22" s="9" t="n"/>
+      <c r="P22" s="9" t="n"/>
+      <c r="Q22" s="9" t="n"/>
+      <c r="R22" s="9" t="n"/>
+      <c r="S22" s="9" t="n"/>
+      <c r="T22" s="9" t="n"/>
+      <c r="U22" s="9" t="n"/>
+      <c r="V22" s="9" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>LIHTC Loans</t>
         </is>
       </c>
-      <c r="B23" s="19" t="n"/>
-      <c r="C23" s="24">
+      <c r="B23" s="18" t="n"/>
+      <c r="C23" s="23">
         <f>C19*C6*C13</f>
         <v/>
       </c>
-      <c r="D23" s="24">
+      <c r="D23" s="23">
         <f>D19*D6*D13</f>
         <v/>
       </c>
-      <c r="E23" s="24">
+      <c r="E23" s="23">
         <f>E19*E6*E13</f>
         <v/>
       </c>
-      <c r="F23" s="24">
+      <c r="F23" s="23">
         <f>F19*F6*F13</f>
         <v/>
       </c>
-      <c r="G23" s="24">
+      <c r="G23" s="23">
         <f>G19*G6*G13</f>
         <v/>
       </c>
-      <c r="H23" s="24">
+      <c r="H23" s="23">
         <f>H19*H6*H13</f>
         <v/>
       </c>
-      <c r="I23" s="24">
+      <c r="I23" s="23">
         <f>I19*I6*I13</f>
         <v/>
       </c>
-      <c r="J23" s="24">
+      <c r="J23" s="23">
         <f>J19*J6*J13</f>
         <v/>
       </c>
-      <c r="K23" s="24">
+      <c r="K23" s="23">
         <f>K19*K6*K13</f>
         <v/>
       </c>
-      <c r="L23" s="24">
+      <c r="L23" s="23">
         <f>L19*L6*L13</f>
         <v/>
       </c>
-      <c r="M23" s="24">
+      <c r="M23" s="23">
         <f>M19*M6*M13</f>
         <v/>
       </c>
-      <c r="N23" s="24">
+      <c r="N23" s="23">
         <f>N19*N6*N13</f>
         <v/>
       </c>
-      <c r="O23" s="24">
+      <c r="O23" s="23">
         <f>O19*O6*O13</f>
         <v/>
       </c>
-      <c r="P23" s="24">
+      <c r="P23" s="23">
         <f>P19*P6*P13</f>
         <v/>
       </c>
-      <c r="Q23" s="24">
+      <c r="Q23" s="23">
         <f>Q19*Q6*Q13</f>
         <v/>
       </c>
-      <c r="R23" s="24">
+      <c r="R23" s="23">
         <f>R19*R6*R13</f>
         <v/>
       </c>
-      <c r="S23" s="24">
+      <c r="S23" s="23">
         <f>S19*S6*S13</f>
         <v/>
       </c>
-      <c r="T23" s="24">
+      <c r="T23" s="23">
         <f>T19*T6*T13</f>
         <v/>
       </c>
-      <c r="U23" s="24">
+      <c r="U23" s="23">
         <f>U19*U6*U13</f>
         <v/>
       </c>
-      <c r="V23" s="24">
+      <c r="V23" s="23">
         <f>V19*V6*V13</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Municipal Bonds</t>
         </is>
       </c>
-      <c r="B24" s="19" t="n"/>
-      <c r="C24" s="24">
+      <c r="B24" s="18" t="n"/>
+      <c r="C24" s="23">
         <f>C19*C7*C14</f>
         <v/>
       </c>
-      <c r="D24" s="24">
+      <c r="D24" s="23">
         <f>D19*D7*D14</f>
         <v/>
       </c>
-      <c r="E24" s="24">
+      <c r="E24" s="23">
         <f>E19*E7*E14</f>
         <v/>
       </c>
-      <c r="F24" s="24">
+      <c r="F24" s="23">
         <f>F19*F7*F14</f>
         <v/>
       </c>
-      <c r="G24" s="24">
+      <c r="G24" s="23">
         <f>G19*G7*G14</f>
         <v/>
       </c>
-      <c r="H24" s="24">
+      <c r="H24" s="23">
         <f>H19*H7*H14</f>
         <v/>
       </c>
-      <c r="I24" s="24">
+      <c r="I24" s="23">
         <f>I19*I7*I14</f>
         <v/>
       </c>
-      <c r="J24" s="24">
+      <c r="J24" s="23">
         <f>J19*J7*J14</f>
         <v/>
       </c>
-      <c r="K24" s="24">
+      <c r="K24" s="23">
         <f>K19*K7*K14</f>
         <v/>
       </c>
-      <c r="L24" s="24">
+      <c r="L24" s="23">
         <f>L19*L7*L14</f>
         <v/>
       </c>
-      <c r="M24" s="24">
+      <c r="M24" s="23">
         <f>M19*M7*M14</f>
         <v/>
       </c>
-      <c r="N24" s="24">
+      <c r="N24" s="23">
         <f>N19*N7*N14</f>
         <v/>
       </c>
-      <c r="O24" s="24">
+      <c r="O24" s="23">
         <f>O19*O7*O14</f>
         <v/>
       </c>
-      <c r="P24" s="24">
+      <c r="P24" s="23">
         <f>P19*P7*P14</f>
         <v/>
       </c>
-      <c r="Q24" s="24">
+      <c r="Q24" s="23">
         <f>Q19*Q7*Q14</f>
         <v/>
       </c>
-      <c r="R24" s="24">
+      <c r="R24" s="23">
         <f>R19*R7*R14</f>
         <v/>
       </c>
-      <c r="S24" s="24">
+      <c r="S24" s="23">
         <f>S19*S7*S14</f>
         <v/>
       </c>
-      <c r="T24" s="24">
+      <c r="T24" s="23">
         <f>T19*T7*T14</f>
         <v/>
       </c>
-      <c r="U24" s="24">
+      <c r="U24" s="23">
         <f>U19*U7*U14</f>
         <v/>
       </c>
-      <c r="V24" s="24">
+      <c r="V24" s="23">
         <f>V19*V7*V14</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>JVs</t>
         </is>
       </c>
-      <c r="B25" s="19" t="n"/>
-      <c r="C25" s="24">
+      <c r="B25" s="18" t="n"/>
+      <c r="C25" s="23">
         <f>C19*C8*C15</f>
         <v/>
       </c>
-      <c r="D25" s="24">
+      <c r="D25" s="23">
         <f>D19*D8*D15</f>
         <v/>
       </c>
-      <c r="E25" s="24">
+      <c r="E25" s="23">
         <f>E19*E8*E15</f>
         <v/>
       </c>
-      <c r="F25" s="24">
+      <c r="F25" s="23">
         <f>F19*F8*F15</f>
         <v/>
       </c>
-      <c r="G25" s="24">
+      <c r="G25" s="23">
         <f>G19*G8*G15</f>
         <v/>
       </c>
-      <c r="H25" s="24">
+      <c r="H25" s="23">
         <f>H19*H8*H15</f>
         <v/>
       </c>
-      <c r="I25" s="24">
+      <c r="I25" s="23">
         <f>I19*I8*I15</f>
         <v/>
       </c>
-      <c r="J25" s="24">
+      <c r="J25" s="23">
         <f>J19*J8*J15</f>
         <v/>
       </c>
-      <c r="K25" s="24">
+      <c r="K25" s="23">
         <f>K19*K8*K15</f>
         <v/>
       </c>
-      <c r="L25" s="24">
+      <c r="L25" s="23">
         <f>L19*L8*L15</f>
         <v/>
       </c>
-      <c r="M25" s="24">
+      <c r="M25" s="23">
         <f>M19*M8*M15</f>
         <v/>
       </c>
-      <c r="N25" s="24">
+      <c r="N25" s="23">
         <f>N19*N8*N15</f>
         <v/>
       </c>
-      <c r="O25" s="24">
+      <c r="O25" s="23">
         <f>O19*O8*O15</f>
         <v/>
       </c>
-      <c r="P25" s="24">
+      <c r="P25" s="23">
         <f>P19*P8*P15</f>
         <v/>
       </c>
-      <c r="Q25" s="24">
+      <c r="Q25" s="23">
         <f>Q19*Q8*Q15</f>
         <v/>
       </c>
-      <c r="R25" s="24">
+      <c r="R25" s="23">
         <f>R19*R8*R15</f>
         <v/>
       </c>
-      <c r="S25" s="24">
+      <c r="S25" s="23">
         <f>S19*S8*S15</f>
         <v/>
       </c>
-      <c r="T25" s="24">
+      <c r="T25" s="23">
         <f>T19*T8*T15</f>
         <v/>
       </c>
-      <c r="U25" s="24">
+      <c r="U25" s="23">
         <f>U19*U8*U15</f>
         <v/>
       </c>
-      <c r="V25" s="24">
+      <c r="V25" s="23">
         <f>V19*V8*V15</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Securitization Residuals (B-Pieces)</t>
         </is>
       </c>
-      <c r="B26" s="19" t="n"/>
-      <c r="C26" s="24">
+      <c r="B26" s="18" t="n"/>
+      <c r="C26" s="23">
         <f>C19*C9*C16</f>
         <v/>
       </c>
-      <c r="D26" s="24">
+      <c r="D26" s="23">
         <f>D19*D9*D16</f>
         <v/>
       </c>
-      <c r="E26" s="24">
+      <c r="E26" s="23">
         <f>E19*E9*E16</f>
         <v/>
       </c>
-      <c r="F26" s="24">
+      <c r="F26" s="23">
         <f>F19*F9*F16</f>
         <v/>
       </c>
-      <c r="G26" s="24">
+      <c r="G26" s="23">
         <f>G19*G9*G16</f>
         <v/>
       </c>
-      <c r="H26" s="24">
+      <c r="H26" s="23">
         <f>H19*H9*H16</f>
         <v/>
       </c>
-      <c r="I26" s="24">
+      <c r="I26" s="23">
         <f>I19*I9*I16</f>
         <v/>
       </c>
-      <c r="J26" s="24">
+      <c r="J26" s="23">
         <f>J19*J9*J16</f>
         <v/>
       </c>
-      <c r="K26" s="24">
+      <c r="K26" s="23">
         <f>K19*K9*K16</f>
         <v/>
       </c>
-      <c r="L26" s="24">
+      <c r="L26" s="23">
         <f>L19*L9*L16</f>
         <v/>
       </c>
-      <c r="M26" s="24">
+      <c r="M26" s="23">
         <f>M19*M9*M16</f>
         <v/>
       </c>
-      <c r="N26" s="24">
+      <c r="N26" s="23">
         <f>N19*N9*N16</f>
         <v/>
       </c>
-      <c r="O26" s="24">
+      <c r="O26" s="23">
         <f>O19*O9*O16</f>
         <v/>
       </c>
-      <c r="P26" s="24">
+      <c r="P26" s="23">
         <f>P19*P9*P16</f>
         <v/>
       </c>
-      <c r="Q26" s="24">
+      <c r="Q26" s="23">
         <f>Q19*Q9*Q16</f>
         <v/>
       </c>
-      <c r="R26" s="24">
+      <c r="R26" s="23">
         <f>R19*R9*R16</f>
         <v/>
       </c>
-      <c r="S26" s="24">
+      <c r="S26" s="23">
         <f>S19*S9*S16</f>
         <v/>
       </c>
-      <c r="T26" s="24">
+      <c r="T26" s="23">
         <f>T19*T9*T16</f>
         <v/>
       </c>
-      <c r="U26" s="24">
+      <c r="U26" s="23">
         <f>U19*U9*U16</f>
         <v/>
       </c>
-      <c r="V26" s="24">
+      <c r="V26" s="23">
         <f>V19*V9*V16</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Cash</t>
         </is>
       </c>
-      <c r="B27" s="19" t="n"/>
-      <c r="C27" s="24">
+      <c r="B27" s="18" t="n"/>
+      <c r="C27" s="23">
         <f>C19*C10*C17</f>
         <v/>
       </c>
-      <c r="D27" s="24">
+      <c r="D27" s="23">
         <f>D19*D10*D17</f>
         <v/>
       </c>
-      <c r="E27" s="24">
+      <c r="E27" s="23">
         <f>E19*E10*E17</f>
         <v/>
       </c>
-      <c r="F27" s="24">
+      <c r="F27" s="23">
         <f>F19*F10*F17</f>
         <v/>
       </c>
-      <c r="G27" s="24">
+      <c r="G27" s="23">
         <f>G19*G10*G17</f>
         <v/>
       </c>
-      <c r="H27" s="24">
+      <c r="H27" s="23">
         <f>H19*H10*H17</f>
         <v/>
       </c>
-      <c r="I27" s="24">
+      <c r="I27" s="23">
         <f>I19*I10*I17</f>
         <v/>
       </c>
-      <c r="J27" s="24">
+      <c r="J27" s="23">
         <f>J19*J10*J17</f>
         <v/>
       </c>
-      <c r="K27" s="24">
+      <c r="K27" s="23">
         <f>K19*K10*K17</f>
         <v/>
       </c>
-      <c r="L27" s="24">
+      <c r="L27" s="23">
         <f>L19*L10*L17</f>
         <v/>
       </c>
-      <c r="M27" s="24">
+      <c r="M27" s="23">
         <f>M19*M10*M17</f>
         <v/>
       </c>
-      <c r="N27" s="24">
+      <c r="N27" s="23">
         <f>N19*N10*N17</f>
         <v/>
       </c>
-      <c r="O27" s="24">
+      <c r="O27" s="23">
         <f>O19*O10*O17</f>
         <v/>
       </c>
-      <c r="P27" s="24">
+      <c r="P27" s="23">
         <f>P19*P10*P17</f>
         <v/>
       </c>
-      <c r="Q27" s="24">
+      <c r="Q27" s="23">
         <f>Q19*Q10*Q17</f>
         <v/>
       </c>
-      <c r="R27" s="24">
+      <c r="R27" s="23">
         <f>R19*R10*R17</f>
         <v/>
       </c>
-      <c r="S27" s="24">
+      <c r="S27" s="23">
         <f>S19*S10*S17</f>
         <v/>
       </c>
-      <c r="T27" s="24">
+      <c r="T27" s="23">
         <f>T19*T10*T17</f>
         <v/>
       </c>
-      <c r="U27" s="24">
+      <c r="U27" s="23">
         <f>U19*U10*U17</f>
         <v/>
       </c>
-      <c r="V27" s="24">
+      <c r="V27" s="23">
         <f>V19*V10*V17</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="21" t="inlineStr">
+      <c r="A28" s="20" t="inlineStr">
         <is>
           <t>Total Asset Income</t>
         </is>
       </c>
-      <c r="B28" s="19" t="n"/>
-      <c r="C28" s="25">
+      <c r="B28" s="18" t="n"/>
+      <c r="C28" s="24">
         <f>SUM(C23:C27)</f>
         <v/>
       </c>
-      <c r="D28" s="25">
+      <c r="D28" s="24">
         <f>SUM(D23:D27)</f>
         <v/>
       </c>
-      <c r="E28" s="25">
+      <c r="E28" s="24">
         <f>SUM(E23:E27)</f>
         <v/>
       </c>
-      <c r="F28" s="25">
+      <c r="F28" s="24">
         <f>SUM(F23:F27)</f>
         <v/>
       </c>
-      <c r="G28" s="25">
+      <c r="G28" s="24">
         <f>SUM(G23:G27)</f>
         <v/>
       </c>
-      <c r="H28" s="25">
+      <c r="H28" s="24">
         <f>SUM(H23:H27)</f>
         <v/>
       </c>
-      <c r="I28" s="25">
+      <c r="I28" s="24">
         <f>SUM(I23:I27)</f>
         <v/>
       </c>
-      <c r="J28" s="25">
+      <c r="J28" s="24">
         <f>SUM(J23:J27)</f>
         <v/>
       </c>
-      <c r="K28" s="25">
+      <c r="K28" s="24">
         <f>SUM(K23:K27)</f>
         <v/>
       </c>
-      <c r="L28" s="25">
+      <c r="L28" s="24">
         <f>SUM(L23:L27)</f>
         <v/>
       </c>
-      <c r="M28" s="25">
+      <c r="M28" s="24">
         <f>SUM(M23:M27)</f>
         <v/>
       </c>
-      <c r="N28" s="25">
+      <c r="N28" s="24">
         <f>SUM(N23:N27)</f>
         <v/>
       </c>
-      <c r="O28" s="25">
+      <c r="O28" s="24">
         <f>SUM(O23:O27)</f>
         <v/>
       </c>
-      <c r="P28" s="25">
+      <c r="P28" s="24">
         <f>SUM(P23:P27)</f>
         <v/>
       </c>
-      <c r="Q28" s="25">
+      <c r="Q28" s="24">
         <f>SUM(Q23:Q27)</f>
         <v/>
       </c>
-      <c r="R28" s="25">
+      <c r="R28" s="24">
         <f>SUM(R23:R27)</f>
         <v/>
       </c>
-      <c r="S28" s="25">
+      <c r="S28" s="24">
         <f>SUM(S23:S27)</f>
         <v/>
       </c>
-      <c r="T28" s="25">
+      <c r="T28" s="24">
         <f>SUM(T23:T27)</f>
         <v/>
       </c>
-      <c r="U28" s="25">
+      <c r="U28" s="24">
         <f>SUM(U23:U27)</f>
         <v/>
       </c>
-      <c r="V28" s="25">
+      <c r="V28" s="24">
         <f>SUM(V23:V27)</f>
         <v/>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>Leverage</t>
-        </is>
-      </c>
-      <c r="B30" s="10" t="inlineStr">
-        <is>
-          <t>$</t>
-        </is>
-      </c>
-      <c r="C30" s="10" t="n"/>
-      <c r="D30" s="10" t="n"/>
-      <c r="E30" s="10" t="n"/>
-      <c r="F30" s="10" t="n"/>
-      <c r="G30" s="10" t="n"/>
-      <c r="H30" s="10" t="n"/>
-      <c r="I30" s="10" t="n"/>
-      <c r="J30" s="10" t="n"/>
-      <c r="K30" s="10" t="n"/>
-      <c r="L30" s="10" t="n"/>
-      <c r="M30" s="10" t="n"/>
-      <c r="N30" s="10" t="n"/>
-      <c r="O30" s="10" t="n"/>
-      <c r="P30" s="10" t="n"/>
-      <c r="Q30" s="10" t="n"/>
-      <c r="R30" s="10" t="n"/>
-      <c r="S30" s="10" t="n"/>
-      <c r="T30" s="10" t="n"/>
-      <c r="U30" s="10" t="n"/>
-      <c r="V30" s="10" t="n"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="11" t="inlineStr">
-        <is>
-          <t>Leveraged AUM</t>
-        </is>
-      </c>
-      <c r="B31" s="19" t="n"/>
-      <c r="C31" s="24">
-        <f>C19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="D31" s="24">
-        <f>D19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="E31" s="24">
-        <f>E19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="F31" s="24">
-        <f>F19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="G31" s="24">
-        <f>G19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="H31" s="24">
-        <f>H19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="I31" s="24">
-        <f>I19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="J31" s="24">
-        <f>J19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="K31" s="24">
-        <f>K19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="L31" s="24">
-        <f>L19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="M31" s="24">
-        <f>M19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="N31" s="24">
-        <f>N19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="O31" s="24">
-        <f>O19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="P31" s="24">
-        <f>P19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="Q31" s="24">
-        <f>Q19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="R31" s="24">
-        <f>R19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="S31" s="24">
-        <f>S19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="T31" s="24">
-        <f>T19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="U31" s="24">
-        <f>U19*Summary!$C$10</f>
-        <v/>
-      </c>
-      <c r="V31" s="24">
-        <f>V19*Summary!$C$10</f>
-        <v/>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="11" t="inlineStr">
-        <is>
-          <t>Leveraged Income</t>
-        </is>
-      </c>
-      <c r="B32" s="19" t="n"/>
-      <c r="C32" s="24">
-        <f>C31*C20</f>
-        <v/>
-      </c>
-      <c r="D32" s="24">
-        <f>D31*D20</f>
-        <v/>
-      </c>
-      <c r="E32" s="24">
-        <f>E31*E20</f>
-        <v/>
-      </c>
-      <c r="F32" s="24">
-        <f>F31*F20</f>
-        <v/>
-      </c>
-      <c r="G32" s="24">
-        <f>G31*G20</f>
-        <v/>
-      </c>
-      <c r="H32" s="24">
-        <f>H31*H20</f>
-        <v/>
-      </c>
-      <c r="I32" s="24">
-        <f>I31*I20</f>
-        <v/>
-      </c>
-      <c r="J32" s="24">
-        <f>J31*J20</f>
-        <v/>
-      </c>
-      <c r="K32" s="24">
-        <f>K31*K20</f>
-        <v/>
-      </c>
-      <c r="L32" s="24">
-        <f>L31*L20</f>
-        <v/>
-      </c>
-      <c r="M32" s="24">
-        <f>M31*M20</f>
-        <v/>
-      </c>
-      <c r="N32" s="24">
-        <f>N31*N20</f>
-        <v/>
-      </c>
-      <c r="O32" s="24">
-        <f>O31*O20</f>
-        <v/>
-      </c>
-      <c r="P32" s="24">
-        <f>P31*P20</f>
-        <v/>
-      </c>
-      <c r="Q32" s="24">
-        <f>Q31*Q20</f>
-        <v/>
-      </c>
-      <c r="R32" s="24">
-        <f>R31*R20</f>
-        <v/>
-      </c>
-      <c r="S32" s="24">
-        <f>S31*S20</f>
-        <v/>
-      </c>
-      <c r="T32" s="24">
-        <f>T31*T20</f>
-        <v/>
-      </c>
-      <c r="U32" s="24">
-        <f>U31*U20</f>
-        <v/>
-      </c>
-      <c r="V32" s="24">
-        <f>V31*V20</f>
-        <v/>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" s="11" t="inlineStr">
-        <is>
-          <t>Leverage Cost</t>
-        </is>
-      </c>
-      <c r="B33" s="19" t="n"/>
-      <c r="C33" s="24">
-        <f>C31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="D33" s="24">
-        <f>D31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="E33" s="24">
-        <f>E31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="F33" s="24">
-        <f>F31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="G33" s="24">
-        <f>G31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="H33" s="24">
-        <f>H31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="I33" s="24">
-        <f>I31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="J33" s="24">
-        <f>J31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="K33" s="24">
-        <f>K31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="L33" s="24">
-        <f>L31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="M33" s="24">
-        <f>M31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="N33" s="24">
-        <f>N31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="O33" s="24">
-        <f>O31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="P33" s="24">
-        <f>P31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="Q33" s="24">
-        <f>Q31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="R33" s="24">
-        <f>R31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="S33" s="24">
-        <f>S31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="T33" s="24">
-        <f>T31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="U33" s="24">
-        <f>U31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-      <c r="V33" s="24">
-        <f>V31*Summary!$C$11/10000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="21" t="inlineStr">
-        <is>
-          <t>Net Leverage Income</t>
-        </is>
-      </c>
-      <c r="B34" s="19" t="n"/>
-      <c r="C34" s="25">
-        <f>C32-C33</f>
-        <v/>
-      </c>
-      <c r="D34" s="25">
-        <f>D32-D33</f>
-        <v/>
-      </c>
-      <c r="E34" s="25">
-        <f>E32-E33</f>
-        <v/>
-      </c>
-      <c r="F34" s="25">
-        <f>F32-F33</f>
-        <v/>
-      </c>
-      <c r="G34" s="25">
-        <f>G32-G33</f>
-        <v/>
-      </c>
-      <c r="H34" s="25">
-        <f>H32-H33</f>
-        <v/>
-      </c>
-      <c r="I34" s="25">
-        <f>I32-I33</f>
-        <v/>
-      </c>
-      <c r="J34" s="25">
-        <f>J32-J33</f>
-        <v/>
-      </c>
-      <c r="K34" s="25">
-        <f>K32-K33</f>
-        <v/>
-      </c>
-      <c r="L34" s="25">
-        <f>L32-L33</f>
-        <v/>
-      </c>
-      <c r="M34" s="25">
-        <f>M32-M33</f>
-        <v/>
-      </c>
-      <c r="N34" s="25">
-        <f>N32-N33</f>
-        <v/>
-      </c>
-      <c r="O34" s="25">
-        <f>O32-O33</f>
-        <v/>
-      </c>
-      <c r="P34" s="25">
-        <f>P32-P33</f>
-        <v/>
-      </c>
-      <c r="Q34" s="25">
-        <f>Q32-Q33</f>
-        <v/>
-      </c>
-      <c r="R34" s="25">
-        <f>R32-R33</f>
-        <v/>
-      </c>
-      <c r="S34" s="25">
-        <f>S32-S33</f>
-        <v/>
-      </c>
-      <c r="T34" s="25">
-        <f>T32-T33</f>
-        <v/>
-      </c>
-      <c r="U34" s="25">
-        <f>U32-U33</f>
-        <v/>
-      </c>
-      <c r="V34" s="25">
-        <f>V32-V33</f>
-        <v/>
-      </c>
-    </row>
     <row r="36">
-      <c r="A36" s="26" t="inlineStr">
+      <c r="A36" s="25" t="inlineStr">
         <is>
           <t>TOTAL GROSS INCOME</t>
         </is>
       </c>
-      <c r="B36" s="27" t="n"/>
-      <c r="C36" s="28">
-        <f>C28+C34</f>
-        <v/>
-      </c>
-      <c r="D36" s="28">
-        <f>D28+D34</f>
-        <v/>
-      </c>
-      <c r="E36" s="28">
-        <f>E28+E34</f>
-        <v/>
-      </c>
-      <c r="F36" s="28">
-        <f>F28+F34</f>
-        <v/>
-      </c>
-      <c r="G36" s="28">
-        <f>G28+G34</f>
-        <v/>
-      </c>
-      <c r="H36" s="28">
-        <f>H28+H34</f>
-        <v/>
-      </c>
-      <c r="I36" s="28">
-        <f>I28+I34</f>
-        <v/>
-      </c>
-      <c r="J36" s="28">
-        <f>J28+J34</f>
-        <v/>
-      </c>
-      <c r="K36" s="28">
-        <f>K28+K34</f>
-        <v/>
-      </c>
-      <c r="L36" s="28">
-        <f>L28+L34</f>
-        <v/>
-      </c>
-      <c r="M36" s="28">
-        <f>M28+M34</f>
-        <v/>
-      </c>
-      <c r="N36" s="28">
-        <f>N28+N34</f>
-        <v/>
-      </c>
-      <c r="O36" s="28">
-        <f>O28+O34</f>
-        <v/>
-      </c>
-      <c r="P36" s="28">
-        <f>P28+P34</f>
-        <v/>
-      </c>
-      <c r="Q36" s="28">
-        <f>Q28+Q34</f>
-        <v/>
-      </c>
-      <c r="R36" s="28">
-        <f>R28+R34</f>
-        <v/>
-      </c>
-      <c r="S36" s="28">
-        <f>S28+S34</f>
-        <v/>
-      </c>
-      <c r="T36" s="28">
-        <f>T28+T34</f>
-        <v/>
-      </c>
-      <c r="U36" s="28">
-        <f>U28+U34</f>
-        <v/>
-      </c>
-      <c r="V36" s="28">
-        <f>V28+V34</f>
+      <c r="B36" s="26" t="n"/>
+      <c r="C36" s="27">
+        <f>C28</f>
+        <v/>
+      </c>
+      <c r="D36" s="27">
+        <f>D28</f>
+        <v/>
+      </c>
+      <c r="E36" s="27">
+        <f>E28</f>
+        <v/>
+      </c>
+      <c r="F36" s="27">
+        <f>F28</f>
+        <v/>
+      </c>
+      <c r="G36" s="27">
+        <f>G28</f>
+        <v/>
+      </c>
+      <c r="H36" s="27">
+        <f>H28</f>
+        <v/>
+      </c>
+      <c r="I36" s="27">
+        <f>I28</f>
+        <v/>
+      </c>
+      <c r="J36" s="27">
+        <f>J28</f>
+        <v/>
+      </c>
+      <c r="K36" s="27">
+        <f>K28</f>
+        <v/>
+      </c>
+      <c r="L36" s="27">
+        <f>L28</f>
+        <v/>
+      </c>
+      <c r="M36" s="27">
+        <f>M28</f>
+        <v/>
+      </c>
+      <c r="N36" s="27">
+        <f>N28</f>
+        <v/>
+      </c>
+      <c r="O36" s="27">
+        <f>O28</f>
+        <v/>
+      </c>
+      <c r="P36" s="27">
+        <f>P28</f>
+        <v/>
+      </c>
+      <c r="Q36" s="27">
+        <f>Q28</f>
+        <v/>
+      </c>
+      <c r="R36" s="27">
+        <f>R28</f>
+        <v/>
+      </c>
+      <c r="S36" s="27">
+        <f>S28</f>
+        <v/>
+      </c>
+      <c r="T36" s="27">
+        <f>T28</f>
+        <v/>
+      </c>
+      <c r="U36" s="27">
+        <f>U28</f>
+        <v/>
+      </c>
+      <c r="V36" s="27">
+        <f>V28</f>
         <v/>
       </c>
     </row>
@@ -3475,441 +3051,441 @@
       <c r="V38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="11" t="inlineStr">
+      <c r="A39" s="10" t="inlineStr">
         <is>
           <t>Management Fee</t>
         </is>
       </c>
-      <c r="B39" s="19" t="n"/>
-      <c r="C39" s="24">
+      <c r="B39" s="18" t="n"/>
+      <c r="C39" s="23">
         <f>C19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="D39" s="24">
+      <c r="D39" s="23">
         <f>D19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="E39" s="24">
+      <c r="E39" s="23">
         <f>E19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="F39" s="24">
+      <c r="F39" s="23">
         <f>F19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="G39" s="24">
+      <c r="G39" s="23">
         <f>G19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="H39" s="24">
+      <c r="H39" s="23">
         <f>H19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="I39" s="24">
+      <c r="I39" s="23">
         <f>I19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="J39" s="24">
+      <c r="J39" s="23">
         <f>J19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="K39" s="24">
+      <c r="K39" s="23">
         <f>K19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="L39" s="24">
+      <c r="L39" s="23">
         <f>L19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="M39" s="24">
+      <c r="M39" s="23">
         <f>M19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="N39" s="24">
+      <c r="N39" s="23">
         <f>N19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="O39" s="24">
+      <c r="O39" s="23">
         <f>O19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="P39" s="24">
+      <c r="P39" s="23">
         <f>P19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="Q39" s="24">
+      <c r="Q39" s="23">
         <f>Q19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="R39" s="24">
+      <c r="R39" s="23">
         <f>R19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="S39" s="24">
+      <c r="S39" s="23">
         <f>S19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="T39" s="24">
+      <c r="T39" s="23">
         <f>T19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="U39" s="24">
+      <c r="U39" s="23">
         <f>U19*Summary!$C$6/10000</f>
         <v/>
       </c>
-      <c r="V39" s="24">
+      <c r="V39" s="23">
         <f>V19*Summary!$C$6/10000</f>
         <v/>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="11" t="inlineStr">
+      <c r="A40" s="10" t="inlineStr">
         <is>
           <t>Return Above Hurdle</t>
         </is>
       </c>
-      <c r="B40" s="19" t="n"/>
-      <c r="C40" s="24">
+      <c r="B40" s="18" t="n"/>
+      <c r="C40" s="23">
         <f>MAX(0,C36-C19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="D40" s="24">
+      <c r="D40" s="23">
         <f>MAX(0,D36-D19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="E40" s="24">
+      <c r="E40" s="23">
         <f>MAX(0,E36-E19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="F40" s="24">
+      <c r="F40" s="23">
         <f>MAX(0,F36-F19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="G40" s="24">
+      <c r="G40" s="23">
         <f>MAX(0,G36-G19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="H40" s="24">
+      <c r="H40" s="23">
         <f>MAX(0,H36-H19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="I40" s="24">
+      <c r="I40" s="23">
         <f>MAX(0,I36-I19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="J40" s="24">
+      <c r="J40" s="23">
         <f>MAX(0,J36-J19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="K40" s="24">
+      <c r="K40" s="23">
         <f>MAX(0,K36-K19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="L40" s="24">
+      <c r="L40" s="23">
         <f>MAX(0,L36-L19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="M40" s="24">
+      <c r="M40" s="23">
         <f>MAX(0,M36-M19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="N40" s="24">
+      <c r="N40" s="23">
         <f>MAX(0,N36-N19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="O40" s="24">
+      <c r="O40" s="23">
         <f>MAX(0,O36-O19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="P40" s="24">
+      <c r="P40" s="23">
         <f>MAX(0,P36-P19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="Q40" s="24">
+      <c r="Q40" s="23">
         <f>MAX(0,Q36-Q19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="R40" s="24">
+      <c r="R40" s="23">
         <f>MAX(0,R36-R19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="S40" s="24">
+      <c r="S40" s="23">
         <f>MAX(0,S36-S19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="T40" s="24">
+      <c r="T40" s="23">
         <f>MAX(0,T36-T19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="U40" s="24">
+      <c r="U40" s="23">
         <f>MAX(0,U36-U19*Summary!$C$8/10000)</f>
         <v/>
       </c>
-      <c r="V40" s="24">
+      <c r="V40" s="23">
         <f>MAX(0,V36-V19*Summary!$C$8/10000)</f>
         <v/>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="11" t="inlineStr">
+      <c r="A41" s="10" t="inlineStr">
         <is>
           <t>Performance Fee</t>
         </is>
       </c>
-      <c r="B41" s="19" t="n"/>
-      <c r="C41" s="24">
+      <c r="B41" s="18" t="n"/>
+      <c r="C41" s="23">
         <f>C40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="D41" s="24">
+      <c r="D41" s="23">
         <f>D40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="E41" s="24">
+      <c r="E41" s="23">
         <f>E40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="F41" s="24">
+      <c r="F41" s="23">
         <f>F40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="G41" s="24">
+      <c r="G41" s="23">
         <f>G40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="H41" s="24">
+      <c r="H41" s="23">
         <f>H40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="I41" s="24">
+      <c r="I41" s="23">
         <f>I40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="J41" s="24">
+      <c r="J41" s="23">
         <f>J40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="K41" s="24">
+      <c r="K41" s="23">
         <f>K40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="L41" s="24">
+      <c r="L41" s="23">
         <f>L40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="M41" s="24">
+      <c r="M41" s="23">
         <f>M40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="N41" s="24">
+      <c r="N41" s="23">
         <f>N40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="O41" s="24">
+      <c r="O41" s="23">
         <f>O40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="P41" s="24">
+      <c r="P41" s="23">
         <f>P40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="Q41" s="24">
+      <c r="Q41" s="23">
         <f>Q40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="R41" s="24">
+      <c r="R41" s="23">
         <f>R40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="S41" s="24">
+      <c r="S41" s="23">
         <f>S40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="T41" s="24">
+      <c r="T41" s="23">
         <f>T40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="U41" s="24">
+      <c r="U41" s="23">
         <f>U40*Summary!$C$7/10000</f>
         <v/>
       </c>
-      <c r="V41" s="24">
+      <c r="V41" s="23">
         <f>V40*Summary!$C$7/10000</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="11" t="inlineStr">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t>Other Expenses</t>
         </is>
       </c>
-      <c r="B42" s="19" t="n"/>
-      <c r="C42" s="24">
+      <c r="B42" s="18" t="n"/>
+      <c r="C42" s="23">
         <f>C19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="D42" s="24">
+      <c r="D42" s="23">
         <f>D19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="E42" s="24">
+      <c r="E42" s="23">
         <f>E19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="F42" s="24">
+      <c r="F42" s="23">
         <f>F19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="G42" s="24">
+      <c r="G42" s="23">
         <f>G19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="H42" s="24">
+      <c r="H42" s="23">
         <f>H19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="I42" s="24">
+      <c r="I42" s="23">
         <f>I19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="J42" s="24">
+      <c r="J42" s="23">
         <f>J19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="K42" s="24">
+      <c r="K42" s="23">
         <f>K19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="L42" s="24">
+      <c r="L42" s="23">
         <f>L19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="M42" s="24">
+      <c r="M42" s="23">
         <f>M19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="N42" s="24">
+      <c r="N42" s="23">
         <f>N19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="O42" s="24">
+      <c r="O42" s="23">
         <f>O19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="P42" s="24">
+      <c r="P42" s="23">
         <f>P19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="Q42" s="24">
+      <c r="Q42" s="23">
         <f>Q19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="R42" s="24">
+      <c r="R42" s="23">
         <f>R19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="S42" s="24">
+      <c r="S42" s="23">
         <f>S19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="T42" s="24">
+      <c r="T42" s="23">
         <f>T19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="U42" s="24">
+      <c r="U42" s="23">
         <f>U19*Summary!$C$9/10000</f>
         <v/>
       </c>
-      <c r="V42" s="24">
+      <c r="V42" s="23">
         <f>V19*Summary!$C$9/10000</f>
         <v/>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="21" t="inlineStr">
+      <c r="A43" s="20" t="inlineStr">
         <is>
           <t>Total Fees &amp; Expenses</t>
         </is>
       </c>
-      <c r="B43" s="19" t="n"/>
-      <c r="C43" s="25">
+      <c r="B43" s="18" t="n"/>
+      <c r="C43" s="24">
         <f>C39+C41+C42</f>
         <v/>
       </c>
-      <c r="D43" s="25">
+      <c r="D43" s="24">
         <f>D39+D41+D42</f>
         <v/>
       </c>
-      <c r="E43" s="25">
+      <c r="E43" s="24">
         <f>E39+E41+E42</f>
         <v/>
       </c>
-      <c r="F43" s="25">
+      <c r="F43" s="24">
         <f>F39+F41+F42</f>
         <v/>
       </c>
-      <c r="G43" s="25">
+      <c r="G43" s="24">
         <f>G39+G41+G42</f>
         <v/>
       </c>
-      <c r="H43" s="25">
+      <c r="H43" s="24">
         <f>H39+H41+H42</f>
         <v/>
       </c>
-      <c r="I43" s="25">
+      <c r="I43" s="24">
         <f>I39+I41+I42</f>
         <v/>
       </c>
-      <c r="J43" s="25">
+      <c r="J43" s="24">
         <f>J39+J41+J42</f>
         <v/>
       </c>
-      <c r="K43" s="25">
+      <c r="K43" s="24">
         <f>K39+K41+K42</f>
         <v/>
       </c>
-      <c r="L43" s="25">
+      <c r="L43" s="24">
         <f>L39+L41+L42</f>
         <v/>
       </c>
-      <c r="M43" s="25">
+      <c r="M43" s="24">
         <f>M39+M41+M42</f>
         <v/>
       </c>
-      <c r="N43" s="25">
+      <c r="N43" s="24">
         <f>N39+N41+N42</f>
         <v/>
       </c>
-      <c r="O43" s="25">
+      <c r="O43" s="24">
         <f>O39+O41+O42</f>
         <v/>
       </c>
-      <c r="P43" s="25">
+      <c r="P43" s="24">
         <f>P39+P41+P42</f>
         <v/>
       </c>
-      <c r="Q43" s="25">
+      <c r="Q43" s="24">
         <f>Q39+Q41+Q42</f>
         <v/>
       </c>
-      <c r="R43" s="25">
+      <c r="R43" s="24">
         <f>R39+R41+R42</f>
         <v/>
       </c>
-      <c r="S43" s="25">
+      <c r="S43" s="24">
         <f>S39+S41+S42</f>
         <v/>
       </c>
-      <c r="T43" s="25">
+      <c r="T43" s="24">
         <f>T39+T41+T42</f>
         <v/>
       </c>
-      <c r="U43" s="25">
+      <c r="U43" s="24">
         <f>U39+U41+U42</f>
         <v/>
       </c>
-      <c r="V43" s="25">
+      <c r="V43" s="24">
         <f>V39+V41+V42</f>
         <v/>
       </c>
@@ -3943,265 +3519,265 @@
       <c r="V45" s="3" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="29" t="inlineStr">
+      <c r="A46" s="28" t="inlineStr">
         <is>
           <t>NET INCOME</t>
         </is>
       </c>
-      <c r="B46" s="30" t="n"/>
-      <c r="C46" s="31">
+      <c r="B46" s="29" t="n"/>
+      <c r="C46" s="30">
         <f>C36-C43</f>
         <v/>
       </c>
-      <c r="D46" s="31">
+      <c r="D46" s="30">
         <f>D36-D43</f>
         <v/>
       </c>
-      <c r="E46" s="31">
+      <c r="E46" s="30">
         <f>E36-E43</f>
         <v/>
       </c>
-      <c r="F46" s="31">
+      <c r="F46" s="30">
         <f>F36-F43</f>
         <v/>
       </c>
-      <c r="G46" s="31">
+      <c r="G46" s="30">
         <f>G36-G43</f>
         <v/>
       </c>
-      <c r="H46" s="31">
+      <c r="H46" s="30">
         <f>H36-H43</f>
         <v/>
       </c>
-      <c r="I46" s="31">
+      <c r="I46" s="30">
         <f>I36-I43</f>
         <v/>
       </c>
-      <c r="J46" s="31">
+      <c r="J46" s="30">
         <f>J36-J43</f>
         <v/>
       </c>
-      <c r="K46" s="31">
+      <c r="K46" s="30">
         <f>K36-K43</f>
         <v/>
       </c>
-      <c r="L46" s="31">
+      <c r="L46" s="30">
         <f>L36-L43</f>
         <v/>
       </c>
-      <c r="M46" s="31">
+      <c r="M46" s="30">
         <f>M36-M43</f>
         <v/>
       </c>
-      <c r="N46" s="31">
+      <c r="N46" s="30">
         <f>N36-N43</f>
         <v/>
       </c>
-      <c r="O46" s="31">
+      <c r="O46" s="30">
         <f>O36-O43</f>
         <v/>
       </c>
-      <c r="P46" s="31">
+      <c r="P46" s="30">
         <f>P36-P43</f>
         <v/>
       </c>
-      <c r="Q46" s="31">
+      <c r="Q46" s="30">
         <f>Q36-Q43</f>
         <v/>
       </c>
-      <c r="R46" s="31">
+      <c r="R46" s="30">
         <f>R36-R43</f>
         <v/>
       </c>
-      <c r="S46" s="31">
+      <c r="S46" s="30">
         <f>S36-S43</f>
         <v/>
       </c>
-      <c r="T46" s="31">
+      <c r="T46" s="30">
         <f>T36-T43</f>
         <v/>
       </c>
-      <c r="U46" s="31">
+      <c r="U46" s="30">
         <f>U36-U43</f>
         <v/>
       </c>
-      <c r="V46" s="31">
+      <c r="V46" s="30">
         <f>V36-V43</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="29" t="inlineStr">
+      <c r="A47" s="28" t="inlineStr">
         <is>
           <t>NET YIELD (Return to LPs)</t>
         </is>
       </c>
-      <c r="B47" s="30" t="n"/>
-      <c r="C47" s="32">
+      <c r="B47" s="29" t="n"/>
+      <c r="C47" s="31">
         <f>IF(C19=0,0,C46/C19)</f>
         <v/>
       </c>
-      <c r="D47" s="32">
+      <c r="D47" s="31">
         <f>IF(D19=0,0,D46/D19)</f>
         <v/>
       </c>
-      <c r="E47" s="32">
+      <c r="E47" s="31">
         <f>IF(E19=0,0,E46/E19)</f>
         <v/>
       </c>
-      <c r="F47" s="32">
+      <c r="F47" s="31">
         <f>IF(F19=0,0,F46/F19)</f>
         <v/>
       </c>
-      <c r="G47" s="32">
+      <c r="G47" s="31">
         <f>IF(G19=0,0,G46/G19)</f>
         <v/>
       </c>
-      <c r="H47" s="32">
+      <c r="H47" s="31">
         <f>IF(H19=0,0,H46/H19)</f>
         <v/>
       </c>
-      <c r="I47" s="32">
+      <c r="I47" s="31">
         <f>IF(I19=0,0,I46/I19)</f>
         <v/>
       </c>
-      <c r="J47" s="32">
+      <c r="J47" s="31">
         <f>IF(J19=0,0,J46/J19)</f>
         <v/>
       </c>
-      <c r="K47" s="32">
+      <c r="K47" s="31">
         <f>IF(K19=0,0,K46/K19)</f>
         <v/>
       </c>
-      <c r="L47" s="32">
+      <c r="L47" s="31">
         <f>IF(L19=0,0,L46/L19)</f>
         <v/>
       </c>
-      <c r="M47" s="32">
+      <c r="M47" s="31">
         <f>IF(M19=0,0,M46/M19)</f>
         <v/>
       </c>
-      <c r="N47" s="32">
+      <c r="N47" s="31">
         <f>IF(N19=0,0,N46/N19)</f>
         <v/>
       </c>
-      <c r="O47" s="32">
+      <c r="O47" s="31">
         <f>IF(O19=0,0,O46/O19)</f>
         <v/>
       </c>
-      <c r="P47" s="32">
+      <c r="P47" s="31">
         <f>IF(P19=0,0,P46/P19)</f>
         <v/>
       </c>
-      <c r="Q47" s="32">
+      <c r="Q47" s="31">
         <f>IF(Q19=0,0,Q46/Q19)</f>
         <v/>
       </c>
-      <c r="R47" s="32">
+      <c r="R47" s="31">
         <f>IF(R19=0,0,R46/R19)</f>
         <v/>
       </c>
-      <c r="S47" s="32">
+      <c r="S47" s="31">
         <f>IF(S19=0,0,S46/S19)</f>
         <v/>
       </c>
-      <c r="T47" s="32">
+      <c r="T47" s="31">
         <f>IF(T19=0,0,T46/T19)</f>
         <v/>
       </c>
-      <c r="U47" s="32">
+      <c r="U47" s="31">
         <f>IF(U19=0,0,U46/U19)</f>
         <v/>
       </c>
-      <c r="V47" s="32">
+      <c r="V47" s="31">
         <f>IF(V19=0,0,V46/V19)</f>
         <v/>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="33" t="inlineStr">
+      <c r="A48" s="32" t="inlineStr">
         <is>
           <t>ENDING AUM</t>
         </is>
       </c>
-      <c r="B48" s="34" t="n"/>
-      <c r="C48" s="35">
+      <c r="B48" s="33" t="n"/>
+      <c r="C48" s="34">
         <f>C19+C46</f>
         <v/>
       </c>
-      <c r="D48" s="35">
+      <c r="D48" s="34">
         <f>D19+D46</f>
         <v/>
       </c>
-      <c r="E48" s="35">
+      <c r="E48" s="34">
         <f>E19+E46</f>
         <v/>
       </c>
-      <c r="F48" s="35">
+      <c r="F48" s="34">
         <f>F19+F46</f>
         <v/>
       </c>
-      <c r="G48" s="35">
+      <c r="G48" s="34">
         <f>G19+G46</f>
         <v/>
       </c>
-      <c r="H48" s="35">
+      <c r="H48" s="34">
         <f>H19+H46</f>
         <v/>
       </c>
-      <c r="I48" s="35">
+      <c r="I48" s="34">
         <f>I19+I46</f>
         <v/>
       </c>
-      <c r="J48" s="35">
+      <c r="J48" s="34">
         <f>J19+J46</f>
         <v/>
       </c>
-      <c r="K48" s="35">
+      <c r="K48" s="34">
         <f>K19+K46</f>
         <v/>
       </c>
-      <c r="L48" s="35">
+      <c r="L48" s="34">
         <f>L19+L46</f>
         <v/>
       </c>
-      <c r="M48" s="35">
+      <c r="M48" s="34">
         <f>M19+M46</f>
         <v/>
       </c>
-      <c r="N48" s="35">
+      <c r="N48" s="34">
         <f>N19+N46</f>
         <v/>
       </c>
-      <c r="O48" s="35">
+      <c r="O48" s="34">
         <f>O19+O46</f>
         <v/>
       </c>
-      <c r="P48" s="35">
+      <c r="P48" s="34">
         <f>P19+P46</f>
         <v/>
       </c>
-      <c r="Q48" s="35">
+      <c r="Q48" s="34">
         <f>Q19+Q46</f>
         <v/>
       </c>
-      <c r="R48" s="35">
+      <c r="R48" s="34">
         <f>R19+R46</f>
         <v/>
       </c>
-      <c r="S48" s="35">
+      <c r="S48" s="34">
         <f>S19+S46</f>
         <v/>
       </c>
-      <c r="T48" s="35">
+      <c r="T48" s="34">
         <f>T19+T46</f>
         <v/>
       </c>
-      <c r="U48" s="35">
+      <c r="U48" s="34">
         <f>U19+U46</f>
         <v/>
       </c>
-      <c r="V48" s="35">
+      <c r="V48" s="34">
         <f>V19+V46</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Adjust AUM for securitization proceeds distributed to LPs
When a securitization is active, the senior tranche proceeds (loan +
JV) represent cash returned to shareholders and must reduce AUM in the
subsequent period. Added a new 'Less: Securitization Proceeds
(Distributed to LPs)' row in the RETURNS section that sums
ROW_LOAN_SENIOR + ROW_JV_SENIOR, and updated the Ending AUM formula:

  Ending AUM = Beg AUM + Net Income − Securitization Proceeds

With zero securitization inputs the new row evaluates to 0 and behaviour
is unchanged. Added 'secur_proceeds' key to the rows mapping dict.

https://claude.ai/code/session_01FUg7ULd3526dZxFrGj5CR2
</commit_message>
<xml_diff>
--- a/LP_Financial_Model.xlsx
+++ b/LP_Financial_Model.xlsx
@@ -840,7 +840,7 @@
         </is>
       </c>
       <c r="C17" s="12">
-        <f>'Annual Model'!V87/Summary!$C$5</f>
+        <f>'Annual Model'!V88/Summary!$C$5</f>
         <v/>
       </c>
     </row>
@@ -862,7 +862,7 @@
         </is>
       </c>
       <c r="C19" s="12">
-        <f>('Annual Model'!V87+'Annual Model'!C85+'Annual Model'!D85+'Annual Model'!E85+'Annual Model'!F85+'Annual Model'!G85+'Annual Model'!H85+'Annual Model'!I85+'Annual Model'!J85+'Annual Model'!K85+'Annual Model'!L85+'Annual Model'!M85+'Annual Model'!N85+'Annual Model'!O85+'Annual Model'!P85+'Annual Model'!Q85+'Annual Model'!R85+'Annual Model'!S85+'Annual Model'!T85+'Annual Model'!U85+'Annual Model'!V85)/Summary!$C$5</f>
+        <f>('Annual Model'!V88+'Annual Model'!C85+'Annual Model'!D85+'Annual Model'!E85+'Annual Model'!F85+'Annual Model'!G85+'Annual Model'!H85+'Annual Model'!I85+'Annual Model'!J85+'Annual Model'!K85+'Annual Model'!L85+'Annual Model'!M85+'Annual Model'!N85+'Annual Model'!O85+'Annual Model'!P85+'Annual Model'!Q85+'Annual Model'!R85+'Annual Model'!S85+'Annual Model'!T85+'Annual Model'!U85+'Annual Model'!V85)/Summary!$C$5</f>
         <v/>
       </c>
     </row>
@@ -898,7 +898,7 @@
         </is>
       </c>
       <c r="C23" s="13">
-        <f>'Annual Model'!V87</f>
+        <f>'Annual Model'!V88</f>
         <v/>
       </c>
     </row>
@@ -909,7 +909,7 @@
         </is>
       </c>
       <c r="C24" s="11">
-        <f>'Annual Model'!V87/Summary!$C$5-1</f>
+        <f>'Annual Model'!V88/Summary!$C$5-1</f>
         <v/>
       </c>
     </row>
@@ -942,7 +942,7 @@
         </is>
       </c>
       <c r="C27" s="13">
-        <f>MAX('Annual Model'!C87,'Annual Model'!D87,'Annual Model'!E87,'Annual Model'!F87,'Annual Model'!G87,'Annual Model'!H87,'Annual Model'!I87,'Annual Model'!J87,'Annual Model'!K87,'Annual Model'!L87,'Annual Model'!M87,'Annual Model'!N87,'Annual Model'!O87,'Annual Model'!P87,'Annual Model'!Q87,'Annual Model'!R87,'Annual Model'!S87,'Annual Model'!T87,'Annual Model'!U87,'Annual Model'!V87)</f>
+        <f>MAX('Annual Model'!C88,'Annual Model'!D88,'Annual Model'!E88,'Annual Model'!F88,'Annual Model'!G88,'Annual Model'!H88,'Annual Model'!I88,'Annual Model'!J88,'Annual Model'!K88,'Annual Model'!L88,'Annual Model'!M88,'Annual Model'!N88,'Annual Model'!O88,'Annual Model'!P88,'Annual Model'!Q88,'Annual Model'!R88,'Annual Model'!S88,'Annual Model'!T88,'Annual Model'!U88,'Annual Model'!V88)</f>
         <v/>
       </c>
     </row>
@@ -2325,7 +2325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V87"/>
+  <dimension ref="A1:V88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -4000,79 +4000,79 @@
         <v/>
       </c>
       <c r="D32" s="13">
-        <f>C87</f>
+        <f>C88</f>
         <v/>
       </c>
       <c r="E32" s="13">
-        <f>D87</f>
+        <f>D88</f>
         <v/>
       </c>
       <c r="F32" s="13">
-        <f>E87</f>
+        <f>E88</f>
         <v/>
       </c>
       <c r="G32" s="13">
-        <f>F87</f>
+        <f>F88</f>
         <v/>
       </c>
       <c r="H32" s="13">
-        <f>G87</f>
+        <f>G88</f>
         <v/>
       </c>
       <c r="I32" s="13">
-        <f>H87</f>
+        <f>H88</f>
         <v/>
       </c>
       <c r="J32" s="13">
-        <f>I87</f>
+        <f>I88</f>
         <v/>
       </c>
       <c r="K32" s="13">
-        <f>J87</f>
+        <f>J88</f>
         <v/>
       </c>
       <c r="L32" s="13">
-        <f>K87</f>
+        <f>K88</f>
         <v/>
       </c>
       <c r="M32" s="13">
-        <f>L87</f>
+        <f>L88</f>
         <v/>
       </c>
       <c r="N32" s="13">
-        <f>M87</f>
+        <f>M88</f>
         <v/>
       </c>
       <c r="O32" s="13">
-        <f>N87</f>
+        <f>N88</f>
         <v/>
       </c>
       <c r="P32" s="13">
-        <f>O87</f>
+        <f>O88</f>
         <v/>
       </c>
       <c r="Q32" s="13">
-        <f>P87</f>
+        <f>P88</f>
         <v/>
       </c>
       <c r="R32" s="13">
-        <f>Q87</f>
+        <f>Q88</f>
         <v/>
       </c>
       <c r="S32" s="13">
-        <f>R87</f>
+        <f>R88</f>
         <v/>
       </c>
       <c r="T32" s="13">
-        <f>S87</f>
+        <f>S88</f>
         <v/>
       </c>
       <c r="U32" s="13">
-        <f>T87</f>
+        <f>T88</f>
         <v/>
       </c>
       <c r="V32" s="13">
-        <f>U87</f>
+        <f>U88</f>
         <v/>
       </c>
     </row>
@@ -7901,95 +7901,183 @@
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="36" t="inlineStr">
+      <c r="A87" s="32" t="inlineStr">
+        <is>
+          <t>Less: Securitization Proceeds (Distributed to LPs)</t>
+        </is>
+      </c>
+      <c r="B87" s="33" t="n"/>
+      <c r="C87" s="34">
+        <f>C57+C66</f>
+        <v/>
+      </c>
+      <c r="D87" s="34">
+        <f>D57+D66</f>
+        <v/>
+      </c>
+      <c r="E87" s="34">
+        <f>E57+E66</f>
+        <v/>
+      </c>
+      <c r="F87" s="34">
+        <f>F57+F66</f>
+        <v/>
+      </c>
+      <c r="G87" s="34">
+        <f>G57+G66</f>
+        <v/>
+      </c>
+      <c r="H87" s="34">
+        <f>H57+H66</f>
+        <v/>
+      </c>
+      <c r="I87" s="34">
+        <f>I57+I66</f>
+        <v/>
+      </c>
+      <c r="J87" s="34">
+        <f>J57+J66</f>
+        <v/>
+      </c>
+      <c r="K87" s="34">
+        <f>K57+K66</f>
+        <v/>
+      </c>
+      <c r="L87" s="34">
+        <f>L57+L66</f>
+        <v/>
+      </c>
+      <c r="M87" s="34">
+        <f>M57+M66</f>
+        <v/>
+      </c>
+      <c r="N87" s="34">
+        <f>N57+N66</f>
+        <v/>
+      </c>
+      <c r="O87" s="34">
+        <f>O57+O66</f>
+        <v/>
+      </c>
+      <c r="P87" s="34">
+        <f>P57+P66</f>
+        <v/>
+      </c>
+      <c r="Q87" s="34">
+        <f>Q57+Q66</f>
+        <v/>
+      </c>
+      <c r="R87" s="34">
+        <f>R57+R66</f>
+        <v/>
+      </c>
+      <c r="S87" s="34">
+        <f>S57+S66</f>
+        <v/>
+      </c>
+      <c r="T87" s="34">
+        <f>T57+T66</f>
+        <v/>
+      </c>
+      <c r="U87" s="34">
+        <f>U57+U66</f>
+        <v/>
+      </c>
+      <c r="V87" s="34">
+        <f>V57+V66</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="36" t="inlineStr">
         <is>
           <t>ENDING AUM</t>
         </is>
       </c>
-      <c r="B87" s="37" t="n"/>
-      <c r="C87" s="38">
-        <f>C32+C85</f>
-        <v/>
-      </c>
-      <c r="D87" s="38">
-        <f>D32+D85</f>
-        <v/>
-      </c>
-      <c r="E87" s="38">
-        <f>E32+E85</f>
-        <v/>
-      </c>
-      <c r="F87" s="38">
-        <f>F32+F85</f>
-        <v/>
-      </c>
-      <c r="G87" s="38">
-        <f>G32+G85</f>
-        <v/>
-      </c>
-      <c r="H87" s="38">
-        <f>H32+H85</f>
-        <v/>
-      </c>
-      <c r="I87" s="38">
-        <f>I32+I85</f>
-        <v/>
-      </c>
-      <c r="J87" s="38">
-        <f>J32+J85</f>
-        <v/>
-      </c>
-      <c r="K87" s="38">
-        <f>K32+K85</f>
-        <v/>
-      </c>
-      <c r="L87" s="38">
-        <f>L32+L85</f>
-        <v/>
-      </c>
-      <c r="M87" s="38">
-        <f>M32+M85</f>
-        <v/>
-      </c>
-      <c r="N87" s="38">
-        <f>N32+N85</f>
-        <v/>
-      </c>
-      <c r="O87" s="38">
-        <f>O32+O85</f>
-        <v/>
-      </c>
-      <c r="P87" s="38">
-        <f>P32+P85</f>
-        <v/>
-      </c>
-      <c r="Q87" s="38">
-        <f>Q32+Q85</f>
-        <v/>
-      </c>
-      <c r="R87" s="38">
-        <f>R32+R85</f>
-        <v/>
-      </c>
-      <c r="S87" s="38">
-        <f>S32+S85</f>
-        <v/>
-      </c>
-      <c r="T87" s="38">
-        <f>T32+T85</f>
-        <v/>
-      </c>
-      <c r="U87" s="38">
-        <f>U32+U85</f>
-        <v/>
-      </c>
-      <c r="V87" s="38">
-        <f>V32+V85</f>
+      <c r="B88" s="37" t="n"/>
+      <c r="C88" s="38">
+        <f>C32+C85-C87</f>
+        <v/>
+      </c>
+      <c r="D88" s="38">
+        <f>D32+D85-D87</f>
+        <v/>
+      </c>
+      <c r="E88" s="38">
+        <f>E32+E85-E87</f>
+        <v/>
+      </c>
+      <c r="F88" s="38">
+        <f>F32+F85-F87</f>
+        <v/>
+      </c>
+      <c r="G88" s="38">
+        <f>G32+G85-G87</f>
+        <v/>
+      </c>
+      <c r="H88" s="38">
+        <f>H32+H85-H87</f>
+        <v/>
+      </c>
+      <c r="I88" s="38">
+        <f>I32+I85-I87</f>
+        <v/>
+      </c>
+      <c r="J88" s="38">
+        <f>J32+J85-J87</f>
+        <v/>
+      </c>
+      <c r="K88" s="38">
+        <f>K32+K85-K87</f>
+        <v/>
+      </c>
+      <c r="L88" s="38">
+        <f>L32+L85-L87</f>
+        <v/>
+      </c>
+      <c r="M88" s="38">
+        <f>M32+M85-M87</f>
+        <v/>
+      </c>
+      <c r="N88" s="38">
+        <f>N32+N85-N87</f>
+        <v/>
+      </c>
+      <c r="O88" s="38">
+        <f>O32+O85-O87</f>
+        <v/>
+      </c>
+      <c r="P88" s="38">
+        <f>P32+P85-P87</f>
+        <v/>
+      </c>
+      <c r="Q88" s="38">
+        <f>Q32+Q85-Q87</f>
+        <v/>
+      </c>
+      <c r="R88" s="38">
+        <f>R32+R85-R87</f>
+        <v/>
+      </c>
+      <c r="S88" s="38">
+        <f>S32+S85-S87</f>
+        <v/>
+      </c>
+      <c r="T88" s="38">
+        <f>T32+T85-T87</f>
+        <v/>
+      </c>
+      <c r="U88" s="38">
+        <f>U32+U85-U87</f>
+        <v/>
+      </c>
+      <c r="V88" s="38">
+        <f>V32+V85-V87</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="11">
+  <mergeCells count="12">
     <mergeCell ref="A54:V54"/>
     <mergeCell ref="A86:B86"/>
     <mergeCell ref="A1:V1"/>
@@ -7997,6 +8085,7 @@
     <mergeCell ref="A85:B85"/>
     <mergeCell ref="A31:V31"/>
     <mergeCell ref="A75:B75"/>
+    <mergeCell ref="A88:B88"/>
     <mergeCell ref="A3:V3"/>
     <mergeCell ref="A77:V77"/>
     <mergeCell ref="A43:V43"/>

</xml_diff>